<commit_message>
test: complete cash flow scaffold contract
</commit_message>
<xml_diff>
--- a/templates/13-week-cash-flow-forecast.xlsx
+++ b/templates/13-week-cash-flow-forecast.xlsx
@@ -2,14 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R834f8b96e8664207"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Rf5fef861a52348ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="Rb8d5dc6877cc48d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13-Week Forecast" sheetId="4" r:id="R18837502142343cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Review" sheetId="5" r:id="R9db952d3f83a468a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks &amp; Sources" sheetId="6" r:id="R7240b13cab8948d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R8422424ed3254cd8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R5c91082a1e444c94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R2078ee11a4bc45e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13-Week Forecast" sheetId="4" r:id="R257a5564b1894f69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Review" sheetId="5" r:id="R6a0c7ecdfe164073"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks &amp; Sources" sheetId="6" r:id="R66855269f32c48a3"/>
   </x:sheets>
   <x:definedNames>
+    <x:definedName name="CashFlowScenario">'Assumptions'!$B$12</x:definedName>
     <x:definedName name="CashFlowSelectedScenario">'Assumptions'!$B$12</x:definedName>
     <x:definedName name="CashFlowScenarioList">'Assumptions'!$B$15:$B$17</x:definedName>
   </x:definedNames>
@@ -27,7 +28,7 @@
     <x:numFmt numFmtId="201" formatCode="&quot;$&quot;#,##0;[Red](&quot;$&quot;#,##0);-"/>
     <x:numFmt numFmtId="202" formatCode="0.0%"/>
   </x:numFmts>
-  <x:fonts count="14">
+  <x:fonts count="13">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -76,11 +77,6 @@
     </x:font>
     <x:font>
       <x:sz val="11"/>
-      <x:color rgb="FF7A5AB5"/>
-      <x:name val="Aptos"/>
-    </x:font>
-    <x:font>
-      <x:sz val="11"/>
       <x:color rgb="FF4F485E"/>
       <x:name val="Aptos"/>
     </x:font>
@@ -103,7 +99,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="10">
+  <x:fills count="11">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -142,6 +138,11 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF7A5AB5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
         <x:fgColor rgb="FFDED9E8"/>
       </x:patternFill>
     </x:fill>
@@ -162,7 +163,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="43">
+  <x:cellXfs count="44">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -193,31 +194,32 @@
     <x:xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="10" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="10" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="10" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="6" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="201" fontId="6" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="6" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="6" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="202" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="11" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="11" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="10" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="201" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="13" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
@@ -479,13 +481,13 @@
       <x:c r="B6" t="str">
         <x:v>1.0 scaffold</x:v>
       </x:c>
-      <x:c r="D6" s="14" t="str">
+      <x:c r="D6" s="23" t="str">
         <x:v>Quick links</x:v>
       </x:c>
-      <x:c r="E6" s="14"/>
-      <x:c r="F6" s="14"/>
-      <x:c r="G6" s="14"/>
-      <x:c r="H6" s="14"/>
+      <x:c r="E6" s="23"/>
+      <x:c r="F6" s="23"/>
+      <x:c r="G6" s="23"/>
+      <x:c r="H6" s="23"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
@@ -494,7 +496,7 @@
       <x:c r="B7" s="11" t="n">
         <x:v>46260</x:v>
       </x:c>
-      <x:c r="D7" s="22" t="e">
+      <x:c r="D7" s="12" t="e">
         <x:f>HYPERLINK("#'Dashboard'!A1","Dashboard")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=#'Dashboard'!A1, friendlyName=Dashboard</x:v>
       </x:c>
@@ -506,7 +508,7 @@
       <x:c r="B8" t="str">
         <x:v>AUD</x:v>
       </x:c>
-      <x:c r="D8" s="22" t="e">
+      <x:c r="D8" s="12" t="e">
         <x:f>HYPERLINK("#'Assumptions'!A1","Assumptions")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=#'Assumptions'!A1, friendlyName=Assumptions</x:v>
       </x:c>
@@ -518,7 +520,7 @@
       <x:c r="B9" t="str">
         <x:v>Whole dollars</x:v>
       </x:c>
-      <x:c r="D9" s="22" t="e">
+      <x:c r="D9" s="12" t="e">
         <x:f>HYPERLINK("#'13-Week Forecast'!A1","13-Week Forecast")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=#'13-Week Forecast'!A1, friendlyName=13-Week Forecast</x:v>
       </x:c>
@@ -531,13 +533,13 @@
         <x:f>'Assumptions'!$B$12</x:f>
         <x:v>Base</x:v>
       </x:c>
-      <x:c r="D10" s="22" t="e">
+      <x:c r="D10" s="12" t="e">
         <x:f>HYPERLINK("#'Weekly Review'!A1","Weekly Review")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=#'Weekly Review'!A1, friendlyName=Weekly Review</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="D11" s="22" t="e">
+      <x:c r="D11" s="12" t="e">
         <x:f>HYPERLINK("#'Checks &amp; Sources'!A1","Checks &amp; Sources")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=#'Checks &amp; Sources'!A1, friendlyName=Checks &amp; Sources</x:v>
       </x:c>
@@ -647,26 +649,26 @@
       </x:c>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" s="26" t="str">
+      <x:c r="A27" s="27" t="str">
         <x:v>Scope limit: this workbook supports short-term cash planning. It is illustrative only and is not tax, payroll, legal or financial advice. Confirm statutory dates and classifications with your adviser.</x:v>
       </x:c>
-      <x:c r="B27" s="26"/>
-      <x:c r="C27" s="26"/>
-      <x:c r="D27" s="26"/>
-      <x:c r="E27" s="26"/>
-      <x:c r="F27" s="26"/>
-      <x:c r="G27" s="26"/>
-      <x:c r="H27" s="26"/>
+      <x:c r="B27" s="27"/>
+      <x:c r="C27" s="27"/>
+      <x:c r="D27" s="27"/>
+      <x:c r="E27" s="27"/>
+      <x:c r="F27" s="27"/>
+      <x:c r="G27" s="27"/>
+      <x:c r="H27" s="27"/>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="26"/>
-      <x:c r="B28" s="26"/>
-      <x:c r="C28" s="26"/>
-      <x:c r="D28" s="26"/>
-      <x:c r="E28" s="26"/>
-      <x:c r="F28" s="26"/>
-      <x:c r="G28" s="26"/>
-      <x:c r="H28" s="26"/>
+      <x:c r="A28" s="27"/>
+      <x:c r="B28" s="27"/>
+      <x:c r="C28" s="27"/>
+      <x:c r="D28" s="27"/>
+      <x:c r="E28" s="27"/>
+      <x:c r="F28" s="27"/>
+      <x:c r="G28" s="27"/>
+      <x:c r="H28" s="27"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -739,41 +741,41 @@
       <x:c r="O2" s="8"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="24" t="str">
+      <x:c r="A4" s="25" t="str">
         <x:v>No cash-flow inputs belong on this sheet. Update Assumptions and the 13-Week Forecast instead.</x:v>
       </x:c>
-      <x:c r="B4" s="24"/>
-      <x:c r="C4" s="24"/>
-      <x:c r="D4" s="24"/>
-      <x:c r="E4" s="24"/>
-      <x:c r="F4" s="24"/>
-      <x:c r="G4" s="24"/>
-      <x:c r="H4" s="24"/>
-      <x:c r="I4" s="24"/>
-      <x:c r="J4" s="24"/>
-      <x:c r="K4" s="24"/>
-      <x:c r="L4" s="24"/>
-      <x:c r="M4" s="24"/>
-      <x:c r="N4" s="24"/>
-      <x:c r="O4" s="24"/>
+      <x:c r="B4" s="25"/>
+      <x:c r="C4" s="25"/>
+      <x:c r="D4" s="25"/>
+      <x:c r="E4" s="25"/>
+      <x:c r="F4" s="25"/>
+      <x:c r="G4" s="25"/>
+      <x:c r="H4" s="25"/>
+      <x:c r="I4" s="25"/>
+      <x:c r="J4" s="25"/>
+      <x:c r="K4" s="25"/>
+      <x:c r="L4" s="25"/>
+      <x:c r="M4" s="25"/>
+      <x:c r="N4" s="25"/>
+      <x:c r="O4" s="25"/>
     </x:row>
     <x:row r="6" ht="32" customHeight="1">
-      <x:c r="A6" s="27" t="str">
+      <x:c r="A6" s="28" t="str">
         <x:v>Selected scenario</x:v>
       </x:c>
-      <x:c r="B6" s="27" t="str">
+      <x:c r="B6" s="28" t="str">
         <x:v>Week 13 closing cash</x:v>
       </x:c>
-      <x:c r="C6" s="27" t="str">
+      <x:c r="C6" s="28" t="str">
         <x:v>Lowest closing cash</x:v>
       </x:c>
-      <x:c r="D6" s="27" t="str">
+      <x:c r="D6" s="28" t="str">
         <x:v>Minimum buffer</x:v>
       </x:c>
-      <x:c r="E6" s="27" t="str">
+      <x:c r="E6" s="28" t="str">
         <x:v>Minimum headroom</x:v>
       </x:c>
-      <x:c r="F6" s="27" t="str">
+      <x:c r="F6" s="28" t="str">
         <x:v>Weeks below buffer</x:v>
       </x:c>
     </x:row>
@@ -865,7 +867,7 @@
       <x:c r="A5" t="str">
         <x:v>Business name</x:v>
       </x:c>
-      <x:c r="B5" s="28" t="str">
+      <x:c r="B5" s="29" t="str">
         <x:v>Illustrative Australian business</x:v>
       </x:c>
     </x:row>
@@ -873,7 +875,7 @@
       <x:c r="A6" t="str">
         <x:v>Currency</x:v>
       </x:c>
-      <x:c r="B6" s="28" t="str">
+      <x:c r="B6" s="29" t="str">
         <x:v>AUD</x:v>
       </x:c>
     </x:row>
@@ -881,7 +883,7 @@
       <x:c r="A7" t="str">
         <x:v>Units</x:v>
       </x:c>
-      <x:c r="B7" s="28" t="str">
+      <x:c r="B7" s="29" t="str">
         <x:v>Whole dollars</x:v>
       </x:c>
     </x:row>
@@ -889,7 +891,7 @@
       <x:c r="A8" t="str">
         <x:v>Forecast start date</x:v>
       </x:c>
-      <x:c r="B8" s="29" t="n">
+      <x:c r="B8" s="30" t="n">
         <x:v>46265</x:v>
       </x:c>
     </x:row>
@@ -897,7 +899,7 @@
       <x:c r="A9" t="str">
         <x:v>As-at date</x:v>
       </x:c>
-      <x:c r="B9" s="29" t="n">
+      <x:c r="B9" s="30" t="n">
         <x:v>46271</x:v>
       </x:c>
     </x:row>
@@ -905,7 +907,7 @@
       <x:c r="A10" t="str">
         <x:v>Opening cash</x:v>
       </x:c>
-      <x:c r="B10" s="30" t="n">
+      <x:c r="B10" s="31" t="n">
         <x:v>400000</x:v>
       </x:c>
     </x:row>
@@ -913,7 +915,7 @@
       <x:c r="A11" t="str">
         <x:v>Minimum cash buffer</x:v>
       </x:c>
-      <x:c r="B11" s="30" t="n">
+      <x:c r="B11" s="31" t="n">
         <x:v>100000</x:v>
       </x:c>
     </x:row>
@@ -921,7 +923,7 @@
       <x:c r="A12" t="str">
         <x:v>Selected scenario</x:v>
       </x:c>
-      <x:c r="B12" s="28" t="str">
+      <x:c r="B12" s="29" t="str">
         <x:v>Base</x:v>
       </x:c>
     </x:row>
@@ -946,10 +948,10 @@
       <x:c r="B15" s="16" t="str">
         <x:v>Base</x:v>
       </x:c>
-      <x:c r="C15" s="31" t="n">
+      <x:c r="C15" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D15" s="31" t="n">
+      <x:c r="D15" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E15" s="16" t="str">
@@ -960,10 +962,10 @@
       <x:c r="B16" s="16" t="str">
         <x:v>Upside</x:v>
       </x:c>
-      <x:c r="C16" s="31" t="n">
+      <x:c r="C16" s="32" t="n">
         <x:v>1.08</x:v>
       </x:c>
-      <x:c r="D16" s="31" t="n">
+      <x:c r="D16" s="32" t="n">
         <x:v>0.98</x:v>
       </x:c>
       <x:c r="E16" s="16" t="str">
@@ -974,10 +976,10 @@
       <x:c r="B17" s="16" t="str">
         <x:v>Downside</x:v>
       </x:c>
-      <x:c r="C17" s="31" t="n">
+      <x:c r="C17" s="32" t="n">
         <x:v>0.85</x:v>
       </x:c>
-      <x:c r="D17" s="31" t="n">
+      <x:c r="D17" s="32" t="n">
         <x:v>1.05</x:v>
       </x:c>
       <x:c r="E17" s="16" t="str">
@@ -995,30 +997,30 @@
       <x:c r="F20" s="14"/>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="26" t="str">
+      <x:c r="A21" s="27" t="str">
         <x:v>Use a Monday forecast start. Keep the as-at date inside the 13-week horizon. Replace illustrative inputs before using this workbook for a decision. Statutory cash dates depend on your reporting cycle, agent concessions and entity circumstances.</x:v>
       </x:c>
-      <x:c r="B21" s="26"/>
-      <x:c r="C21" s="26"/>
-      <x:c r="D21" s="26"/>
-      <x:c r="E21" s="26"/>
-      <x:c r="F21" s="26"/>
+      <x:c r="B21" s="27"/>
+      <x:c r="C21" s="27"/>
+      <x:c r="D21" s="27"/>
+      <x:c r="E21" s="27"/>
+      <x:c r="F21" s="27"/>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="26"/>
-      <x:c r="B22" s="26"/>
-      <x:c r="C22" s="26"/>
-      <x:c r="D22" s="26"/>
-      <x:c r="E22" s="26"/>
-      <x:c r="F22" s="26"/>
+      <x:c r="A22" s="27"/>
+      <x:c r="B22" s="27"/>
+      <x:c r="C22" s="27"/>
+      <x:c r="D22" s="27"/>
+      <x:c r="E22" s="27"/>
+      <x:c r="F22" s="27"/>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="26"/>
-      <x:c r="B23" s="26"/>
-      <x:c r="C23" s="26"/>
-      <x:c r="D23" s="26"/>
-      <x:c r="E23" s="26"/>
-      <x:c r="F23" s="26"/>
+      <x:c r="A23" s="27"/>
+      <x:c r="B23" s="27"/>
+      <x:c r="C23" s="27"/>
+      <x:c r="D23" s="27"/>
+      <x:c r="E23" s="27"/>
+      <x:c r="F23" s="27"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1099,43 +1101,43 @@
       <x:c r="A5" t="str">
         <x:v>Week commencing</x:v>
       </x:c>
-      <x:c r="B5" s="33" t="n">
+      <x:c r="B5" s="34" t="n">
         <x:v>46265</x:v>
       </x:c>
-      <x:c r="C5" s="33" t="n">
+      <x:c r="C5" s="34" t="n">
         <x:v>46272</x:v>
       </x:c>
-      <x:c r="D5" s="33" t="n">
+      <x:c r="D5" s="34" t="n">
         <x:v>46279</x:v>
       </x:c>
-      <x:c r="E5" s="33" t="n">
+      <x:c r="E5" s="34" t="n">
         <x:v>46286</x:v>
       </x:c>
-      <x:c r="F5" s="33" t="n">
+      <x:c r="F5" s="34" t="n">
         <x:v>46293</x:v>
       </x:c>
-      <x:c r="G5" s="33" t="n">
+      <x:c r="G5" s="34" t="n">
         <x:v>46300</x:v>
       </x:c>
-      <x:c r="H5" s="33" t="n">
+      <x:c r="H5" s="34" t="n">
         <x:v>46307</x:v>
       </x:c>
-      <x:c r="I5" s="33" t="n">
+      <x:c r="I5" s="34" t="n">
         <x:v>46314</x:v>
       </x:c>
-      <x:c r="J5" s="33" t="n">
+      <x:c r="J5" s="34" t="n">
         <x:v>46321</x:v>
       </x:c>
-      <x:c r="K5" s="33" t="n">
+      <x:c r="K5" s="34" t="n">
         <x:v>46328</x:v>
       </x:c>
-      <x:c r="L5" s="33" t="n">
+      <x:c r="L5" s="34" t="n">
         <x:v>46335</x:v>
       </x:c>
-      <x:c r="M5" s="33" t="n">
+      <x:c r="M5" s="34" t="n">
         <x:v>46342</x:v>
       </x:c>
-      <x:c r="N5" s="33" t="n">
+      <x:c r="N5" s="34" t="n">
         <x:v>46349</x:v>
       </x:c>
       <x:c r="O5" t="str">
@@ -1146,43 +1148,43 @@
       <x:c r="A6" t="str">
         <x:v>Week ending</x:v>
       </x:c>
-      <x:c r="B6" s="33" t="n">
+      <x:c r="B6" s="34" t="n">
         <x:v>46271</x:v>
       </x:c>
-      <x:c r="C6" s="33" t="n">
+      <x:c r="C6" s="34" t="n">
         <x:v>46278</x:v>
       </x:c>
-      <x:c r="D6" s="33" t="n">
+      <x:c r="D6" s="34" t="n">
         <x:v>46285</x:v>
       </x:c>
-      <x:c r="E6" s="33" t="n">
+      <x:c r="E6" s="34" t="n">
         <x:v>46292</x:v>
       </x:c>
-      <x:c r="F6" s="33" t="n">
+      <x:c r="F6" s="34" t="n">
         <x:v>46299</x:v>
       </x:c>
-      <x:c r="G6" s="33" t="n">
+      <x:c r="G6" s="34" t="n">
         <x:v>46306</x:v>
       </x:c>
-      <x:c r="H6" s="33" t="n">
+      <x:c r="H6" s="34" t="n">
         <x:v>46313</x:v>
       </x:c>
-      <x:c r="I6" s="33" t="n">
+      <x:c r="I6" s="34" t="n">
         <x:v>46320</x:v>
       </x:c>
-      <x:c r="J6" s="33" t="n">
+      <x:c r="J6" s="34" t="n">
         <x:v>46327</x:v>
       </x:c>
-      <x:c r="K6" s="33" t="n">
+      <x:c r="K6" s="34" t="n">
         <x:v>46334</x:v>
       </x:c>
-      <x:c r="L6" s="33" t="n">
+      <x:c r="L6" s="34" t="n">
         <x:v>46341</x:v>
       </x:c>
-      <x:c r="M6" s="33" t="n">
+      <x:c r="M6" s="34" t="n">
         <x:v>46348</x:v>
       </x:c>
-      <x:c r="N6" s="33" t="n">
+      <x:c r="N6" s="34" t="n">
         <x:v>46355</x:v>
       </x:c>
       <x:c r="O6" t="str">
@@ -1193,43 +1195,43 @@
       <x:c r="A7" t="str">
         <x:v>Actual / Forecast</x:v>
       </x:c>
-      <x:c r="B7" s="34" t="str">
+      <x:c r="B7" s="35" t="str">
         <x:v>Forecast</x:v>
       </x:c>
-      <x:c r="C7" s="34" t="str">
+      <x:c r="C7" s="35" t="str">
         <x:v>Forecast</x:v>
       </x:c>
-      <x:c r="D7" s="34" t="str">
+      <x:c r="D7" s="35" t="str">
         <x:v>Forecast</x:v>
       </x:c>
-      <x:c r="E7" s="34" t="str">
+      <x:c r="E7" s="35" t="str">
         <x:v>Forecast</x:v>
       </x:c>
-      <x:c r="F7" s="34" t="str">
+      <x:c r="F7" s="35" t="str">
         <x:v>Forecast</x:v>
       </x:c>
-      <x:c r="G7" s="34" t="str">
+      <x:c r="G7" s="35" t="str">
         <x:v>Forecast</x:v>
       </x:c>
-      <x:c r="H7" s="34" t="str">
+      <x:c r="H7" s="35" t="str">
         <x:v>Forecast</x:v>
       </x:c>
-      <x:c r="I7" s="34" t="str">
+      <x:c r="I7" s="35" t="str">
         <x:v>Forecast</x:v>
       </x:c>
-      <x:c r="J7" s="34" t="str">
+      <x:c r="J7" s="35" t="str">
         <x:v>Forecast</x:v>
       </x:c>
-      <x:c r="K7" s="34" t="str">
+      <x:c r="K7" s="35" t="str">
         <x:v>Forecast</x:v>
       </x:c>
-      <x:c r="L7" s="34" t="str">
+      <x:c r="L7" s="35" t="str">
         <x:v>Forecast</x:v>
       </x:c>
-      <x:c r="M7" s="34" t="str">
+      <x:c r="M7" s="35" t="str">
         <x:v>Forecast</x:v>
       </x:c>
-      <x:c r="N7" s="34" t="str">
+      <x:c r="N7" s="35" t="str">
         <x:v>Forecast</x:v>
       </x:c>
       <x:c r="O7" t="str"/>
@@ -1257,774 +1259,774 @@
       <x:c r="A10" t="str">
         <x:v>Customer receipts</x:v>
       </x:c>
-      <x:c r="B10" s="37"/>
-      <x:c r="C10" s="37"/>
-      <x:c r="D10" s="37"/>
-      <x:c r="E10" s="37"/>
-      <x:c r="F10" s="37"/>
-      <x:c r="G10" s="37"/>
-      <x:c r="H10" s="37"/>
-      <x:c r="I10" s="37"/>
-      <x:c r="J10" s="37"/>
-      <x:c r="K10" s="37"/>
-      <x:c r="L10" s="37"/>
-      <x:c r="M10" s="37"/>
-      <x:c r="N10" s="37"/>
-      <x:c r="O10" s="37"/>
+      <x:c r="B10" s="38"/>
+      <x:c r="C10" s="38"/>
+      <x:c r="D10" s="38"/>
+      <x:c r="E10" s="38"/>
+      <x:c r="F10" s="38"/>
+      <x:c r="G10" s="38"/>
+      <x:c r="H10" s="38"/>
+      <x:c r="I10" s="38"/>
+      <x:c r="J10" s="38"/>
+      <x:c r="K10" s="38"/>
+      <x:c r="L10" s="38"/>
+      <x:c r="M10" s="38"/>
+      <x:c r="N10" s="38"/>
+      <x:c r="O10" s="38"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="str">
         <x:v>Overdue receipts</x:v>
       </x:c>
-      <x:c r="B11" s="37"/>
-      <x:c r="C11" s="37"/>
-      <x:c r="D11" s="37"/>
-      <x:c r="E11" s="37"/>
-      <x:c r="F11" s="37"/>
-      <x:c r="G11" s="37"/>
-      <x:c r="H11" s="37"/>
-      <x:c r="I11" s="37"/>
-      <x:c r="J11" s="37"/>
-      <x:c r="K11" s="37"/>
-      <x:c r="L11" s="37"/>
-      <x:c r="M11" s="37"/>
-      <x:c r="N11" s="37"/>
-      <x:c r="O11" s="37"/>
+      <x:c r="B11" s="38"/>
+      <x:c r="C11" s="38"/>
+      <x:c r="D11" s="38"/>
+      <x:c r="E11" s="38"/>
+      <x:c r="F11" s="38"/>
+      <x:c r="G11" s="38"/>
+      <x:c r="H11" s="38"/>
+      <x:c r="I11" s="38"/>
+      <x:c r="J11" s="38"/>
+      <x:c r="K11" s="38"/>
+      <x:c r="L11" s="38"/>
+      <x:c r="M11" s="38"/>
+      <x:c r="N11" s="38"/>
+      <x:c r="O11" s="38"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="str">
         <x:v>Cash / EFTPOS sales</x:v>
       </x:c>
-      <x:c r="B12" s="37"/>
-      <x:c r="C12" s="37"/>
-      <x:c r="D12" s="37"/>
-      <x:c r="E12" s="37"/>
-      <x:c r="F12" s="37"/>
-      <x:c r="G12" s="37"/>
-      <x:c r="H12" s="37"/>
-      <x:c r="I12" s="37"/>
-      <x:c r="J12" s="37"/>
-      <x:c r="K12" s="37"/>
-      <x:c r="L12" s="37"/>
-      <x:c r="M12" s="37"/>
-      <x:c r="N12" s="37"/>
-      <x:c r="O12" s="37"/>
+      <x:c r="B12" s="38"/>
+      <x:c r="C12" s="38"/>
+      <x:c r="D12" s="38"/>
+      <x:c r="E12" s="38"/>
+      <x:c r="F12" s="38"/>
+      <x:c r="G12" s="38"/>
+      <x:c r="H12" s="38"/>
+      <x:c r="I12" s="38"/>
+      <x:c r="J12" s="38"/>
+      <x:c r="K12" s="38"/>
+      <x:c r="L12" s="38"/>
+      <x:c r="M12" s="38"/>
+      <x:c r="N12" s="38"/>
+      <x:c r="O12" s="38"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="str">
         <x:v>GST refunds / credits</x:v>
       </x:c>
-      <x:c r="B13" s="37"/>
-      <x:c r="C13" s="37"/>
-      <x:c r="D13" s="37"/>
-      <x:c r="E13" s="37"/>
-      <x:c r="F13" s="37"/>
-      <x:c r="G13" s="37"/>
-      <x:c r="H13" s="37"/>
-      <x:c r="I13" s="37"/>
-      <x:c r="J13" s="37"/>
-      <x:c r="K13" s="37"/>
-      <x:c r="L13" s="37"/>
-      <x:c r="M13" s="37"/>
-      <x:c r="N13" s="37"/>
-      <x:c r="O13" s="37"/>
+      <x:c r="B13" s="38"/>
+      <x:c r="C13" s="38"/>
+      <x:c r="D13" s="38"/>
+      <x:c r="E13" s="38"/>
+      <x:c r="F13" s="38"/>
+      <x:c r="G13" s="38"/>
+      <x:c r="H13" s="38"/>
+      <x:c r="I13" s="38"/>
+      <x:c r="J13" s="38"/>
+      <x:c r="K13" s="38"/>
+      <x:c r="L13" s="38"/>
+      <x:c r="M13" s="38"/>
+      <x:c r="N13" s="38"/>
+      <x:c r="O13" s="38"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="str">
         <x:v>Other operating</x:v>
       </x:c>
-      <x:c r="B14" s="37"/>
-      <x:c r="C14" s="37"/>
-      <x:c r="D14" s="37"/>
-      <x:c r="E14" s="37"/>
-      <x:c r="F14" s="37"/>
-      <x:c r="G14" s="37"/>
-      <x:c r="H14" s="37"/>
-      <x:c r="I14" s="37"/>
-      <x:c r="J14" s="37"/>
-      <x:c r="K14" s="37"/>
-      <x:c r="L14" s="37"/>
-      <x:c r="M14" s="37"/>
-      <x:c r="N14" s="37"/>
-      <x:c r="O14" s="37"/>
+      <x:c r="B14" s="38"/>
+      <x:c r="C14" s="38"/>
+      <x:c r="D14" s="38"/>
+      <x:c r="E14" s="38"/>
+      <x:c r="F14" s="38"/>
+      <x:c r="G14" s="38"/>
+      <x:c r="H14" s="38"/>
+      <x:c r="I14" s="38"/>
+      <x:c r="J14" s="38"/>
+      <x:c r="K14" s="38"/>
+      <x:c r="L14" s="38"/>
+      <x:c r="M14" s="38"/>
+      <x:c r="N14" s="38"/>
+      <x:c r="O14" s="38"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" t="str">
         <x:v>Asset sale proceeds</x:v>
       </x:c>
-      <x:c r="B15" s="37"/>
-      <x:c r="C15" s="37"/>
-      <x:c r="D15" s="37"/>
-      <x:c r="E15" s="37"/>
-      <x:c r="F15" s="37"/>
-      <x:c r="G15" s="37"/>
-      <x:c r="H15" s="37"/>
-      <x:c r="I15" s="37"/>
-      <x:c r="J15" s="37"/>
-      <x:c r="K15" s="37"/>
-      <x:c r="L15" s="37"/>
-      <x:c r="M15" s="37"/>
-      <x:c r="N15" s="37"/>
-      <x:c r="O15" s="37"/>
+      <x:c r="B15" s="38"/>
+      <x:c r="C15" s="38"/>
+      <x:c r="D15" s="38"/>
+      <x:c r="E15" s="38"/>
+      <x:c r="F15" s="38"/>
+      <x:c r="G15" s="38"/>
+      <x:c r="H15" s="38"/>
+      <x:c r="I15" s="38"/>
+      <x:c r="J15" s="38"/>
+      <x:c r="K15" s="38"/>
+      <x:c r="L15" s="38"/>
+      <x:c r="M15" s="38"/>
+      <x:c r="N15" s="38"/>
+      <x:c r="O15" s="38"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" t="str">
         <x:v>Equity / owner funding</x:v>
       </x:c>
-      <x:c r="B16" s="37"/>
-      <x:c r="C16" s="37"/>
-      <x:c r="D16" s="37"/>
-      <x:c r="E16" s="37"/>
-      <x:c r="F16" s="37"/>
-      <x:c r="G16" s="37"/>
-      <x:c r="H16" s="37"/>
-      <x:c r="I16" s="37"/>
-      <x:c r="J16" s="37"/>
-      <x:c r="K16" s="37"/>
-      <x:c r="L16" s="37"/>
-      <x:c r="M16" s="37"/>
-      <x:c r="N16" s="37"/>
-      <x:c r="O16" s="37"/>
+      <x:c r="B16" s="38"/>
+      <x:c r="C16" s="38"/>
+      <x:c r="D16" s="38"/>
+      <x:c r="E16" s="38"/>
+      <x:c r="F16" s="38"/>
+      <x:c r="G16" s="38"/>
+      <x:c r="H16" s="38"/>
+      <x:c r="I16" s="38"/>
+      <x:c r="J16" s="38"/>
+      <x:c r="K16" s="38"/>
+      <x:c r="L16" s="38"/>
+      <x:c r="M16" s="38"/>
+      <x:c r="N16" s="38"/>
+      <x:c r="O16" s="38"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" t="str">
         <x:v>Loan proceeds</x:v>
       </x:c>
-      <x:c r="B17" s="37"/>
-      <x:c r="C17" s="37"/>
-      <x:c r="D17" s="37"/>
-      <x:c r="E17" s="37"/>
-      <x:c r="F17" s="37"/>
-      <x:c r="G17" s="37"/>
-      <x:c r="H17" s="37"/>
-      <x:c r="I17" s="37"/>
-      <x:c r="J17" s="37"/>
-      <x:c r="K17" s="37"/>
-      <x:c r="L17" s="37"/>
-      <x:c r="M17" s="37"/>
-      <x:c r="N17" s="37"/>
-      <x:c r="O17" s="37"/>
+      <x:c r="B17" s="38"/>
+      <x:c r="C17" s="38"/>
+      <x:c r="D17" s="38"/>
+      <x:c r="E17" s="38"/>
+      <x:c r="F17" s="38"/>
+      <x:c r="G17" s="38"/>
+      <x:c r="H17" s="38"/>
+      <x:c r="I17" s="38"/>
+      <x:c r="J17" s="38"/>
+      <x:c r="K17" s="38"/>
+      <x:c r="L17" s="38"/>
+      <x:c r="M17" s="38"/>
+      <x:c r="N17" s="38"/>
+      <x:c r="O17" s="38"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" t="str">
         <x:v>Scenario receipt adjustment</x:v>
       </x:c>
-      <x:c r="B18" s="37"/>
-      <x:c r="C18" s="37"/>
-      <x:c r="D18" s="37"/>
-      <x:c r="E18" s="37"/>
-      <x:c r="F18" s="37"/>
-      <x:c r="G18" s="37"/>
-      <x:c r="H18" s="37"/>
-      <x:c r="I18" s="37"/>
-      <x:c r="J18" s="37"/>
-      <x:c r="K18" s="37"/>
-      <x:c r="L18" s="37"/>
-      <x:c r="M18" s="37"/>
-      <x:c r="N18" s="37"/>
-      <x:c r="O18" s="37"/>
+      <x:c r="B18" s="38"/>
+      <x:c r="C18" s="38"/>
+      <x:c r="D18" s="38"/>
+      <x:c r="E18" s="38"/>
+      <x:c r="F18" s="38"/>
+      <x:c r="G18" s="38"/>
+      <x:c r="H18" s="38"/>
+      <x:c r="I18" s="38"/>
+      <x:c r="J18" s="38"/>
+      <x:c r="K18" s="38"/>
+      <x:c r="L18" s="38"/>
+      <x:c r="M18" s="38"/>
+      <x:c r="N18" s="38"/>
+      <x:c r="O18" s="38"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="36" t="str">
+      <x:c r="A19" s="37" t="str">
         <x:v>Total cash receipts</x:v>
       </x:c>
-      <x:c r="B19" s="38"/>
-      <x:c r="C19" s="38"/>
-      <x:c r="D19" s="38"/>
-      <x:c r="E19" s="38"/>
-      <x:c r="F19" s="38"/>
-      <x:c r="G19" s="38"/>
-      <x:c r="H19" s="38"/>
-      <x:c r="I19" s="38"/>
-      <x:c r="J19" s="38"/>
-      <x:c r="K19" s="38"/>
-      <x:c r="L19" s="38"/>
-      <x:c r="M19" s="38"/>
-      <x:c r="N19" s="38"/>
-      <x:c r="O19" s="38"/>
+      <x:c r="B19" s="39"/>
+      <x:c r="C19" s="39"/>
+      <x:c r="D19" s="39"/>
+      <x:c r="E19" s="39"/>
+      <x:c r="F19" s="39"/>
+      <x:c r="G19" s="39"/>
+      <x:c r="H19" s="39"/>
+      <x:c r="I19" s="39"/>
+      <x:c r="J19" s="39"/>
+      <x:c r="K19" s="39"/>
+      <x:c r="L19" s="39"/>
+      <x:c r="M19" s="39"/>
+      <x:c r="N19" s="39"/>
+      <x:c r="O19" s="39"/>
     </x:row>
     <x:row r="20">
-      <x:c r="B20" s="37"/>
-      <x:c r="C20" s="37"/>
-      <x:c r="D20" s="37"/>
-      <x:c r="E20" s="37"/>
-      <x:c r="F20" s="37"/>
-      <x:c r="G20" s="37"/>
-      <x:c r="H20" s="37"/>
-      <x:c r="I20" s="37"/>
-      <x:c r="J20" s="37"/>
-      <x:c r="K20" s="37"/>
-      <x:c r="L20" s="37"/>
-      <x:c r="M20" s="37"/>
-      <x:c r="N20" s="37"/>
-      <x:c r="O20" s="37"/>
+      <x:c r="B20" s="38"/>
+      <x:c r="C20" s="38"/>
+      <x:c r="D20" s="38"/>
+      <x:c r="E20" s="38"/>
+      <x:c r="F20" s="38"/>
+      <x:c r="G20" s="38"/>
+      <x:c r="H20" s="38"/>
+      <x:c r="I20" s="38"/>
+      <x:c r="J20" s="38"/>
+      <x:c r="K20" s="38"/>
+      <x:c r="L20" s="38"/>
+      <x:c r="M20" s="38"/>
+      <x:c r="N20" s="38"/>
+      <x:c r="O20" s="38"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="14" t="str">
         <x:v>CASH PAYMENTS</x:v>
       </x:c>
-      <x:c r="B21" s="39"/>
-      <x:c r="C21" s="39"/>
-      <x:c r="D21" s="39"/>
-      <x:c r="E21" s="39"/>
-      <x:c r="F21" s="39"/>
-      <x:c r="G21" s="39"/>
-      <x:c r="H21" s="39"/>
-      <x:c r="I21" s="39"/>
-      <x:c r="J21" s="39"/>
-      <x:c r="K21" s="39"/>
-      <x:c r="L21" s="39"/>
-      <x:c r="M21" s="39"/>
-      <x:c r="N21" s="39"/>
-      <x:c r="O21" s="39"/>
+      <x:c r="B21" s="40"/>
+      <x:c r="C21" s="40"/>
+      <x:c r="D21" s="40"/>
+      <x:c r="E21" s="40"/>
+      <x:c r="F21" s="40"/>
+      <x:c r="G21" s="40"/>
+      <x:c r="H21" s="40"/>
+      <x:c r="I21" s="40"/>
+      <x:c r="J21" s="40"/>
+      <x:c r="K21" s="40"/>
+      <x:c r="L21" s="40"/>
+      <x:c r="M21" s="40"/>
+      <x:c r="N21" s="40"/>
+      <x:c r="O21" s="40"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" t="str">
         <x:v>Suppliers and inventory</x:v>
       </x:c>
-      <x:c r="B22" s="37"/>
-      <x:c r="C22" s="37"/>
-      <x:c r="D22" s="37"/>
-      <x:c r="E22" s="37"/>
-      <x:c r="F22" s="37"/>
-      <x:c r="G22" s="37"/>
-      <x:c r="H22" s="37"/>
-      <x:c r="I22" s="37"/>
-      <x:c r="J22" s="37"/>
-      <x:c r="K22" s="37"/>
-      <x:c r="L22" s="37"/>
-      <x:c r="M22" s="37"/>
-      <x:c r="N22" s="37"/>
-      <x:c r="O22" s="37"/>
+      <x:c r="B22" s="38"/>
+      <x:c r="C22" s="38"/>
+      <x:c r="D22" s="38"/>
+      <x:c r="E22" s="38"/>
+      <x:c r="F22" s="38"/>
+      <x:c r="G22" s="38"/>
+      <x:c r="H22" s="38"/>
+      <x:c r="I22" s="38"/>
+      <x:c r="J22" s="38"/>
+      <x:c r="K22" s="38"/>
+      <x:c r="L22" s="38"/>
+      <x:c r="M22" s="38"/>
+      <x:c r="N22" s="38"/>
+      <x:c r="O22" s="38"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" t="str">
         <x:v>Net wages</x:v>
       </x:c>
-      <x:c r="B23" s="37"/>
-      <x:c r="C23" s="37"/>
-      <x:c r="D23" s="37"/>
-      <x:c r="E23" s="37"/>
-      <x:c r="F23" s="37"/>
-      <x:c r="G23" s="37"/>
-      <x:c r="H23" s="37"/>
-      <x:c r="I23" s="37"/>
-      <x:c r="J23" s="37"/>
-      <x:c r="K23" s="37"/>
-      <x:c r="L23" s="37"/>
-      <x:c r="M23" s="37"/>
-      <x:c r="N23" s="37"/>
-      <x:c r="O23" s="37"/>
+      <x:c r="B23" s="38"/>
+      <x:c r="C23" s="38"/>
+      <x:c r="D23" s="38"/>
+      <x:c r="E23" s="38"/>
+      <x:c r="F23" s="38"/>
+      <x:c r="G23" s="38"/>
+      <x:c r="H23" s="38"/>
+      <x:c r="I23" s="38"/>
+      <x:c r="J23" s="38"/>
+      <x:c r="K23" s="38"/>
+      <x:c r="L23" s="38"/>
+      <x:c r="M23" s="38"/>
+      <x:c r="N23" s="38"/>
+      <x:c r="O23" s="38"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" t="str">
         <x:v>PAYG withholding</x:v>
       </x:c>
-      <x:c r="B24" s="37"/>
-      <x:c r="C24" s="37"/>
-      <x:c r="D24" s="37"/>
-      <x:c r="E24" s="37"/>
-      <x:c r="F24" s="37"/>
-      <x:c r="G24" s="37"/>
-      <x:c r="H24" s="37"/>
-      <x:c r="I24" s="37"/>
-      <x:c r="J24" s="37"/>
-      <x:c r="K24" s="37"/>
-      <x:c r="L24" s="37"/>
-      <x:c r="M24" s="37"/>
-      <x:c r="N24" s="37"/>
-      <x:c r="O24" s="37"/>
+      <x:c r="B24" s="38"/>
+      <x:c r="C24" s="38"/>
+      <x:c r="D24" s="38"/>
+      <x:c r="E24" s="38"/>
+      <x:c r="F24" s="38"/>
+      <x:c r="G24" s="38"/>
+      <x:c r="H24" s="38"/>
+      <x:c r="I24" s="38"/>
+      <x:c r="J24" s="38"/>
+      <x:c r="K24" s="38"/>
+      <x:c r="L24" s="38"/>
+      <x:c r="M24" s="38"/>
+      <x:c r="N24" s="38"/>
+      <x:c r="O24" s="38"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" t="str">
         <x:v>Superannuation</x:v>
       </x:c>
-      <x:c r="B25" s="37"/>
-      <x:c r="C25" s="37"/>
-      <x:c r="D25" s="37"/>
-      <x:c r="E25" s="37"/>
-      <x:c r="F25" s="37"/>
-      <x:c r="G25" s="37"/>
-      <x:c r="H25" s="37"/>
-      <x:c r="I25" s="37"/>
-      <x:c r="J25" s="37"/>
-      <x:c r="K25" s="37"/>
-      <x:c r="L25" s="37"/>
-      <x:c r="M25" s="37"/>
-      <x:c r="N25" s="37"/>
-      <x:c r="O25" s="37"/>
+      <x:c r="B25" s="38"/>
+      <x:c r="C25" s="38"/>
+      <x:c r="D25" s="38"/>
+      <x:c r="E25" s="38"/>
+      <x:c r="F25" s="38"/>
+      <x:c r="G25" s="38"/>
+      <x:c r="H25" s="38"/>
+      <x:c r="I25" s="38"/>
+      <x:c r="J25" s="38"/>
+      <x:c r="K25" s="38"/>
+      <x:c r="L25" s="38"/>
+      <x:c r="M25" s="38"/>
+      <x:c r="N25" s="38"/>
+      <x:c r="O25" s="38"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" t="str">
         <x:v>Payroll tax / workers compensation</x:v>
       </x:c>
-      <x:c r="B26" s="37"/>
-      <x:c r="C26" s="37"/>
-      <x:c r="D26" s="37"/>
-      <x:c r="E26" s="37"/>
-      <x:c r="F26" s="37"/>
-      <x:c r="G26" s="37"/>
-      <x:c r="H26" s="37"/>
-      <x:c r="I26" s="37"/>
-      <x:c r="J26" s="37"/>
-      <x:c r="K26" s="37"/>
-      <x:c r="L26" s="37"/>
-      <x:c r="M26" s="37"/>
-      <x:c r="N26" s="37"/>
-      <x:c r="O26" s="37"/>
+      <x:c r="B26" s="38"/>
+      <x:c r="C26" s="38"/>
+      <x:c r="D26" s="38"/>
+      <x:c r="E26" s="38"/>
+      <x:c r="F26" s="38"/>
+      <x:c r="G26" s="38"/>
+      <x:c r="H26" s="38"/>
+      <x:c r="I26" s="38"/>
+      <x:c r="J26" s="38"/>
+      <x:c r="K26" s="38"/>
+      <x:c r="L26" s="38"/>
+      <x:c r="M26" s="38"/>
+      <x:c r="N26" s="38"/>
+      <x:c r="O26" s="38"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" t="str">
         <x:v>Rent</x:v>
       </x:c>
-      <x:c r="B27" s="37"/>
-      <x:c r="C27" s="37"/>
-      <x:c r="D27" s="37"/>
-      <x:c r="E27" s="37"/>
-      <x:c r="F27" s="37"/>
-      <x:c r="G27" s="37"/>
-      <x:c r="H27" s="37"/>
-      <x:c r="I27" s="37"/>
-      <x:c r="J27" s="37"/>
-      <x:c r="K27" s="37"/>
-      <x:c r="L27" s="37"/>
-      <x:c r="M27" s="37"/>
-      <x:c r="N27" s="37"/>
-      <x:c r="O27" s="37"/>
+      <x:c r="B27" s="38"/>
+      <x:c r="C27" s="38"/>
+      <x:c r="D27" s="38"/>
+      <x:c r="E27" s="38"/>
+      <x:c r="F27" s="38"/>
+      <x:c r="G27" s="38"/>
+      <x:c r="H27" s="38"/>
+      <x:c r="I27" s="38"/>
+      <x:c r="J27" s="38"/>
+      <x:c r="K27" s="38"/>
+      <x:c r="L27" s="38"/>
+      <x:c r="M27" s="38"/>
+      <x:c r="N27" s="38"/>
+      <x:c r="O27" s="38"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" t="str">
         <x:v>Utilities</x:v>
       </x:c>
-      <x:c r="B28" s="37"/>
-      <x:c r="C28" s="37"/>
-      <x:c r="D28" s="37"/>
-      <x:c r="E28" s="37"/>
-      <x:c r="F28" s="37"/>
-      <x:c r="G28" s="37"/>
-      <x:c r="H28" s="37"/>
-      <x:c r="I28" s="37"/>
-      <x:c r="J28" s="37"/>
-      <x:c r="K28" s="37"/>
-      <x:c r="L28" s="37"/>
-      <x:c r="M28" s="37"/>
-      <x:c r="N28" s="37"/>
-      <x:c r="O28" s="37"/>
+      <x:c r="B28" s="38"/>
+      <x:c r="C28" s="38"/>
+      <x:c r="D28" s="38"/>
+      <x:c r="E28" s="38"/>
+      <x:c r="F28" s="38"/>
+      <x:c r="G28" s="38"/>
+      <x:c r="H28" s="38"/>
+      <x:c r="I28" s="38"/>
+      <x:c r="J28" s="38"/>
+      <x:c r="K28" s="38"/>
+      <x:c r="L28" s="38"/>
+      <x:c r="M28" s="38"/>
+      <x:c r="N28" s="38"/>
+      <x:c r="O28" s="38"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" t="str">
         <x:v>Insurance</x:v>
       </x:c>
-      <x:c r="B29" s="37"/>
-      <x:c r="C29" s="37"/>
-      <x:c r="D29" s="37"/>
-      <x:c r="E29" s="37"/>
-      <x:c r="F29" s="37"/>
-      <x:c r="G29" s="37"/>
-      <x:c r="H29" s="37"/>
-      <x:c r="I29" s="37"/>
-      <x:c r="J29" s="37"/>
-      <x:c r="K29" s="37"/>
-      <x:c r="L29" s="37"/>
-      <x:c r="M29" s="37"/>
-      <x:c r="N29" s="37"/>
-      <x:c r="O29" s="37"/>
+      <x:c r="B29" s="38"/>
+      <x:c r="C29" s="38"/>
+      <x:c r="D29" s="38"/>
+      <x:c r="E29" s="38"/>
+      <x:c r="F29" s="38"/>
+      <x:c r="G29" s="38"/>
+      <x:c r="H29" s="38"/>
+      <x:c r="I29" s="38"/>
+      <x:c r="J29" s="38"/>
+      <x:c r="K29" s="38"/>
+      <x:c r="L29" s="38"/>
+      <x:c r="M29" s="38"/>
+      <x:c r="N29" s="38"/>
+      <x:c r="O29" s="38"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" t="str">
         <x:v>Software and subscriptions</x:v>
       </x:c>
-      <x:c r="B30" s="37"/>
-      <x:c r="C30" s="37"/>
-      <x:c r="D30" s="37"/>
-      <x:c r="E30" s="37"/>
-      <x:c r="F30" s="37"/>
-      <x:c r="G30" s="37"/>
-      <x:c r="H30" s="37"/>
-      <x:c r="I30" s="37"/>
-      <x:c r="J30" s="37"/>
-      <x:c r="K30" s="37"/>
-      <x:c r="L30" s="37"/>
-      <x:c r="M30" s="37"/>
-      <x:c r="N30" s="37"/>
-      <x:c r="O30" s="37"/>
+      <x:c r="B30" s="38"/>
+      <x:c r="C30" s="38"/>
+      <x:c r="D30" s="38"/>
+      <x:c r="E30" s="38"/>
+      <x:c r="F30" s="38"/>
+      <x:c r="G30" s="38"/>
+      <x:c r="H30" s="38"/>
+      <x:c r="I30" s="38"/>
+      <x:c r="J30" s="38"/>
+      <x:c r="K30" s="38"/>
+      <x:c r="L30" s="38"/>
+      <x:c r="M30" s="38"/>
+      <x:c r="N30" s="38"/>
+      <x:c r="O30" s="38"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" t="str">
         <x:v>Marketing</x:v>
       </x:c>
-      <x:c r="B31" s="37"/>
-      <x:c r="C31" s="37"/>
-      <x:c r="D31" s="37"/>
-      <x:c r="E31" s="37"/>
-      <x:c r="F31" s="37"/>
-      <x:c r="G31" s="37"/>
-      <x:c r="H31" s="37"/>
-      <x:c r="I31" s="37"/>
-      <x:c r="J31" s="37"/>
-      <x:c r="K31" s="37"/>
-      <x:c r="L31" s="37"/>
-      <x:c r="M31" s="37"/>
-      <x:c r="N31" s="37"/>
-      <x:c r="O31" s="37"/>
+      <x:c r="B31" s="38"/>
+      <x:c r="C31" s="38"/>
+      <x:c r="D31" s="38"/>
+      <x:c r="E31" s="38"/>
+      <x:c r="F31" s="38"/>
+      <x:c r="G31" s="38"/>
+      <x:c r="H31" s="38"/>
+      <x:c r="I31" s="38"/>
+      <x:c r="J31" s="38"/>
+      <x:c r="K31" s="38"/>
+      <x:c r="L31" s="38"/>
+      <x:c r="M31" s="38"/>
+      <x:c r="N31" s="38"/>
+      <x:c r="O31" s="38"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" t="str">
         <x:v>Professional services</x:v>
       </x:c>
-      <x:c r="B32" s="37"/>
-      <x:c r="C32" s="37"/>
-      <x:c r="D32" s="37"/>
-      <x:c r="E32" s="37"/>
-      <x:c r="F32" s="37"/>
-      <x:c r="G32" s="37"/>
-      <x:c r="H32" s="37"/>
-      <x:c r="I32" s="37"/>
-      <x:c r="J32" s="37"/>
-      <x:c r="K32" s="37"/>
-      <x:c r="L32" s="37"/>
-      <x:c r="M32" s="37"/>
-      <x:c r="N32" s="37"/>
-      <x:c r="O32" s="37"/>
+      <x:c r="B32" s="38"/>
+      <x:c r="C32" s="38"/>
+      <x:c r="D32" s="38"/>
+      <x:c r="E32" s="38"/>
+      <x:c r="F32" s="38"/>
+      <x:c r="G32" s="38"/>
+      <x:c r="H32" s="38"/>
+      <x:c r="I32" s="38"/>
+      <x:c r="J32" s="38"/>
+      <x:c r="K32" s="38"/>
+      <x:c r="L32" s="38"/>
+      <x:c r="M32" s="38"/>
+      <x:c r="N32" s="38"/>
+      <x:c r="O32" s="38"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" t="str">
         <x:v>Freight, vehicles and travel</x:v>
       </x:c>
-      <x:c r="B33" s="37"/>
-      <x:c r="C33" s="37"/>
-      <x:c r="D33" s="37"/>
-      <x:c r="E33" s="37"/>
-      <x:c r="F33" s="37"/>
-      <x:c r="G33" s="37"/>
-      <x:c r="H33" s="37"/>
-      <x:c r="I33" s="37"/>
-      <x:c r="J33" s="37"/>
-      <x:c r="K33" s="37"/>
-      <x:c r="L33" s="37"/>
-      <x:c r="M33" s="37"/>
-      <x:c r="N33" s="37"/>
-      <x:c r="O33" s="37"/>
+      <x:c r="B33" s="38"/>
+      <x:c r="C33" s="38"/>
+      <x:c r="D33" s="38"/>
+      <x:c r="E33" s="38"/>
+      <x:c r="F33" s="38"/>
+      <x:c r="G33" s="38"/>
+      <x:c r="H33" s="38"/>
+      <x:c r="I33" s="38"/>
+      <x:c r="J33" s="38"/>
+      <x:c r="K33" s="38"/>
+      <x:c r="L33" s="38"/>
+      <x:c r="M33" s="38"/>
+      <x:c r="N33" s="38"/>
+      <x:c r="O33" s="38"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" t="str">
         <x:v>GST / BAS payments</x:v>
       </x:c>
-      <x:c r="B34" s="37"/>
-      <x:c r="C34" s="37"/>
-      <x:c r="D34" s="37"/>
-      <x:c r="E34" s="37"/>
-      <x:c r="F34" s="37"/>
-      <x:c r="G34" s="37"/>
-      <x:c r="H34" s="37"/>
-      <x:c r="I34" s="37"/>
-      <x:c r="J34" s="37"/>
-      <x:c r="K34" s="37"/>
-      <x:c r="L34" s="37"/>
-      <x:c r="M34" s="37"/>
-      <x:c r="N34" s="37"/>
-      <x:c r="O34" s="37"/>
+      <x:c r="B34" s="38"/>
+      <x:c r="C34" s="38"/>
+      <x:c r="D34" s="38"/>
+      <x:c r="E34" s="38"/>
+      <x:c r="F34" s="38"/>
+      <x:c r="G34" s="38"/>
+      <x:c r="H34" s="38"/>
+      <x:c r="I34" s="38"/>
+      <x:c r="J34" s="38"/>
+      <x:c r="K34" s="38"/>
+      <x:c r="L34" s="38"/>
+      <x:c r="M34" s="38"/>
+      <x:c r="N34" s="38"/>
+      <x:c r="O34" s="38"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" t="str">
         <x:v>PAYG income tax instalments</x:v>
       </x:c>
-      <x:c r="B35" s="37"/>
-      <x:c r="C35" s="37"/>
-      <x:c r="D35" s="37"/>
-      <x:c r="E35" s="37"/>
-      <x:c r="F35" s="37"/>
-      <x:c r="G35" s="37"/>
-      <x:c r="H35" s="37"/>
-      <x:c r="I35" s="37"/>
-      <x:c r="J35" s="37"/>
-      <x:c r="K35" s="37"/>
-      <x:c r="L35" s="37"/>
-      <x:c r="M35" s="37"/>
-      <x:c r="N35" s="37"/>
-      <x:c r="O35" s="37"/>
+      <x:c r="B35" s="38"/>
+      <x:c r="C35" s="38"/>
+      <x:c r="D35" s="38"/>
+      <x:c r="E35" s="38"/>
+      <x:c r="F35" s="38"/>
+      <x:c r="G35" s="38"/>
+      <x:c r="H35" s="38"/>
+      <x:c r="I35" s="38"/>
+      <x:c r="J35" s="38"/>
+      <x:c r="K35" s="38"/>
+      <x:c r="L35" s="38"/>
+      <x:c r="M35" s="38"/>
+      <x:c r="N35" s="38"/>
+      <x:c r="O35" s="38"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" t="str">
         <x:v>FBT / other tax</x:v>
       </x:c>
-      <x:c r="B36" s="37"/>
-      <x:c r="C36" s="37"/>
-      <x:c r="D36" s="37"/>
-      <x:c r="E36" s="37"/>
-      <x:c r="F36" s="37"/>
-      <x:c r="G36" s="37"/>
-      <x:c r="H36" s="37"/>
-      <x:c r="I36" s="37"/>
-      <x:c r="J36" s="37"/>
-      <x:c r="K36" s="37"/>
-      <x:c r="L36" s="37"/>
-      <x:c r="M36" s="37"/>
-      <x:c r="N36" s="37"/>
-      <x:c r="O36" s="37"/>
+      <x:c r="B36" s="38"/>
+      <x:c r="C36" s="38"/>
+      <x:c r="D36" s="38"/>
+      <x:c r="E36" s="38"/>
+      <x:c r="F36" s="38"/>
+      <x:c r="G36" s="38"/>
+      <x:c r="H36" s="38"/>
+      <x:c r="I36" s="38"/>
+      <x:c r="J36" s="38"/>
+      <x:c r="K36" s="38"/>
+      <x:c r="L36" s="38"/>
+      <x:c r="M36" s="38"/>
+      <x:c r="N36" s="38"/>
+      <x:c r="O36" s="38"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" t="str">
         <x:v>Interest and bank fees</x:v>
       </x:c>
-      <x:c r="B37" s="37"/>
-      <x:c r="C37" s="37"/>
-      <x:c r="D37" s="37"/>
-      <x:c r="E37" s="37"/>
-      <x:c r="F37" s="37"/>
-      <x:c r="G37" s="37"/>
-      <x:c r="H37" s="37"/>
-      <x:c r="I37" s="37"/>
-      <x:c r="J37" s="37"/>
-      <x:c r="K37" s="37"/>
-      <x:c r="L37" s="37"/>
-      <x:c r="M37" s="37"/>
-      <x:c r="N37" s="37"/>
-      <x:c r="O37" s="37"/>
+      <x:c r="B37" s="38"/>
+      <x:c r="C37" s="38"/>
+      <x:c r="D37" s="38"/>
+      <x:c r="E37" s="38"/>
+      <x:c r="F37" s="38"/>
+      <x:c r="G37" s="38"/>
+      <x:c r="H37" s="38"/>
+      <x:c r="I37" s="38"/>
+      <x:c r="J37" s="38"/>
+      <x:c r="K37" s="38"/>
+      <x:c r="L37" s="38"/>
+      <x:c r="M37" s="38"/>
+      <x:c r="N37" s="38"/>
+      <x:c r="O37" s="38"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" t="str">
         <x:v>Loan principal</x:v>
       </x:c>
-      <x:c r="B38" s="37"/>
-      <x:c r="C38" s="37"/>
-      <x:c r="D38" s="37"/>
-      <x:c r="E38" s="37"/>
-      <x:c r="F38" s="37"/>
-      <x:c r="G38" s="37"/>
-      <x:c r="H38" s="37"/>
-      <x:c r="I38" s="37"/>
-      <x:c r="J38" s="37"/>
-      <x:c r="K38" s="37"/>
-      <x:c r="L38" s="37"/>
-      <x:c r="M38" s="37"/>
-      <x:c r="N38" s="37"/>
-      <x:c r="O38" s="37"/>
+      <x:c r="B38" s="38"/>
+      <x:c r="C38" s="38"/>
+      <x:c r="D38" s="38"/>
+      <x:c r="E38" s="38"/>
+      <x:c r="F38" s="38"/>
+      <x:c r="G38" s="38"/>
+      <x:c r="H38" s="38"/>
+      <x:c r="I38" s="38"/>
+      <x:c r="J38" s="38"/>
+      <x:c r="K38" s="38"/>
+      <x:c r="L38" s="38"/>
+      <x:c r="M38" s="38"/>
+      <x:c r="N38" s="38"/>
+      <x:c r="O38" s="38"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" t="str">
         <x:v>Capital expenditure</x:v>
       </x:c>
-      <x:c r="B39" s="37"/>
-      <x:c r="C39" s="37"/>
-      <x:c r="D39" s="37"/>
-      <x:c r="E39" s="37"/>
-      <x:c r="F39" s="37"/>
-      <x:c r="G39" s="37"/>
-      <x:c r="H39" s="37"/>
-      <x:c r="I39" s="37"/>
-      <x:c r="J39" s="37"/>
-      <x:c r="K39" s="37"/>
-      <x:c r="L39" s="37"/>
-      <x:c r="M39" s="37"/>
-      <x:c r="N39" s="37"/>
-      <x:c r="O39" s="37"/>
+      <x:c r="B39" s="38"/>
+      <x:c r="C39" s="38"/>
+      <x:c r="D39" s="38"/>
+      <x:c r="E39" s="38"/>
+      <x:c r="F39" s="38"/>
+      <x:c r="G39" s="38"/>
+      <x:c r="H39" s="38"/>
+      <x:c r="I39" s="38"/>
+      <x:c r="J39" s="38"/>
+      <x:c r="K39" s="38"/>
+      <x:c r="L39" s="38"/>
+      <x:c r="M39" s="38"/>
+      <x:c r="N39" s="38"/>
+      <x:c r="O39" s="38"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" t="str">
         <x:v>Dividends / distributions</x:v>
       </x:c>
-      <x:c r="B40" s="37"/>
-      <x:c r="C40" s="37"/>
-      <x:c r="D40" s="37"/>
-      <x:c r="E40" s="37"/>
-      <x:c r="F40" s="37"/>
-      <x:c r="G40" s="37"/>
-      <x:c r="H40" s="37"/>
-      <x:c r="I40" s="37"/>
-      <x:c r="J40" s="37"/>
-      <x:c r="K40" s="37"/>
-      <x:c r="L40" s="37"/>
-      <x:c r="M40" s="37"/>
-      <x:c r="N40" s="37"/>
-      <x:c r="O40" s="37"/>
+      <x:c r="B40" s="38"/>
+      <x:c r="C40" s="38"/>
+      <x:c r="D40" s="38"/>
+      <x:c r="E40" s="38"/>
+      <x:c r="F40" s="38"/>
+      <x:c r="G40" s="38"/>
+      <x:c r="H40" s="38"/>
+      <x:c r="I40" s="38"/>
+      <x:c r="J40" s="38"/>
+      <x:c r="K40" s="38"/>
+      <x:c r="L40" s="38"/>
+      <x:c r="M40" s="38"/>
+      <x:c r="N40" s="38"/>
+      <x:c r="O40" s="38"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" t="str">
         <x:v>Other operating</x:v>
       </x:c>
-      <x:c r="B41" s="37"/>
-      <x:c r="C41" s="37"/>
-      <x:c r="D41" s="37"/>
-      <x:c r="E41" s="37"/>
-      <x:c r="F41" s="37"/>
-      <x:c r="G41" s="37"/>
-      <x:c r="H41" s="37"/>
-      <x:c r="I41" s="37"/>
-      <x:c r="J41" s="37"/>
-      <x:c r="K41" s="37"/>
-      <x:c r="L41" s="37"/>
-      <x:c r="M41" s="37"/>
-      <x:c r="N41" s="37"/>
-      <x:c r="O41" s="37"/>
+      <x:c r="B41" s="38"/>
+      <x:c r="C41" s="38"/>
+      <x:c r="D41" s="38"/>
+      <x:c r="E41" s="38"/>
+      <x:c r="F41" s="38"/>
+      <x:c r="G41" s="38"/>
+      <x:c r="H41" s="38"/>
+      <x:c r="I41" s="38"/>
+      <x:c r="J41" s="38"/>
+      <x:c r="K41" s="38"/>
+      <x:c r="L41" s="38"/>
+      <x:c r="M41" s="38"/>
+      <x:c r="N41" s="38"/>
+      <x:c r="O41" s="38"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" t="str">
         <x:v>Scenario payment adjustment</x:v>
       </x:c>
-      <x:c r="B42" s="37"/>
-      <x:c r="C42" s="37"/>
-      <x:c r="D42" s="37"/>
-      <x:c r="E42" s="37"/>
-      <x:c r="F42" s="37"/>
-      <x:c r="G42" s="37"/>
-      <x:c r="H42" s="37"/>
-      <x:c r="I42" s="37"/>
-      <x:c r="J42" s="37"/>
-      <x:c r="K42" s="37"/>
-      <x:c r="L42" s="37"/>
-      <x:c r="M42" s="37"/>
-      <x:c r="N42" s="37"/>
-      <x:c r="O42" s="37"/>
+      <x:c r="B42" s="38"/>
+      <x:c r="C42" s="38"/>
+      <x:c r="D42" s="38"/>
+      <x:c r="E42" s="38"/>
+      <x:c r="F42" s="38"/>
+      <x:c r="G42" s="38"/>
+      <x:c r="H42" s="38"/>
+      <x:c r="I42" s="38"/>
+      <x:c r="J42" s="38"/>
+      <x:c r="K42" s="38"/>
+      <x:c r="L42" s="38"/>
+      <x:c r="M42" s="38"/>
+      <x:c r="N42" s="38"/>
+      <x:c r="O42" s="38"/>
     </x:row>
     <x:row r="43">
-      <x:c r="A43" s="36" t="str">
+      <x:c r="A43" s="37" t="str">
         <x:v>Total cash payments</x:v>
       </x:c>
-      <x:c r="B43" s="38"/>
-      <x:c r="C43" s="38"/>
-      <x:c r="D43" s="38"/>
-      <x:c r="E43" s="38"/>
-      <x:c r="F43" s="38"/>
-      <x:c r="G43" s="38"/>
-      <x:c r="H43" s="38"/>
-      <x:c r="I43" s="38"/>
-      <x:c r="J43" s="38"/>
-      <x:c r="K43" s="38"/>
-      <x:c r="L43" s="38"/>
-      <x:c r="M43" s="38"/>
-      <x:c r="N43" s="38"/>
-      <x:c r="O43" s="38"/>
+      <x:c r="B43" s="39"/>
+      <x:c r="C43" s="39"/>
+      <x:c r="D43" s="39"/>
+      <x:c r="E43" s="39"/>
+      <x:c r="F43" s="39"/>
+      <x:c r="G43" s="39"/>
+      <x:c r="H43" s="39"/>
+      <x:c r="I43" s="39"/>
+      <x:c r="J43" s="39"/>
+      <x:c r="K43" s="39"/>
+      <x:c r="L43" s="39"/>
+      <x:c r="M43" s="39"/>
+      <x:c r="N43" s="39"/>
+      <x:c r="O43" s="39"/>
     </x:row>
     <x:row r="44">
-      <x:c r="B44" s="37"/>
-      <x:c r="C44" s="37"/>
-      <x:c r="D44" s="37"/>
-      <x:c r="E44" s="37"/>
-      <x:c r="F44" s="37"/>
-      <x:c r="G44" s="37"/>
-      <x:c r="H44" s="37"/>
-      <x:c r="I44" s="37"/>
-      <x:c r="J44" s="37"/>
-      <x:c r="K44" s="37"/>
-      <x:c r="L44" s="37"/>
-      <x:c r="M44" s="37"/>
-      <x:c r="N44" s="37"/>
-      <x:c r="O44" s="37"/>
+      <x:c r="B44" s="38"/>
+      <x:c r="C44" s="38"/>
+      <x:c r="D44" s="38"/>
+      <x:c r="E44" s="38"/>
+      <x:c r="F44" s="38"/>
+      <x:c r="G44" s="38"/>
+      <x:c r="H44" s="38"/>
+      <x:c r="I44" s="38"/>
+      <x:c r="J44" s="38"/>
+      <x:c r="K44" s="38"/>
+      <x:c r="L44" s="38"/>
+      <x:c r="M44" s="38"/>
+      <x:c r="N44" s="38"/>
+      <x:c r="O44" s="38"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="14" t="str">
         <x:v>CASH POSITION</x:v>
       </x:c>
-      <x:c r="B45" s="39"/>
-      <x:c r="C45" s="39"/>
-      <x:c r="D45" s="39"/>
-      <x:c r="E45" s="39"/>
-      <x:c r="F45" s="39"/>
-      <x:c r="G45" s="39"/>
-      <x:c r="H45" s="39"/>
-      <x:c r="I45" s="39"/>
-      <x:c r="J45" s="39"/>
-      <x:c r="K45" s="39"/>
-      <x:c r="L45" s="39"/>
-      <x:c r="M45" s="39"/>
-      <x:c r="N45" s="39"/>
-      <x:c r="O45" s="39"/>
+      <x:c r="B45" s="40"/>
+      <x:c r="C45" s="40"/>
+      <x:c r="D45" s="40"/>
+      <x:c r="E45" s="40"/>
+      <x:c r="F45" s="40"/>
+      <x:c r="G45" s="40"/>
+      <x:c r="H45" s="40"/>
+      <x:c r="I45" s="40"/>
+      <x:c r="J45" s="40"/>
+      <x:c r="K45" s="40"/>
+      <x:c r="L45" s="40"/>
+      <x:c r="M45" s="40"/>
+      <x:c r="N45" s="40"/>
+      <x:c r="O45" s="40"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" t="str">
         <x:v>Opening cash balance</x:v>
       </x:c>
-      <x:c r="B46" s="37"/>
-      <x:c r="C46" s="37"/>
-      <x:c r="D46" s="37"/>
-      <x:c r="E46" s="37"/>
-      <x:c r="F46" s="37"/>
-      <x:c r="G46" s="37"/>
-      <x:c r="H46" s="37"/>
-      <x:c r="I46" s="37"/>
-      <x:c r="J46" s="37"/>
-      <x:c r="K46" s="37"/>
-      <x:c r="L46" s="37"/>
-      <x:c r="M46" s="37"/>
-      <x:c r="N46" s="37"/>
-      <x:c r="O46" s="37"/>
+      <x:c r="B46" s="38"/>
+      <x:c r="C46" s="38"/>
+      <x:c r="D46" s="38"/>
+      <x:c r="E46" s="38"/>
+      <x:c r="F46" s="38"/>
+      <x:c r="G46" s="38"/>
+      <x:c r="H46" s="38"/>
+      <x:c r="I46" s="38"/>
+      <x:c r="J46" s="38"/>
+      <x:c r="K46" s="38"/>
+      <x:c r="L46" s="38"/>
+      <x:c r="M46" s="38"/>
+      <x:c r="N46" s="38"/>
+      <x:c r="O46" s="38"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" t="str">
         <x:v>Net cash movement</x:v>
       </x:c>
-      <x:c r="B47" s="37"/>
-      <x:c r="C47" s="37"/>
-      <x:c r="D47" s="37"/>
-      <x:c r="E47" s="37"/>
-      <x:c r="F47" s="37"/>
-      <x:c r="G47" s="37"/>
-      <x:c r="H47" s="37"/>
-      <x:c r="I47" s="37"/>
-      <x:c r="J47" s="37"/>
-      <x:c r="K47" s="37"/>
-      <x:c r="L47" s="37"/>
-      <x:c r="M47" s="37"/>
-      <x:c r="N47" s="37"/>
-      <x:c r="O47" s="37"/>
+      <x:c r="B47" s="38"/>
+      <x:c r="C47" s="38"/>
+      <x:c r="D47" s="38"/>
+      <x:c r="E47" s="38"/>
+      <x:c r="F47" s="38"/>
+      <x:c r="G47" s="38"/>
+      <x:c r="H47" s="38"/>
+      <x:c r="I47" s="38"/>
+      <x:c r="J47" s="38"/>
+      <x:c r="K47" s="38"/>
+      <x:c r="L47" s="38"/>
+      <x:c r="M47" s="38"/>
+      <x:c r="N47" s="38"/>
+      <x:c r="O47" s="38"/>
     </x:row>
     <x:row r="48">
-      <x:c r="A48" s="36" t="str">
+      <x:c r="A48" s="37" t="str">
         <x:v>Closing cash balance</x:v>
       </x:c>
-      <x:c r="B48" s="38"/>
-      <x:c r="C48" s="38"/>
-      <x:c r="D48" s="38"/>
-      <x:c r="E48" s="38"/>
-      <x:c r="F48" s="38"/>
-      <x:c r="G48" s="38"/>
-      <x:c r="H48" s="38"/>
-      <x:c r="I48" s="38"/>
-      <x:c r="J48" s="38"/>
-      <x:c r="K48" s="38"/>
-      <x:c r="L48" s="38"/>
-      <x:c r="M48" s="38"/>
-      <x:c r="N48" s="38"/>
-      <x:c r="O48" s="38"/>
+      <x:c r="B48" s="39"/>
+      <x:c r="C48" s="39"/>
+      <x:c r="D48" s="39"/>
+      <x:c r="E48" s="39"/>
+      <x:c r="F48" s="39"/>
+      <x:c r="G48" s="39"/>
+      <x:c r="H48" s="39"/>
+      <x:c r="I48" s="39"/>
+      <x:c r="J48" s="39"/>
+      <x:c r="K48" s="39"/>
+      <x:c r="L48" s="39"/>
+      <x:c r="M48" s="39"/>
+      <x:c r="N48" s="39"/>
+      <x:c r="O48" s="39"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" t="str">
         <x:v>Minimum cash buffer</x:v>
       </x:c>
-      <x:c r="B49" s="37"/>
-      <x:c r="C49" s="37"/>
-      <x:c r="D49" s="37"/>
-      <x:c r="E49" s="37"/>
-      <x:c r="F49" s="37"/>
-      <x:c r="G49" s="37"/>
-      <x:c r="H49" s="37"/>
-      <x:c r="I49" s="37"/>
-      <x:c r="J49" s="37"/>
-      <x:c r="K49" s="37"/>
-      <x:c r="L49" s="37"/>
-      <x:c r="M49" s="37"/>
-      <x:c r="N49" s="37"/>
-      <x:c r="O49" s="37"/>
+      <x:c r="B49" s="38"/>
+      <x:c r="C49" s="38"/>
+      <x:c r="D49" s="38"/>
+      <x:c r="E49" s="38"/>
+      <x:c r="F49" s="38"/>
+      <x:c r="G49" s="38"/>
+      <x:c r="H49" s="38"/>
+      <x:c r="I49" s="38"/>
+      <x:c r="J49" s="38"/>
+      <x:c r="K49" s="38"/>
+      <x:c r="L49" s="38"/>
+      <x:c r="M49" s="38"/>
+      <x:c r="N49" s="38"/>
+      <x:c r="O49" s="38"/>
     </x:row>
     <x:row r="50">
-      <x:c r="A50" s="36" t="str">
+      <x:c r="A50" s="37" t="str">
         <x:v>Headroom / (gap)</x:v>
       </x:c>
-      <x:c r="B50" s="38"/>
-      <x:c r="C50" s="38"/>
-      <x:c r="D50" s="38"/>
-      <x:c r="E50" s="38"/>
-      <x:c r="F50" s="38"/>
-      <x:c r="G50" s="38"/>
-      <x:c r="H50" s="38"/>
-      <x:c r="I50" s="38"/>
-      <x:c r="J50" s="38"/>
-      <x:c r="K50" s="38"/>
-      <x:c r="L50" s="38"/>
-      <x:c r="M50" s="38"/>
-      <x:c r="N50" s="38"/>
-      <x:c r="O50" s="38"/>
+      <x:c r="B50" s="39"/>
+      <x:c r="C50" s="39"/>
+      <x:c r="D50" s="39"/>
+      <x:c r="E50" s="39"/>
+      <x:c r="F50" s="39"/>
+      <x:c r="G50" s="39"/>
+      <x:c r="H50" s="39"/>
+      <x:c r="I50" s="39"/>
+      <x:c r="J50" s="39"/>
+      <x:c r="K50" s="39"/>
+      <x:c r="L50" s="39"/>
+      <x:c r="M50" s="39"/>
+      <x:c r="N50" s="39"/>
+      <x:c r="O50" s="39"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" t="str">
@@ -2097,46 +2099,46 @@
       <x:c r="N2" s="8"/>
     </x:row>
     <x:row r="5" ht="32" customHeight="1">
-      <x:c r="A5" s="27" t="str">
+      <x:c r="A5" s="28" t="str">
         <x:v>Week</x:v>
       </x:c>
-      <x:c r="B5" s="27" t="str">
+      <x:c r="B5" s="28" t="str">
         <x:v>Week commencing</x:v>
       </x:c>
-      <x:c r="C5" s="27" t="str">
+      <x:c r="C5" s="28" t="str">
         <x:v>Week ending</x:v>
       </x:c>
-      <x:c r="D5" s="27" t="str">
+      <x:c r="D5" s="28" t="str">
         <x:v>Forecast receipts</x:v>
       </x:c>
-      <x:c r="E5" s="27" t="str">
+      <x:c r="E5" s="28" t="str">
         <x:v>Actual receipts</x:v>
       </x:c>
-      <x:c r="F5" s="27" t="str">
+      <x:c r="F5" s="28" t="str">
         <x:v>Receipt variance</x:v>
       </x:c>
-      <x:c r="G5" s="27" t="str">
+      <x:c r="G5" s="28" t="str">
         <x:v>Forecast payments</x:v>
       </x:c>
-      <x:c r="H5" s="27" t="str">
+      <x:c r="H5" s="28" t="str">
         <x:v>Actual payments</x:v>
       </x:c>
-      <x:c r="I5" s="27" t="str">
+      <x:c r="I5" s="28" t="str">
         <x:v>Payment variance</x:v>
       </x:c>
-      <x:c r="J5" s="27" t="str">
+      <x:c r="J5" s="28" t="str">
         <x:v>Forecast closing cash</x:v>
       </x:c>
-      <x:c r="K5" s="27" t="str">
+      <x:c r="K5" s="28" t="str">
         <x:v>Actual closing cash</x:v>
       </x:c>
-      <x:c r="L5" s="27" t="str">
+      <x:c r="L5" s="28" t="str">
         <x:v>Cash variance</x:v>
       </x:c>
-      <x:c r="M5" s="27" t="str">
+      <x:c r="M5" s="28" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="N5" s="27" t="str">
+      <x:c r="N5" s="28" t="str">
         <x:v>Commentary / action</x:v>
       </x:c>
     </x:row>
@@ -2279,16 +2281,16 @@
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="40" t="str">
+      <x:c r="A6" s="41" t="str">
         <x:v>MODEL STATUS: prepared for formula-driven integrity checks</x:v>
       </x:c>
-      <x:c r="B6" s="40"/>
-      <x:c r="C6" s="40"/>
-      <x:c r="D6" s="40"/>
-      <x:c r="E6" s="40"/>
-      <x:c r="F6" s="40"/>
-      <x:c r="G6" s="40"/>
-      <x:c r="H6" s="40"/>
+      <x:c r="B6" s="41"/>
+      <x:c r="C6" s="41"/>
+      <x:c r="D6" s="41"/>
+      <x:c r="E6" s="41"/>
+      <x:c r="F6" s="41"/>
+      <x:c r="G6" s="41"/>
+      <x:c r="H6" s="41"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="14" t="str">
@@ -2311,22 +2313,22 @@
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="42" t="str">
+      <x:c r="A11" s="43" t="str">
         <x:v>Statutory dates and classifications require confirmation for your entity, reporting cycle and agent arrangements.</x:v>
       </x:c>
-      <x:c r="B11" s="42"/>
-      <x:c r="C11" s="42"/>
-      <x:c r="D11" s="42"/>
-      <x:c r="E11" s="42"/>
-      <x:c r="F11" s="42"/>
+      <x:c r="B11" s="43"/>
+      <x:c r="C11" s="43"/>
+      <x:c r="D11" s="43"/>
+      <x:c r="E11" s="43"/>
+      <x:c r="F11" s="43"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="42"/>
-      <x:c r="B12" s="42"/>
-      <x:c r="C12" s="42"/>
-      <x:c r="D12" s="42"/>
-      <x:c r="E12" s="42"/>
-      <x:c r="F12" s="42"/>
+      <x:c r="A12" s="43"/>
+      <x:c r="B12" s="43"/>
+      <x:c r="C12" s="43"/>
+      <x:c r="D12" s="43"/>
+      <x:c r="E12" s="43"/>
+      <x:c r="F12" s="43"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
feat: add 13-week forecast engine
</commit_message>
<xml_diff>
--- a/templates/13-week-cash-flow-forecast.xlsx
+++ b/templates/13-week-cash-flow-forecast.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R8422424ed3254cd8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R5c91082a1e444c94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R2078ee11a4bc45e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13-Week Forecast" sheetId="4" r:id="R257a5564b1894f69"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Review" sheetId="5" r:id="R6a0c7ecdfe164073"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks &amp; Sources" sheetId="6" r:id="R66855269f32c48a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R163eef40803243ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R36a323b4bd524392"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R55e1d91aef2144cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13-Week Forecast" sheetId="4" r:id="R3a5216492bc244a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Review" sheetId="5" r:id="R6e15a48bc1404b42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks &amp; Sources" sheetId="6" r:id="R40686c5f31a64d21"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="CashFlowScenario">'Assumptions'!$B$12</x:definedName>
@@ -15,6 +15,59 @@
     <x:definedName name="CashFlowScenarioList">'Assumptions'!$B$15:$B$17</x:definedName>
   </x:definedNames>
 </x:workbook>
+</file>
+
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:authors>
+    <x:author>tc={E28899D8-E974-D419-CBA0-A3EAED613B76}</x:author>
+    <x:author>tc={17D25D66-7DB0-58F0-CE5E-E2EB2DCDA11F}</x:author>
+    <x:author>tc={6D6F189E-71DD-5AB0-A5B5-8089484B0A68}</x:author>
+    <x:author>tc={E870F557-83E1-4DD3-E5B6-7E48039B894E}</x:author>
+  </x:authors>
+  <x:commentList>
+    <x:comment ref="B18" authorId="0">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Scenario receipt adjustment applies the selected scenario only to customer receipts and cash / EFTPOS sales. Week 1 is Actual, so the adjustment is zero.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="B42" authorId="1">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Scenario payment adjustment applies the selected scenario only to suppliers, marketing, freight / vehicles / travel and other operating payments. Week 1 is Actual, so the adjustment is zero.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="B34" authorId="2">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    GST / BAS cash timing is illustrative. Confirm your entity's reporting cycle, due date and payment arrangement before relying on this forecast.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="B35" authorId="3">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    PAYG income-tax instalment timing and amount are illustrative. Confirm the applicable ATO notice and adviser instructions.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+  </x:commentList>
+</x:comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -28,7 +81,7 @@
     <x:numFmt numFmtId="201" formatCode="&quot;$&quot;#,##0;[Red](&quot;$&quot;#,##0);-"/>
     <x:numFmt numFmtId="202" formatCode="0.0%"/>
   </x:numFmts>
-  <x:fonts count="13">
+  <x:fonts count="14">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -90,6 +143,12 @@
       <x:b/>
       <x:sz val="11"/>
       <x:color rgb="FF04001F"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF000000"/>
       <x:name val="Aptos"/>
     </x:font>
     <x:font>
@@ -163,7 +222,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="44">
+  <x:cellXfs count="50">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -216,10 +275,16 @@
     <x:xf numFmtId="0" fontId="10" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="12" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
@@ -230,7 +295,48 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
+  <x:dxfs count="3">
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFC00000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFCE4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF5C2D91"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFDED9E8"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF008000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFE2F0D9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+  </x:dxfs>
 </x:styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
+  <xltc:person displayName="User" id="{D4E71844-CD76-4BEE-BAA9-387BBDF1B51C}"/>
+</xltc:personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -424,6 +530,23 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
+<xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
+  <xltc:threadedComment ref="B18" dT="2026-08-26T13:22:07.159" personId="{D4E71844-CD76-4BEE-BAA9-387BBDF1B51C}" id="{E28899D8-E974-D419-CBA0-A3EAED613B76}">
+    <xltc:text>Scenario receipt adjustment applies the selected scenario only to customer receipts and cash / EFTPOS sales. Week 1 is Actual, so the adjustment is zero.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="B42" dT="2026-08-26T13:22:07.159" personId="{D4E71844-CD76-4BEE-BAA9-387BBDF1B51C}" id="{17D25D66-7DB0-58F0-CE5E-E2EB2DCDA11F}">
+    <xltc:text>Scenario payment adjustment applies the selected scenario only to suppliers, marketing, freight / vehicles / travel and other operating payments. Week 1 is Actual, so the adjustment is zero.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="B34" dT="2026-08-26T13:22:07.159" personId="{D4E71844-CD76-4BEE-BAA9-387BBDF1B51C}" id="{6D6F189E-71DD-5AB0-A5B5-8089484B0A68}">
+    <xltc:text>GST / BAS cash timing is illustrative. Confirm your entity's reporting cycle, due date and payment arrangement before relying on this forecast.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="B35" dT="2026-08-26T13:22:07.159" personId="{D4E71844-CD76-4BEE-BAA9-387BBDF1B51C}" id="{E870F557-83E1-4DD3-E5B6-7E48039B894E}">
+    <xltc:text>PAYG income-tax instalment timing and amount are illustrative. Confirm the applicable ATO notice and adviser instructions.</xltc:text>
+  </xltc:threadedComment>
+</xltc:ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
@@ -1080,7 +1203,7 @@
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>Weekly cash-flow structure. The forecast engine and editable operating inputs are added in the next build step.</x:v>
+        <x:v>Blue cells are illustrative weekly inputs. Formula and linked cells update automatically from the Assumptions control panel.</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -1102,42 +1225,55 @@
         <x:v>Week commencing</x:v>
       </x:c>
       <x:c r="B5" s="34" t="n">
+        <x:f>'Assumptions'!$B$8</x:f>
         <x:v>46265</x:v>
       </x:c>
       <x:c r="C5" s="34" t="n">
+        <x:f>B5+7</x:f>
         <x:v>46272</x:v>
       </x:c>
       <x:c r="D5" s="34" t="n">
+        <x:f>C5+7</x:f>
         <x:v>46279</x:v>
       </x:c>
       <x:c r="E5" s="34" t="n">
+        <x:f>D5+7</x:f>
         <x:v>46286</x:v>
       </x:c>
       <x:c r="F5" s="34" t="n">
+        <x:f>E5+7</x:f>
         <x:v>46293</x:v>
       </x:c>
       <x:c r="G5" s="34" t="n">
+        <x:f>F5+7</x:f>
         <x:v>46300</x:v>
       </x:c>
       <x:c r="H5" s="34" t="n">
+        <x:f>G5+7</x:f>
         <x:v>46307</x:v>
       </x:c>
       <x:c r="I5" s="34" t="n">
+        <x:f>H5+7</x:f>
         <x:v>46314</x:v>
       </x:c>
       <x:c r="J5" s="34" t="n">
+        <x:f>I5+7</x:f>
         <x:v>46321</x:v>
       </x:c>
       <x:c r="K5" s="34" t="n">
+        <x:f>J5+7</x:f>
         <x:v>46328</x:v>
       </x:c>
       <x:c r="L5" s="34" t="n">
+        <x:f>K5+7</x:f>
         <x:v>46335</x:v>
       </x:c>
       <x:c r="M5" s="34" t="n">
+        <x:f>L5+7</x:f>
         <x:v>46342</x:v>
       </x:c>
       <x:c r="N5" s="34" t="n">
+        <x:f>M5+7</x:f>
         <x:v>46349</x:v>
       </x:c>
       <x:c r="O5" t="str">
@@ -1149,42 +1285,55 @@
         <x:v>Week ending</x:v>
       </x:c>
       <x:c r="B6" s="34" t="n">
+        <x:f>B5+6</x:f>
         <x:v>46271</x:v>
       </x:c>
       <x:c r="C6" s="34" t="n">
+        <x:f>C5+6</x:f>
         <x:v>46278</x:v>
       </x:c>
       <x:c r="D6" s="34" t="n">
+        <x:f>D5+6</x:f>
         <x:v>46285</x:v>
       </x:c>
       <x:c r="E6" s="34" t="n">
+        <x:f>E5+6</x:f>
         <x:v>46292</x:v>
       </x:c>
       <x:c r="F6" s="34" t="n">
+        <x:f>F5+6</x:f>
         <x:v>46299</x:v>
       </x:c>
       <x:c r="G6" s="34" t="n">
+        <x:f>G5+6</x:f>
         <x:v>46306</x:v>
       </x:c>
       <x:c r="H6" s="34" t="n">
+        <x:f>H5+6</x:f>
         <x:v>46313</x:v>
       </x:c>
       <x:c r="I6" s="34" t="n">
+        <x:f>I5+6</x:f>
         <x:v>46320</x:v>
       </x:c>
       <x:c r="J6" s="34" t="n">
+        <x:f>J5+6</x:f>
         <x:v>46327</x:v>
       </x:c>
       <x:c r="K6" s="34" t="n">
+        <x:f>K5+6</x:f>
         <x:v>46334</x:v>
       </x:c>
       <x:c r="L6" s="34" t="n">
+        <x:f>L5+6</x:f>
         <x:v>46341</x:v>
       </x:c>
       <x:c r="M6" s="34" t="n">
+        <x:f>M5+6</x:f>
         <x:v>46348</x:v>
       </x:c>
       <x:c r="N6" s="34" t="n">
+        <x:f>N5+6</x:f>
         <x:v>46355</x:v>
       </x:c>
       <x:c r="O6" t="str">
@@ -1196,42 +1345,55 @@
         <x:v>Actual / Forecast</x:v>
       </x:c>
       <x:c r="B7" s="35" t="str">
+        <x:f>IF(B6&lt;='Assumptions'!$B$9,"Actual","Forecast")</x:f>
+        <x:v>Actual</x:v>
+      </x:c>
+      <x:c r="C7" s="35" t="str">
+        <x:f>IF(C6&lt;='Assumptions'!$B$9,"Actual","Forecast")</x:f>
         <x:v>Forecast</x:v>
       </x:c>
-      <x:c r="C7" s="35" t="str">
+      <x:c r="D7" s="35" t="str">
+        <x:f>IF(D6&lt;='Assumptions'!$B$9,"Actual","Forecast")</x:f>
         <x:v>Forecast</x:v>
       </x:c>
-      <x:c r="D7" s="35" t="str">
+      <x:c r="E7" s="35" t="str">
+        <x:f>IF(E6&lt;='Assumptions'!$B$9,"Actual","Forecast")</x:f>
         <x:v>Forecast</x:v>
       </x:c>
-      <x:c r="E7" s="35" t="str">
+      <x:c r="F7" s="35" t="str">
+        <x:f>IF(F6&lt;='Assumptions'!$B$9,"Actual","Forecast")</x:f>
         <x:v>Forecast</x:v>
       </x:c>
-      <x:c r="F7" s="35" t="str">
+      <x:c r="G7" s="35" t="str">
+        <x:f>IF(G6&lt;='Assumptions'!$B$9,"Actual","Forecast")</x:f>
         <x:v>Forecast</x:v>
       </x:c>
-      <x:c r="G7" s="35" t="str">
+      <x:c r="H7" s="35" t="str">
+        <x:f>IF(H6&lt;='Assumptions'!$B$9,"Actual","Forecast")</x:f>
         <x:v>Forecast</x:v>
       </x:c>
-      <x:c r="H7" s="35" t="str">
+      <x:c r="I7" s="35" t="str">
+        <x:f>IF(I6&lt;='Assumptions'!$B$9,"Actual","Forecast")</x:f>
         <x:v>Forecast</x:v>
       </x:c>
-      <x:c r="I7" s="35" t="str">
+      <x:c r="J7" s="35" t="str">
+        <x:f>IF(J6&lt;='Assumptions'!$B$9,"Actual","Forecast")</x:f>
         <x:v>Forecast</x:v>
       </x:c>
-      <x:c r="J7" s="35" t="str">
+      <x:c r="K7" s="35" t="str">
+        <x:f>IF(K6&lt;='Assumptions'!$B$9,"Actual","Forecast")</x:f>
         <x:v>Forecast</x:v>
       </x:c>
-      <x:c r="K7" s="35" t="str">
+      <x:c r="L7" s="35" t="str">
+        <x:f>IF(L6&lt;='Assumptions'!$B$9,"Actual","Forecast")</x:f>
         <x:v>Forecast</x:v>
       </x:c>
-      <x:c r="L7" s="35" t="str">
+      <x:c r="M7" s="35" t="str">
+        <x:f>IF(M6&lt;='Assumptions'!$B$9,"Actual","Forecast")</x:f>
         <x:v>Forecast</x:v>
       </x:c>
-      <x:c r="M7" s="35" t="str">
-        <x:v>Forecast</x:v>
-      </x:c>
       <x:c r="N7" s="35" t="str">
+        <x:f>IF(N6&lt;='Assumptions'!$B$9,"Actual","Forecast")</x:f>
         <x:v>Forecast</x:v>
       </x:c>
       <x:c r="O7" t="str"/>
@@ -1259,778 +1421,2024 @@
       <x:c r="A10" t="str">
         <x:v>Customer receipts</x:v>
       </x:c>
-      <x:c r="B10" s="38"/>
-      <x:c r="C10" s="38"/>
-      <x:c r="D10" s="38"/>
-      <x:c r="E10" s="38"/>
-      <x:c r="F10" s="38"/>
-      <x:c r="G10" s="38"/>
-      <x:c r="H10" s="38"/>
-      <x:c r="I10" s="38"/>
-      <x:c r="J10" s="38"/>
-      <x:c r="K10" s="38"/>
-      <x:c r="L10" s="38"/>
-      <x:c r="M10" s="38"/>
-      <x:c r="N10" s="38"/>
-      <x:c r="O10" s="38"/>
+      <x:c r="B10" s="38" t="n">
+        <x:v>118000</x:v>
+      </x:c>
+      <x:c r="C10" s="38" t="n">
+        <x:v>125000</x:v>
+      </x:c>
+      <x:c r="D10" s="38" t="n">
+        <x:v>120000</x:v>
+      </x:c>
+      <x:c r="E10" s="38" t="n">
+        <x:v>115000</x:v>
+      </x:c>
+      <x:c r="F10" s="38" t="n">
+        <x:v>110000</x:v>
+      </x:c>
+      <x:c r="G10" s="38" t="n">
+        <x:v>112000</x:v>
+      </x:c>
+      <x:c r="H10" s="38" t="n">
+        <x:v>105000</x:v>
+      </x:c>
+      <x:c r="I10" s="38" t="n">
+        <x:v>108000</x:v>
+      </x:c>
+      <x:c r="J10" s="38" t="n">
+        <x:v>110000</x:v>
+      </x:c>
+      <x:c r="K10" s="38" t="n">
+        <x:v>116000</x:v>
+      </x:c>
+      <x:c r="L10" s="38" t="n">
+        <x:v>120000</x:v>
+      </x:c>
+      <x:c r="M10" s="38" t="n">
+        <x:v>125000</x:v>
+      </x:c>
+      <x:c r="N10" s="38" t="n">
+        <x:v>130000</x:v>
+      </x:c>
+      <x:c r="O10" s="39" t="n">
+        <x:f>SUM(B10:N10)</x:f>
+        <x:v>1514000</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="str">
         <x:v>Overdue receipts</x:v>
       </x:c>
-      <x:c r="B11" s="38"/>
-      <x:c r="C11" s="38"/>
-      <x:c r="D11" s="38"/>
-      <x:c r="E11" s="38"/>
-      <x:c r="F11" s="38"/>
-      <x:c r="G11" s="38"/>
-      <x:c r="H11" s="38"/>
-      <x:c r="I11" s="38"/>
-      <x:c r="J11" s="38"/>
-      <x:c r="K11" s="38"/>
-      <x:c r="L11" s="38"/>
-      <x:c r="M11" s="38"/>
-      <x:c r="N11" s="38"/>
-      <x:c r="O11" s="38"/>
+      <x:c r="B11" s="38" t="n">
+        <x:v>30000</x:v>
+      </x:c>
+      <x:c r="C11" s="38" t="n">
+        <x:v>20000</x:v>
+      </x:c>
+      <x:c r="D11" s="38" t="n">
+        <x:v>15000</x:v>
+      </x:c>
+      <x:c r="E11" s="38" t="n">
+        <x:v>10000</x:v>
+      </x:c>
+      <x:c r="F11" s="38" t="n">
+        <x:v>8000</x:v>
+      </x:c>
+      <x:c r="G11" s="38" t="n">
+        <x:v>8000</x:v>
+      </x:c>
+      <x:c r="H11" s="38" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="I11" s="38" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="J11" s="38" t="n">
+        <x:v>7000</x:v>
+      </x:c>
+      <x:c r="K11" s="38" t="n">
+        <x:v>10000</x:v>
+      </x:c>
+      <x:c r="L11" s="38" t="n">
+        <x:v>10000</x:v>
+      </x:c>
+      <x:c r="M11" s="38" t="n">
+        <x:v>12000</x:v>
+      </x:c>
+      <x:c r="N11" s="38" t="n">
+        <x:v>12000</x:v>
+      </x:c>
+      <x:c r="O11" s="39" t="n">
+        <x:f>SUM(B11:N11)</x:f>
+        <x:v>152000</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="str">
         <x:v>Cash / EFTPOS sales</x:v>
       </x:c>
-      <x:c r="B12" s="38"/>
-      <x:c r="C12" s="38"/>
-      <x:c r="D12" s="38"/>
-      <x:c r="E12" s="38"/>
-      <x:c r="F12" s="38"/>
-      <x:c r="G12" s="38"/>
-      <x:c r="H12" s="38"/>
-      <x:c r="I12" s="38"/>
-      <x:c r="J12" s="38"/>
-      <x:c r="K12" s="38"/>
-      <x:c r="L12" s="38"/>
-      <x:c r="M12" s="38"/>
-      <x:c r="N12" s="38"/>
-      <x:c r="O12" s="38"/>
+      <x:c r="B12" s="38" t="n">
+        <x:v>18000</x:v>
+      </x:c>
+      <x:c r="C12" s="38" t="n">
+        <x:v>20000</x:v>
+      </x:c>
+      <x:c r="D12" s="38" t="n">
+        <x:v>19000</x:v>
+      </x:c>
+      <x:c r="E12" s="38" t="n">
+        <x:v>18000</x:v>
+      </x:c>
+      <x:c r="F12" s="38" t="n">
+        <x:v>18000</x:v>
+      </x:c>
+      <x:c r="G12" s="38" t="n">
+        <x:v>17000</x:v>
+      </x:c>
+      <x:c r="H12" s="38" t="n">
+        <x:v>17000</x:v>
+      </x:c>
+      <x:c r="I12" s="38" t="n">
+        <x:v>18000</x:v>
+      </x:c>
+      <x:c r="J12" s="38" t="n">
+        <x:v>18000</x:v>
+      </x:c>
+      <x:c r="K12" s="38" t="n">
+        <x:v>19000</x:v>
+      </x:c>
+      <x:c r="L12" s="38" t="n">
+        <x:v>20000</x:v>
+      </x:c>
+      <x:c r="M12" s="38" t="n">
+        <x:v>21000</x:v>
+      </x:c>
+      <x:c r="N12" s="38" t="n">
+        <x:v>22000</x:v>
+      </x:c>
+      <x:c r="O12" s="39" t="n">
+        <x:f>SUM(B12:N12)</x:f>
+        <x:v>245000</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="str">
         <x:v>GST refunds / credits</x:v>
       </x:c>
-      <x:c r="B13" s="38"/>
-      <x:c r="C13" s="38"/>
-      <x:c r="D13" s="38"/>
-      <x:c r="E13" s="38"/>
-      <x:c r="F13" s="38"/>
-      <x:c r="G13" s="38"/>
-      <x:c r="H13" s="38"/>
-      <x:c r="I13" s="38"/>
-      <x:c r="J13" s="38"/>
-      <x:c r="K13" s="38"/>
-      <x:c r="L13" s="38"/>
-      <x:c r="M13" s="38"/>
-      <x:c r="N13" s="38"/>
-      <x:c r="O13" s="38"/>
+      <x:c r="B13" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C13" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D13" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E13" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F13" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G13" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H13" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I13" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J13" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K13" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L13" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M13" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N13" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O13" s="39" t="n">
+        <x:f>SUM(B13:N13)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="str">
         <x:v>Other operating</x:v>
       </x:c>
-      <x:c r="B14" s="38"/>
-      <x:c r="C14" s="38"/>
-      <x:c r="D14" s="38"/>
-      <x:c r="E14" s="38"/>
-      <x:c r="F14" s="38"/>
-      <x:c r="G14" s="38"/>
-      <x:c r="H14" s="38"/>
-      <x:c r="I14" s="38"/>
-      <x:c r="J14" s="38"/>
-      <x:c r="K14" s="38"/>
-      <x:c r="L14" s="38"/>
-      <x:c r="M14" s="38"/>
-      <x:c r="N14" s="38"/>
-      <x:c r="O14" s="38"/>
+      <x:c r="B14" s="38" t="n">
+        <x:v>4000</x:v>
+      </x:c>
+      <x:c r="C14" s="38" t="n">
+        <x:v>4000</x:v>
+      </x:c>
+      <x:c r="D14" s="38" t="n">
+        <x:v>4000</x:v>
+      </x:c>
+      <x:c r="E14" s="38" t="n">
+        <x:v>4000</x:v>
+      </x:c>
+      <x:c r="F14" s="38" t="n">
+        <x:v>4000</x:v>
+      </x:c>
+      <x:c r="G14" s="38" t="n">
+        <x:v>4000</x:v>
+      </x:c>
+      <x:c r="H14" s="38" t="n">
+        <x:v>4000</x:v>
+      </x:c>
+      <x:c r="I14" s="38" t="n">
+        <x:v>4000</x:v>
+      </x:c>
+      <x:c r="J14" s="38" t="n">
+        <x:v>4000</x:v>
+      </x:c>
+      <x:c r="K14" s="38" t="n">
+        <x:v>4000</x:v>
+      </x:c>
+      <x:c r="L14" s="38" t="n">
+        <x:v>4000</x:v>
+      </x:c>
+      <x:c r="M14" s="38" t="n">
+        <x:v>4000</x:v>
+      </x:c>
+      <x:c r="N14" s="38" t="n">
+        <x:v>4000</x:v>
+      </x:c>
+      <x:c r="O14" s="39" t="n">
+        <x:f>SUM(B14:N14)</x:f>
+        <x:v>52000</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" t="str">
         <x:v>Asset sale proceeds</x:v>
       </x:c>
-      <x:c r="B15" s="38"/>
-      <x:c r="C15" s="38"/>
-      <x:c r="D15" s="38"/>
-      <x:c r="E15" s="38"/>
-      <x:c r="F15" s="38"/>
-      <x:c r="G15" s="38"/>
-      <x:c r="H15" s="38"/>
-      <x:c r="I15" s="38"/>
-      <x:c r="J15" s="38"/>
-      <x:c r="K15" s="38"/>
-      <x:c r="L15" s="38"/>
-      <x:c r="M15" s="38"/>
-      <x:c r="N15" s="38"/>
-      <x:c r="O15" s="38"/>
+      <x:c r="B15" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C15" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D15" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E15" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F15" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G15" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H15" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I15" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J15" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K15" s="38" t="n">
+        <x:v>100000</x:v>
+      </x:c>
+      <x:c r="L15" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M15" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N15" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O15" s="39" t="n">
+        <x:f>SUM(B15:N15)</x:f>
+        <x:v>100000</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" t="str">
         <x:v>Equity / owner funding</x:v>
       </x:c>
-      <x:c r="B16" s="38"/>
-      <x:c r="C16" s="38"/>
-      <x:c r="D16" s="38"/>
-      <x:c r="E16" s="38"/>
-      <x:c r="F16" s="38"/>
-      <x:c r="G16" s="38"/>
-      <x:c r="H16" s="38"/>
-      <x:c r="I16" s="38"/>
-      <x:c r="J16" s="38"/>
-      <x:c r="K16" s="38"/>
-      <x:c r="L16" s="38"/>
-      <x:c r="M16" s="38"/>
-      <x:c r="N16" s="38"/>
-      <x:c r="O16" s="38"/>
+      <x:c r="B16" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C16" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D16" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E16" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F16" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G16" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H16" s="38" t="n">
+        <x:v>150000</x:v>
+      </x:c>
+      <x:c r="I16" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J16" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K16" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L16" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M16" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N16" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O16" s="39" t="n">
+        <x:f>SUM(B16:N16)</x:f>
+        <x:v>150000</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" t="str">
         <x:v>Loan proceeds</x:v>
       </x:c>
-      <x:c r="B17" s="38"/>
-      <x:c r="C17" s="38"/>
-      <x:c r="D17" s="38"/>
-      <x:c r="E17" s="38"/>
-      <x:c r="F17" s="38"/>
-      <x:c r="G17" s="38"/>
-      <x:c r="H17" s="38"/>
-      <x:c r="I17" s="38"/>
-      <x:c r="J17" s="38"/>
-      <x:c r="K17" s="38"/>
-      <x:c r="L17" s="38"/>
-      <x:c r="M17" s="38"/>
-      <x:c r="N17" s="38"/>
-      <x:c r="O17" s="38"/>
+      <x:c r="B17" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C17" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D17" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E17" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F17" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G17" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H17" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I17" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J17" s="38" t="n">
+        <x:v>125000</x:v>
+      </x:c>
+      <x:c r="K17" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L17" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M17" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N17" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O17" s="39" t="n">
+        <x:f>SUM(B17:N17)</x:f>
+        <x:v>125000</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" t="str">
         <x:v>Scenario receipt adjustment</x:v>
       </x:c>
-      <x:c r="B18" s="38"/>
-      <x:c r="C18" s="38"/>
-      <x:c r="D18" s="38"/>
-      <x:c r="E18" s="38"/>
-      <x:c r="F18" s="38"/>
-      <x:c r="G18" s="38"/>
-      <x:c r="H18" s="38"/>
-      <x:c r="I18" s="38"/>
-      <x:c r="J18" s="38"/>
-      <x:c r="K18" s="38"/>
-      <x:c r="L18" s="38"/>
-      <x:c r="M18" s="38"/>
-      <x:c r="N18" s="38"/>
-      <x:c r="O18" s="38"/>
+      <x:c r="B18" s="42" t="n">
+        <x:f>IF(B$7="Actual",0,SUM(B10:B12)*(INDEX(Assumptions!$C$15:$C$17,MATCH(Assumptions!$B$12,Assumptions!$B$15:$B$17,0))-1))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C18" s="42" t="n">
+        <x:f>IF(C$7="Actual",0,SUM(C10:C12)*(INDEX(Assumptions!$C$15:$C$17,MATCH(Assumptions!$B$12,Assumptions!$B$15:$B$17,0))-1))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D18" s="42" t="n">
+        <x:f>IF(D$7="Actual",0,SUM(D10:D12)*(INDEX(Assumptions!$C$15:$C$17,MATCH(Assumptions!$B$12,Assumptions!$B$15:$B$17,0))-1))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E18" s="42" t="n">
+        <x:f>IF(E$7="Actual",0,SUM(E10:E12)*(INDEX(Assumptions!$C$15:$C$17,MATCH(Assumptions!$B$12,Assumptions!$B$15:$B$17,0))-1))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F18" s="42" t="n">
+        <x:f>IF(F$7="Actual",0,SUM(F10:F12)*(INDEX(Assumptions!$C$15:$C$17,MATCH(Assumptions!$B$12,Assumptions!$B$15:$B$17,0))-1))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G18" s="42" t="n">
+        <x:f>IF(G$7="Actual",0,SUM(G10:G12)*(INDEX(Assumptions!$C$15:$C$17,MATCH(Assumptions!$B$12,Assumptions!$B$15:$B$17,0))-1))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H18" s="42" t="n">
+        <x:f>IF(H$7="Actual",0,SUM(H10:H12)*(INDEX(Assumptions!$C$15:$C$17,MATCH(Assumptions!$B$12,Assumptions!$B$15:$B$17,0))-1))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I18" s="42" t="n">
+        <x:f>IF(I$7="Actual",0,SUM(I10:I12)*(INDEX(Assumptions!$C$15:$C$17,MATCH(Assumptions!$B$12,Assumptions!$B$15:$B$17,0))-1))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J18" s="42" t="n">
+        <x:f>IF(J$7="Actual",0,SUM(J10:J12)*(INDEX(Assumptions!$C$15:$C$17,MATCH(Assumptions!$B$12,Assumptions!$B$15:$B$17,0))-1))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K18" s="42" t="n">
+        <x:f>IF(K$7="Actual",0,SUM(K10:K12)*(INDEX(Assumptions!$C$15:$C$17,MATCH(Assumptions!$B$12,Assumptions!$B$15:$B$17,0))-1))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L18" s="42" t="n">
+        <x:f>IF(L$7="Actual",0,SUM(L10:L12)*(INDEX(Assumptions!$C$15:$C$17,MATCH(Assumptions!$B$12,Assumptions!$B$15:$B$17,0))-1))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M18" s="42" t="n">
+        <x:f>IF(M$7="Actual",0,SUM(M10:M12)*(INDEX(Assumptions!$C$15:$C$17,MATCH(Assumptions!$B$12,Assumptions!$B$15:$B$17,0))-1))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N18" s="42" t="n">
+        <x:f>IF(N$7="Actual",0,SUM(N10:N12)*(INDEX(Assumptions!$C$15:$C$17,MATCH(Assumptions!$B$12,Assumptions!$B$15:$B$17,0))-1))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O18" s="39" t="n">
+        <x:f>SUM(B18:N18)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="37" t="str">
         <x:v>Total cash receipts</x:v>
       </x:c>
-      <x:c r="B19" s="39"/>
-      <x:c r="C19" s="39"/>
-      <x:c r="D19" s="39"/>
-      <x:c r="E19" s="39"/>
-      <x:c r="F19" s="39"/>
-      <x:c r="G19" s="39"/>
-      <x:c r="H19" s="39"/>
-      <x:c r="I19" s="39"/>
-      <x:c r="J19" s="39"/>
-      <x:c r="K19" s="39"/>
-      <x:c r="L19" s="39"/>
-      <x:c r="M19" s="39"/>
-      <x:c r="N19" s="39"/>
-      <x:c r="O19" s="39"/>
+      <x:c r="B19" s="43" t="n">
+        <x:f>SUM(B10:B18)</x:f>
+        <x:v>170000</x:v>
+      </x:c>
+      <x:c r="C19" s="43" t="n">
+        <x:f>SUM(C10:C18)</x:f>
+        <x:v>169000</x:v>
+      </x:c>
+      <x:c r="D19" s="43" t="n">
+        <x:f>SUM(D10:D18)</x:f>
+        <x:v>158000</x:v>
+      </x:c>
+      <x:c r="E19" s="43" t="n">
+        <x:f>SUM(E10:E18)</x:f>
+        <x:v>147000</x:v>
+      </x:c>
+      <x:c r="F19" s="43" t="n">
+        <x:f>SUM(F10:F18)</x:f>
+        <x:v>140000</x:v>
+      </x:c>
+      <x:c r="G19" s="43" t="n">
+        <x:f>SUM(G10:G18)</x:f>
+        <x:v>141000</x:v>
+      </x:c>
+      <x:c r="H19" s="43" t="n">
+        <x:f>SUM(H10:H18)</x:f>
+        <x:v>281000</x:v>
+      </x:c>
+      <x:c r="I19" s="43" t="n">
+        <x:f>SUM(I10:I18)</x:f>
+        <x:v>135000</x:v>
+      </x:c>
+      <x:c r="J19" s="43" t="n">
+        <x:f>SUM(J10:J18)</x:f>
+        <x:v>264000</x:v>
+      </x:c>
+      <x:c r="K19" s="43" t="n">
+        <x:f>SUM(K10:K18)</x:f>
+        <x:v>249000</x:v>
+      </x:c>
+      <x:c r="L19" s="43" t="n">
+        <x:f>SUM(L10:L18)</x:f>
+        <x:v>154000</x:v>
+      </x:c>
+      <x:c r="M19" s="43" t="n">
+        <x:f>SUM(M10:M18)</x:f>
+        <x:v>162000</x:v>
+      </x:c>
+      <x:c r="N19" s="43" t="n">
+        <x:f>SUM(N10:N18)</x:f>
+        <x:v>168000</x:v>
+      </x:c>
+      <x:c r="O19" s="40" t="n">
+        <x:f>SUM(B19:N19)</x:f>
+        <x:v>2338000</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
-      <x:c r="B20" s="38"/>
-      <x:c r="C20" s="38"/>
-      <x:c r="D20" s="38"/>
-      <x:c r="E20" s="38"/>
-      <x:c r="F20" s="38"/>
-      <x:c r="G20" s="38"/>
-      <x:c r="H20" s="38"/>
-      <x:c r="I20" s="38"/>
-      <x:c r="J20" s="38"/>
-      <x:c r="K20" s="38"/>
-      <x:c r="L20" s="38"/>
-      <x:c r="M20" s="38"/>
-      <x:c r="N20" s="38"/>
-      <x:c r="O20" s="38"/>
+      <x:c r="B20" s="39"/>
+      <x:c r="C20" s="39"/>
+      <x:c r="D20" s="39"/>
+      <x:c r="E20" s="39"/>
+      <x:c r="F20" s="39"/>
+      <x:c r="G20" s="39"/>
+      <x:c r="H20" s="39"/>
+      <x:c r="I20" s="39"/>
+      <x:c r="J20" s="39"/>
+      <x:c r="K20" s="39"/>
+      <x:c r="L20" s="39"/>
+      <x:c r="M20" s="39"/>
+      <x:c r="N20" s="39"/>
+      <x:c r="O20" s="39"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="14" t="str">
         <x:v>CASH PAYMENTS</x:v>
       </x:c>
-      <x:c r="B21" s="40"/>
-      <x:c r="C21" s="40"/>
-      <x:c r="D21" s="40"/>
-      <x:c r="E21" s="40"/>
-      <x:c r="F21" s="40"/>
-      <x:c r="G21" s="40"/>
-      <x:c r="H21" s="40"/>
-      <x:c r="I21" s="40"/>
-      <x:c r="J21" s="40"/>
-      <x:c r="K21" s="40"/>
-      <x:c r="L21" s="40"/>
-      <x:c r="M21" s="40"/>
-      <x:c r="N21" s="40"/>
-      <x:c r="O21" s="40"/>
+      <x:c r="B21" s="41"/>
+      <x:c r="C21" s="41"/>
+      <x:c r="D21" s="41"/>
+      <x:c r="E21" s="41"/>
+      <x:c r="F21" s="41"/>
+      <x:c r="G21" s="41"/>
+      <x:c r="H21" s="41"/>
+      <x:c r="I21" s="41"/>
+      <x:c r="J21" s="41"/>
+      <x:c r="K21" s="41"/>
+      <x:c r="L21" s="41"/>
+      <x:c r="M21" s="41"/>
+      <x:c r="N21" s="41"/>
+      <x:c r="O21" s="41"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" t="str">
         <x:v>Suppliers and inventory</x:v>
       </x:c>
-      <x:c r="B22" s="38"/>
-      <x:c r="C22" s="38"/>
-      <x:c r="D22" s="38"/>
-      <x:c r="E22" s="38"/>
-      <x:c r="F22" s="38"/>
-      <x:c r="G22" s="38"/>
-      <x:c r="H22" s="38"/>
-      <x:c r="I22" s="38"/>
-      <x:c r="J22" s="38"/>
-      <x:c r="K22" s="38"/>
-      <x:c r="L22" s="38"/>
-      <x:c r="M22" s="38"/>
-      <x:c r="N22" s="38"/>
-      <x:c r="O22" s="38"/>
+      <x:c r="B22" s="38" t="n">
+        <x:v>82000</x:v>
+      </x:c>
+      <x:c r="C22" s="38" t="n">
+        <x:v>88000</x:v>
+      </x:c>
+      <x:c r="D22" s="38" t="n">
+        <x:v>90000</x:v>
+      </x:c>
+      <x:c r="E22" s="38" t="n">
+        <x:v>95000</x:v>
+      </x:c>
+      <x:c r="F22" s="38" t="n">
+        <x:v>98000</x:v>
+      </x:c>
+      <x:c r="G22" s="38" t="n">
+        <x:v>100000</x:v>
+      </x:c>
+      <x:c r="H22" s="38" t="n">
+        <x:v>105000</x:v>
+      </x:c>
+      <x:c r="I22" s="38" t="n">
+        <x:v>108000</x:v>
+      </x:c>
+      <x:c r="J22" s="38" t="n">
+        <x:v>110000</x:v>
+      </x:c>
+      <x:c r="K22" s="38" t="n">
+        <x:v>105000</x:v>
+      </x:c>
+      <x:c r="L22" s="38" t="n">
+        <x:v>100000</x:v>
+      </x:c>
+      <x:c r="M22" s="38" t="n">
+        <x:v>95000</x:v>
+      </x:c>
+      <x:c r="N22" s="38" t="n">
+        <x:v>90000</x:v>
+      </x:c>
+      <x:c r="O22" s="39" t="n">
+        <x:f>SUM(B22:N22)</x:f>
+        <x:v>1266000</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" t="str">
         <x:v>Net wages</x:v>
       </x:c>
-      <x:c r="B23" s="38"/>
-      <x:c r="C23" s="38"/>
-      <x:c r="D23" s="38"/>
-      <x:c r="E23" s="38"/>
-      <x:c r="F23" s="38"/>
-      <x:c r="G23" s="38"/>
-      <x:c r="H23" s="38"/>
-      <x:c r="I23" s="38"/>
-      <x:c r="J23" s="38"/>
-      <x:c r="K23" s="38"/>
-      <x:c r="L23" s="38"/>
-      <x:c r="M23" s="38"/>
-      <x:c r="N23" s="38"/>
-      <x:c r="O23" s="38"/>
+      <x:c r="B23" s="38" t="n">
+        <x:v>42000</x:v>
+      </x:c>
+      <x:c r="C23" s="38" t="n">
+        <x:v>42000</x:v>
+      </x:c>
+      <x:c r="D23" s="38" t="n">
+        <x:v>42000</x:v>
+      </x:c>
+      <x:c r="E23" s="38" t="n">
+        <x:v>42000</x:v>
+      </x:c>
+      <x:c r="F23" s="38" t="n">
+        <x:v>42000</x:v>
+      </x:c>
+      <x:c r="G23" s="38" t="n">
+        <x:v>42000</x:v>
+      </x:c>
+      <x:c r="H23" s="38" t="n">
+        <x:v>42000</x:v>
+      </x:c>
+      <x:c r="I23" s="38" t="n">
+        <x:v>42000</x:v>
+      </x:c>
+      <x:c r="J23" s="38" t="n">
+        <x:v>42000</x:v>
+      </x:c>
+      <x:c r="K23" s="38" t="n">
+        <x:v>42000</x:v>
+      </x:c>
+      <x:c r="L23" s="38" t="n">
+        <x:v>42000</x:v>
+      </x:c>
+      <x:c r="M23" s="38" t="n">
+        <x:v>42000</x:v>
+      </x:c>
+      <x:c r="N23" s="38" t="n">
+        <x:v>42000</x:v>
+      </x:c>
+      <x:c r="O23" s="39" t="n">
+        <x:f>SUM(B23:N23)</x:f>
+        <x:v>546000</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" t="str">
         <x:v>PAYG withholding</x:v>
       </x:c>
-      <x:c r="B24" s="38"/>
-      <x:c r="C24" s="38"/>
-      <x:c r="D24" s="38"/>
-      <x:c r="E24" s="38"/>
-      <x:c r="F24" s="38"/>
-      <x:c r="G24" s="38"/>
-      <x:c r="H24" s="38"/>
-      <x:c r="I24" s="38"/>
-      <x:c r="J24" s="38"/>
-      <x:c r="K24" s="38"/>
-      <x:c r="L24" s="38"/>
-      <x:c r="M24" s="38"/>
-      <x:c r="N24" s="38"/>
-      <x:c r="O24" s="38"/>
+      <x:c r="B24" s="38" t="n">
+        <x:v>12000</x:v>
+      </x:c>
+      <x:c r="C24" s="38" t="n">
+        <x:v>12000</x:v>
+      </x:c>
+      <x:c r="D24" s="38" t="n">
+        <x:v>12000</x:v>
+      </x:c>
+      <x:c r="E24" s="38" t="n">
+        <x:v>12000</x:v>
+      </x:c>
+      <x:c r="F24" s="38" t="n">
+        <x:v>12000</x:v>
+      </x:c>
+      <x:c r="G24" s="38" t="n">
+        <x:v>12000</x:v>
+      </x:c>
+      <x:c r="H24" s="38" t="n">
+        <x:v>12000</x:v>
+      </x:c>
+      <x:c r="I24" s="38" t="n">
+        <x:v>12000</x:v>
+      </x:c>
+      <x:c r="J24" s="38" t="n">
+        <x:v>12000</x:v>
+      </x:c>
+      <x:c r="K24" s="38" t="n">
+        <x:v>12000</x:v>
+      </x:c>
+      <x:c r="L24" s="38" t="n">
+        <x:v>12000</x:v>
+      </x:c>
+      <x:c r="M24" s="38" t="n">
+        <x:v>12000</x:v>
+      </x:c>
+      <x:c r="N24" s="38" t="n">
+        <x:v>12000</x:v>
+      </x:c>
+      <x:c r="O24" s="39" t="n">
+        <x:f>SUM(B24:N24)</x:f>
+        <x:v>156000</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" t="str">
         <x:v>Superannuation</x:v>
       </x:c>
-      <x:c r="B25" s="38"/>
-      <x:c r="C25" s="38"/>
-      <x:c r="D25" s="38"/>
-      <x:c r="E25" s="38"/>
-      <x:c r="F25" s="38"/>
-      <x:c r="G25" s="38"/>
-      <x:c r="H25" s="38"/>
-      <x:c r="I25" s="38"/>
-      <x:c r="J25" s="38"/>
-      <x:c r="K25" s="38"/>
-      <x:c r="L25" s="38"/>
-      <x:c r="M25" s="38"/>
-      <x:c r="N25" s="38"/>
-      <x:c r="O25" s="38"/>
+      <x:c r="B25" s="38" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="C25" s="38" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="D25" s="38" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="E25" s="38" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="F25" s="38" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="G25" s="38" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="H25" s="38" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="I25" s="38" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="J25" s="38" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="K25" s="38" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="L25" s="38" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="M25" s="38" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="N25" s="38" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="O25" s="39" t="n">
+        <x:f>SUM(B25:N25)</x:f>
+        <x:v>78000</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" t="str">
         <x:v>Payroll tax / workers compensation</x:v>
       </x:c>
-      <x:c r="B26" s="38"/>
-      <x:c r="C26" s="38"/>
-      <x:c r="D26" s="38"/>
-      <x:c r="E26" s="38"/>
-      <x:c r="F26" s="38"/>
-      <x:c r="G26" s="38"/>
-      <x:c r="H26" s="38"/>
-      <x:c r="I26" s="38"/>
-      <x:c r="J26" s="38"/>
-      <x:c r="K26" s="38"/>
-      <x:c r="L26" s="38"/>
-      <x:c r="M26" s="38"/>
-      <x:c r="N26" s="38"/>
-      <x:c r="O26" s="38"/>
+      <x:c r="B26" s="38" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="C26" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D26" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E26" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F26" s="38" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="G26" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H26" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I26" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J26" s="38" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="K26" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L26" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M26" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N26" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O26" s="39" t="n">
+        <x:f>SUM(B26:N26)</x:f>
+        <x:v>15000</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" t="str">
         <x:v>Rent</x:v>
       </x:c>
-      <x:c r="B27" s="38"/>
-      <x:c r="C27" s="38"/>
-      <x:c r="D27" s="38"/>
-      <x:c r="E27" s="38"/>
-      <x:c r="F27" s="38"/>
-      <x:c r="G27" s="38"/>
-      <x:c r="H27" s="38"/>
-      <x:c r="I27" s="38"/>
-      <x:c r="J27" s="38"/>
-      <x:c r="K27" s="38"/>
-      <x:c r="L27" s="38"/>
-      <x:c r="M27" s="38"/>
-      <x:c r="N27" s="38"/>
-      <x:c r="O27" s="38"/>
+      <x:c r="B27" s="38" t="n">
+        <x:v>25000</x:v>
+      </x:c>
+      <x:c r="C27" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D27" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E27" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F27" s="38" t="n">
+        <x:v>25000</x:v>
+      </x:c>
+      <x:c r="G27" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H27" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I27" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J27" s="38" t="n">
+        <x:v>25000</x:v>
+      </x:c>
+      <x:c r="K27" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L27" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M27" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N27" s="38" t="n">
+        <x:v>25000</x:v>
+      </x:c>
+      <x:c r="O27" s="39" t="n">
+        <x:f>SUM(B27:N27)</x:f>
+        <x:v>100000</x:v>
+      </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" t="str">
         <x:v>Utilities</x:v>
       </x:c>
-      <x:c r="B28" s="38"/>
-      <x:c r="C28" s="38"/>
-      <x:c r="D28" s="38"/>
-      <x:c r="E28" s="38"/>
-      <x:c r="F28" s="38"/>
-      <x:c r="G28" s="38"/>
-      <x:c r="H28" s="38"/>
-      <x:c r="I28" s="38"/>
-      <x:c r="J28" s="38"/>
-      <x:c r="K28" s="38"/>
-      <x:c r="L28" s="38"/>
-      <x:c r="M28" s="38"/>
-      <x:c r="N28" s="38"/>
-      <x:c r="O28" s="38"/>
+      <x:c r="B28" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C28" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D28" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E28" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F28" s="38" t="n">
+        <x:v>4000</x:v>
+      </x:c>
+      <x:c r="G28" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H28" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I28" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J28" s="38" t="n">
+        <x:v>4000</x:v>
+      </x:c>
+      <x:c r="K28" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L28" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M28" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N28" s="38" t="n">
+        <x:v>4000</x:v>
+      </x:c>
+      <x:c r="O28" s="39" t="n">
+        <x:f>SUM(B28:N28)</x:f>
+        <x:v>12000</x:v>
+      </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" t="str">
         <x:v>Insurance</x:v>
       </x:c>
-      <x:c r="B29" s="38"/>
-      <x:c r="C29" s="38"/>
-      <x:c r="D29" s="38"/>
-      <x:c r="E29" s="38"/>
-      <x:c r="F29" s="38"/>
-      <x:c r="G29" s="38"/>
-      <x:c r="H29" s="38"/>
-      <x:c r="I29" s="38"/>
-      <x:c r="J29" s="38"/>
-      <x:c r="K29" s="38"/>
-      <x:c r="L29" s="38"/>
-      <x:c r="M29" s="38"/>
-      <x:c r="N29" s="38"/>
-      <x:c r="O29" s="38"/>
+      <x:c r="B29" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C29" s="38" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="D29" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E29" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F29" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G29" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H29" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I29" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J29" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K29" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L29" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M29" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N29" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O29" s="39" t="n">
+        <x:f>SUM(B29:N29)</x:f>
+        <x:v>6000</x:v>
+      </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" t="str">
         <x:v>Software and subscriptions</x:v>
       </x:c>
-      <x:c r="B30" s="38"/>
-      <x:c r="C30" s="38"/>
-      <x:c r="D30" s="38"/>
-      <x:c r="E30" s="38"/>
-      <x:c r="F30" s="38"/>
-      <x:c r="G30" s="38"/>
-      <x:c r="H30" s="38"/>
-      <x:c r="I30" s="38"/>
-      <x:c r="J30" s="38"/>
-      <x:c r="K30" s="38"/>
-      <x:c r="L30" s="38"/>
-      <x:c r="M30" s="38"/>
-      <x:c r="N30" s="38"/>
-      <x:c r="O30" s="38"/>
+      <x:c r="B30" s="38" t="n">
+        <x:v>3000</x:v>
+      </x:c>
+      <x:c r="C30" s="38" t="n">
+        <x:v>3000</x:v>
+      </x:c>
+      <x:c r="D30" s="38" t="n">
+        <x:v>3000</x:v>
+      </x:c>
+      <x:c r="E30" s="38" t="n">
+        <x:v>3000</x:v>
+      </x:c>
+      <x:c r="F30" s="38" t="n">
+        <x:v>3000</x:v>
+      </x:c>
+      <x:c r="G30" s="38" t="n">
+        <x:v>3000</x:v>
+      </x:c>
+      <x:c r="H30" s="38" t="n">
+        <x:v>3000</x:v>
+      </x:c>
+      <x:c r="I30" s="38" t="n">
+        <x:v>3000</x:v>
+      </x:c>
+      <x:c r="J30" s="38" t="n">
+        <x:v>3000</x:v>
+      </x:c>
+      <x:c r="K30" s="38" t="n">
+        <x:v>3000</x:v>
+      </x:c>
+      <x:c r="L30" s="38" t="n">
+        <x:v>3000</x:v>
+      </x:c>
+      <x:c r="M30" s="38" t="n">
+        <x:v>3000</x:v>
+      </x:c>
+      <x:c r="N30" s="38" t="n">
+        <x:v>3000</x:v>
+      </x:c>
+      <x:c r="O30" s="39" t="n">
+        <x:f>SUM(B30:N30)</x:f>
+        <x:v>39000</x:v>
+      </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" t="str">
         <x:v>Marketing</x:v>
       </x:c>
-      <x:c r="B31" s="38"/>
-      <x:c r="C31" s="38"/>
-      <x:c r="D31" s="38"/>
-      <x:c r="E31" s="38"/>
-      <x:c r="F31" s="38"/>
-      <x:c r="G31" s="38"/>
-      <x:c r="H31" s="38"/>
-      <x:c r="I31" s="38"/>
-      <x:c r="J31" s="38"/>
-      <x:c r="K31" s="38"/>
-      <x:c r="L31" s="38"/>
-      <x:c r="M31" s="38"/>
-      <x:c r="N31" s="38"/>
-      <x:c r="O31" s="38"/>
+      <x:c r="B31" s="38" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="C31" s="38" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="D31" s="38" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="E31" s="38" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="F31" s="38" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="G31" s="38" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="H31" s="38" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="I31" s="38" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="J31" s="38" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="K31" s="38" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="L31" s="38" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="M31" s="38" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="N31" s="38" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="O31" s="39" t="n">
+        <x:f>SUM(B31:N31)</x:f>
+        <x:v>78000</x:v>
+      </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" t="str">
         <x:v>Professional services</x:v>
       </x:c>
-      <x:c r="B32" s="38"/>
-      <x:c r="C32" s="38"/>
-      <x:c r="D32" s="38"/>
-      <x:c r="E32" s="38"/>
-      <x:c r="F32" s="38"/>
-      <x:c r="G32" s="38"/>
-      <x:c r="H32" s="38"/>
-      <x:c r="I32" s="38"/>
-      <x:c r="J32" s="38"/>
-      <x:c r="K32" s="38"/>
-      <x:c r="L32" s="38"/>
-      <x:c r="M32" s="38"/>
-      <x:c r="N32" s="38"/>
-      <x:c r="O32" s="38"/>
+      <x:c r="B32" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C32" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D32" s="38" t="n">
+        <x:v>8000</x:v>
+      </x:c>
+      <x:c r="E32" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F32" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G32" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H32" s="38" t="n">
+        <x:v>8000</x:v>
+      </x:c>
+      <x:c r="I32" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J32" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K32" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L32" s="38" t="n">
+        <x:v>8000</x:v>
+      </x:c>
+      <x:c r="M32" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N32" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O32" s="39" t="n">
+        <x:f>SUM(B32:N32)</x:f>
+        <x:v>24000</x:v>
+      </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" t="str">
         <x:v>Freight, vehicles and travel</x:v>
       </x:c>
-      <x:c r="B33" s="38"/>
-      <x:c r="C33" s="38"/>
-      <x:c r="D33" s="38"/>
-      <x:c r="E33" s="38"/>
-      <x:c r="F33" s="38"/>
-      <x:c r="G33" s="38"/>
-      <x:c r="H33" s="38"/>
-      <x:c r="I33" s="38"/>
-      <x:c r="J33" s="38"/>
-      <x:c r="K33" s="38"/>
-      <x:c r="L33" s="38"/>
-      <x:c r="M33" s="38"/>
-      <x:c r="N33" s="38"/>
-      <x:c r="O33" s="38"/>
+      <x:c r="B33" s="38" t="n">
+        <x:v>10000</x:v>
+      </x:c>
+      <x:c r="C33" s="38" t="n">
+        <x:v>10000</x:v>
+      </x:c>
+      <x:c r="D33" s="38" t="n">
+        <x:v>10000</x:v>
+      </x:c>
+      <x:c r="E33" s="38" t="n">
+        <x:v>10000</x:v>
+      </x:c>
+      <x:c r="F33" s="38" t="n">
+        <x:v>10000</x:v>
+      </x:c>
+      <x:c r="G33" s="38" t="n">
+        <x:v>10000</x:v>
+      </x:c>
+      <x:c r="H33" s="38" t="n">
+        <x:v>10000</x:v>
+      </x:c>
+      <x:c r="I33" s="38" t="n">
+        <x:v>10000</x:v>
+      </x:c>
+      <x:c r="J33" s="38" t="n">
+        <x:v>10000</x:v>
+      </x:c>
+      <x:c r="K33" s="38" t="n">
+        <x:v>10000</x:v>
+      </x:c>
+      <x:c r="L33" s="38" t="n">
+        <x:v>10000</x:v>
+      </x:c>
+      <x:c r="M33" s="38" t="n">
+        <x:v>10000</x:v>
+      </x:c>
+      <x:c r="N33" s="38" t="n">
+        <x:v>10000</x:v>
+      </x:c>
+      <x:c r="O33" s="39" t="n">
+        <x:f>SUM(B33:N33)</x:f>
+        <x:v>130000</x:v>
+      </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" t="str">
         <x:v>GST / BAS payments</x:v>
       </x:c>
-      <x:c r="B34" s="38"/>
-      <x:c r="C34" s="38"/>
-      <x:c r="D34" s="38"/>
-      <x:c r="E34" s="38"/>
-      <x:c r="F34" s="38"/>
-      <x:c r="G34" s="38"/>
-      <x:c r="H34" s="38"/>
-      <x:c r="I34" s="38"/>
-      <x:c r="J34" s="38"/>
-      <x:c r="K34" s="38"/>
-      <x:c r="L34" s="38"/>
-      <x:c r="M34" s="38"/>
-      <x:c r="N34" s="38"/>
-      <x:c r="O34" s="38"/>
+      <x:c r="B34" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C34" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D34" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E34" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F34" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G34" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H34" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I34" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J34" s="38" t="n">
+        <x:v>45000</x:v>
+      </x:c>
+      <x:c r="K34" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L34" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M34" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N34" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O34" s="39" t="n">
+        <x:f>SUM(B34:N34)</x:f>
+        <x:v>45000</x:v>
+      </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" t="str">
         <x:v>PAYG income tax instalments</x:v>
       </x:c>
-      <x:c r="B35" s="38"/>
-      <x:c r="C35" s="38"/>
-      <x:c r="D35" s="38"/>
-      <x:c r="E35" s="38"/>
-      <x:c r="F35" s="38"/>
-      <x:c r="G35" s="38"/>
-      <x:c r="H35" s="38"/>
-      <x:c r="I35" s="38"/>
-      <x:c r="J35" s="38"/>
-      <x:c r="K35" s="38"/>
-      <x:c r="L35" s="38"/>
-      <x:c r="M35" s="38"/>
-      <x:c r="N35" s="38"/>
-      <x:c r="O35" s="38"/>
+      <x:c r="B35" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C35" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D35" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E35" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F35" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G35" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H35" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I35" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J35" s="38" t="n">
+        <x:v>18000</x:v>
+      </x:c>
+      <x:c r="K35" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L35" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M35" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N35" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O35" s="39" t="n">
+        <x:f>SUM(B35:N35)</x:f>
+        <x:v>18000</x:v>
+      </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" t="str">
         <x:v>FBT / other tax</x:v>
       </x:c>
-      <x:c r="B36" s="38"/>
-      <x:c r="C36" s="38"/>
-      <x:c r="D36" s="38"/>
-      <x:c r="E36" s="38"/>
-      <x:c r="F36" s="38"/>
-      <x:c r="G36" s="38"/>
-      <x:c r="H36" s="38"/>
-      <x:c r="I36" s="38"/>
-      <x:c r="J36" s="38"/>
-      <x:c r="K36" s="38"/>
-      <x:c r="L36" s="38"/>
-      <x:c r="M36" s="38"/>
-      <x:c r="N36" s="38"/>
-      <x:c r="O36" s="38"/>
+      <x:c r="B36" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C36" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D36" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E36" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F36" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G36" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H36" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I36" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J36" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K36" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L36" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M36" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N36" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O36" s="39" t="n">
+        <x:f>SUM(B36:N36)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" t="str">
         <x:v>Interest and bank fees</x:v>
       </x:c>
-      <x:c r="B37" s="38"/>
-      <x:c r="C37" s="38"/>
-      <x:c r="D37" s="38"/>
-      <x:c r="E37" s="38"/>
-      <x:c r="F37" s="38"/>
-      <x:c r="G37" s="38"/>
-      <x:c r="H37" s="38"/>
-      <x:c r="I37" s="38"/>
-      <x:c r="J37" s="38"/>
-      <x:c r="K37" s="38"/>
-      <x:c r="L37" s="38"/>
-      <x:c r="M37" s="38"/>
-      <x:c r="N37" s="38"/>
-      <x:c r="O37" s="38"/>
+      <x:c r="B37" s="38" t="n">
+        <x:v>4000</x:v>
+      </x:c>
+      <x:c r="C37" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D37" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E37" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F37" s="38" t="n">
+        <x:v>4000</x:v>
+      </x:c>
+      <x:c r="G37" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H37" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I37" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J37" s="38" t="n">
+        <x:v>4000</x:v>
+      </x:c>
+      <x:c r="K37" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L37" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M37" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N37" s="38" t="n">
+        <x:v>4000</x:v>
+      </x:c>
+      <x:c r="O37" s="39" t="n">
+        <x:f>SUM(B37:N37)</x:f>
+        <x:v>16000</x:v>
+      </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" t="str">
         <x:v>Loan principal</x:v>
       </x:c>
-      <x:c r="B38" s="38"/>
-      <x:c r="C38" s="38"/>
-      <x:c r="D38" s="38"/>
-      <x:c r="E38" s="38"/>
-      <x:c r="F38" s="38"/>
-      <x:c r="G38" s="38"/>
-      <x:c r="H38" s="38"/>
-      <x:c r="I38" s="38"/>
-      <x:c r="J38" s="38"/>
-      <x:c r="K38" s="38"/>
-      <x:c r="L38" s="38"/>
-      <x:c r="M38" s="38"/>
-      <x:c r="N38" s="38"/>
-      <x:c r="O38" s="38"/>
+      <x:c r="B38" s="38" t="n">
+        <x:v>12000</x:v>
+      </x:c>
+      <x:c r="C38" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D38" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E38" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F38" s="38" t="n">
+        <x:v>12000</x:v>
+      </x:c>
+      <x:c r="G38" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H38" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I38" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J38" s="38" t="n">
+        <x:v>12000</x:v>
+      </x:c>
+      <x:c r="K38" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L38" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M38" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N38" s="38" t="n">
+        <x:v>12000</x:v>
+      </x:c>
+      <x:c r="O38" s="39" t="n">
+        <x:f>SUM(B38:N38)</x:f>
+        <x:v>48000</x:v>
+      </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" t="str">
         <x:v>Capital expenditure</x:v>
       </x:c>
-      <x:c r="B39" s="38"/>
-      <x:c r="C39" s="38"/>
-      <x:c r="D39" s="38"/>
-      <x:c r="E39" s="38"/>
-      <x:c r="F39" s="38"/>
-      <x:c r="G39" s="38"/>
-      <x:c r="H39" s="38"/>
-      <x:c r="I39" s="38"/>
-      <x:c r="J39" s="38"/>
-      <x:c r="K39" s="38"/>
-      <x:c r="L39" s="38"/>
-      <x:c r="M39" s="38"/>
-      <x:c r="N39" s="38"/>
-      <x:c r="O39" s="38"/>
+      <x:c r="B39" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C39" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D39" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E39" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F39" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G39" s="38" t="n">
+        <x:v>25000</x:v>
+      </x:c>
+      <x:c r="H39" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I39" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J39" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K39" s="38" t="n">
+        <x:v>40000</x:v>
+      </x:c>
+      <x:c r="L39" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M39" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N39" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O39" s="39" t="n">
+        <x:f>SUM(B39:N39)</x:f>
+        <x:v>65000</x:v>
+      </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" t="str">
         <x:v>Dividends / distributions</x:v>
       </x:c>
-      <x:c r="B40" s="38"/>
-      <x:c r="C40" s="38"/>
-      <x:c r="D40" s="38"/>
-      <x:c r="E40" s="38"/>
-      <x:c r="F40" s="38"/>
-      <x:c r="G40" s="38"/>
-      <x:c r="H40" s="38"/>
-      <x:c r="I40" s="38"/>
-      <x:c r="J40" s="38"/>
-      <x:c r="K40" s="38"/>
-      <x:c r="L40" s="38"/>
-      <x:c r="M40" s="38"/>
-      <x:c r="N40" s="38"/>
-      <x:c r="O40" s="38"/>
+      <x:c r="B40" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C40" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D40" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E40" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F40" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G40" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H40" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I40" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J40" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K40" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L40" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M40" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N40" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O40" s="39" t="n">
+        <x:f>SUM(B40:N40)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" t="str">
         <x:v>Other operating</x:v>
       </x:c>
-      <x:c r="B41" s="38"/>
-      <x:c r="C41" s="38"/>
-      <x:c r="D41" s="38"/>
-      <x:c r="E41" s="38"/>
-      <x:c r="F41" s="38"/>
-      <x:c r="G41" s="38"/>
-      <x:c r="H41" s="38"/>
-      <x:c r="I41" s="38"/>
-      <x:c r="J41" s="38"/>
-      <x:c r="K41" s="38"/>
-      <x:c r="L41" s="38"/>
-      <x:c r="M41" s="38"/>
-      <x:c r="N41" s="38"/>
-      <x:c r="O41" s="38"/>
+      <x:c r="B41" s="38" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="C41" s="38" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="D41" s="38" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="E41" s="38" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="F41" s="38" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="G41" s="38" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="H41" s="38" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="I41" s="38" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="J41" s="38" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="K41" s="38" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="L41" s="38" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="M41" s="38" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="N41" s="38" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="O41" s="39" t="n">
+        <x:f>SUM(B41:N41)</x:f>
+        <x:v>65000</x:v>
+      </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" t="str">
         <x:v>Scenario payment adjustment</x:v>
       </x:c>
-      <x:c r="B42" s="38"/>
-      <x:c r="C42" s="38"/>
-      <x:c r="D42" s="38"/>
-      <x:c r="E42" s="38"/>
-      <x:c r="F42" s="38"/>
-      <x:c r="G42" s="38"/>
-      <x:c r="H42" s="38"/>
-      <x:c r="I42" s="38"/>
-      <x:c r="J42" s="38"/>
-      <x:c r="K42" s="38"/>
-      <x:c r="L42" s="38"/>
-      <x:c r="M42" s="38"/>
-      <x:c r="N42" s="38"/>
-      <x:c r="O42" s="38"/>
+      <x:c r="B42" s="42" t="n">
+        <x:f>IF(B$7="Actual",0,SUM(B22,B31,B33,B41)*(INDEX(Assumptions!$D$15:$D$17,MATCH(Assumptions!$B$12,Assumptions!$B$15:$B$17,0))-1))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C42" s="42" t="n">
+        <x:f>IF(C$7="Actual",0,SUM(C22,C31,C33,C41)*(INDEX(Assumptions!$D$15:$D$17,MATCH(Assumptions!$B$12,Assumptions!$B$15:$B$17,0))-1))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D42" s="42" t="n">
+        <x:f>IF(D$7="Actual",0,SUM(D22,D31,D33,D41)*(INDEX(Assumptions!$D$15:$D$17,MATCH(Assumptions!$B$12,Assumptions!$B$15:$B$17,0))-1))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E42" s="42" t="n">
+        <x:f>IF(E$7="Actual",0,SUM(E22,E31,E33,E41)*(INDEX(Assumptions!$D$15:$D$17,MATCH(Assumptions!$B$12,Assumptions!$B$15:$B$17,0))-1))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F42" s="42" t="n">
+        <x:f>IF(F$7="Actual",0,SUM(F22,F31,F33,F41)*(INDEX(Assumptions!$D$15:$D$17,MATCH(Assumptions!$B$12,Assumptions!$B$15:$B$17,0))-1))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G42" s="42" t="n">
+        <x:f>IF(G$7="Actual",0,SUM(G22,G31,G33,G41)*(INDEX(Assumptions!$D$15:$D$17,MATCH(Assumptions!$B$12,Assumptions!$B$15:$B$17,0))-1))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H42" s="42" t="n">
+        <x:f>IF(H$7="Actual",0,SUM(H22,H31,H33,H41)*(INDEX(Assumptions!$D$15:$D$17,MATCH(Assumptions!$B$12,Assumptions!$B$15:$B$17,0))-1))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I42" s="42" t="n">
+        <x:f>IF(I$7="Actual",0,SUM(I22,I31,I33,I41)*(INDEX(Assumptions!$D$15:$D$17,MATCH(Assumptions!$B$12,Assumptions!$B$15:$B$17,0))-1))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J42" s="42" t="n">
+        <x:f>IF(J$7="Actual",0,SUM(J22,J31,J33,J41)*(INDEX(Assumptions!$D$15:$D$17,MATCH(Assumptions!$B$12,Assumptions!$B$15:$B$17,0))-1))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K42" s="42" t="n">
+        <x:f>IF(K$7="Actual",0,SUM(K22,K31,K33,K41)*(INDEX(Assumptions!$D$15:$D$17,MATCH(Assumptions!$B$12,Assumptions!$B$15:$B$17,0))-1))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L42" s="42" t="n">
+        <x:f>IF(L$7="Actual",0,SUM(L22,L31,L33,L41)*(INDEX(Assumptions!$D$15:$D$17,MATCH(Assumptions!$B$12,Assumptions!$B$15:$B$17,0))-1))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M42" s="42" t="n">
+        <x:f>IF(M$7="Actual",0,SUM(M22,M31,M33,M41)*(INDEX(Assumptions!$D$15:$D$17,MATCH(Assumptions!$B$12,Assumptions!$B$15:$B$17,0))-1))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N42" s="42" t="n">
+        <x:f>IF(N$7="Actual",0,SUM(N22,N31,N33,N41)*(INDEX(Assumptions!$D$15:$D$17,MATCH(Assumptions!$B$12,Assumptions!$B$15:$B$17,0))-1))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O42" s="39" t="n">
+        <x:f>SUM(B42:N42)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="37" t="str">
         <x:v>Total cash payments</x:v>
       </x:c>
-      <x:c r="B43" s="39"/>
-      <x:c r="C43" s="39"/>
-      <x:c r="D43" s="39"/>
-      <x:c r="E43" s="39"/>
-      <x:c r="F43" s="39"/>
-      <x:c r="G43" s="39"/>
-      <x:c r="H43" s="39"/>
-      <x:c r="I43" s="39"/>
-      <x:c r="J43" s="39"/>
-      <x:c r="K43" s="39"/>
-      <x:c r="L43" s="39"/>
-      <x:c r="M43" s="39"/>
-      <x:c r="N43" s="39"/>
-      <x:c r="O43" s="39"/>
+      <x:c r="B43" s="43" t="n">
+        <x:f>SUM(B22:B42)</x:f>
+        <x:v>212000</x:v>
+      </x:c>
+      <x:c r="C43" s="43" t="n">
+        <x:f>SUM(C22:C42)</x:f>
+        <x:v>178000</x:v>
+      </x:c>
+      <x:c r="D43" s="43" t="n">
+        <x:f>SUM(D22:D42)</x:f>
+        <x:v>182000</x:v>
+      </x:c>
+      <x:c r="E43" s="43" t="n">
+        <x:f>SUM(E22:E42)</x:f>
+        <x:v>179000</x:v>
+      </x:c>
+      <x:c r="F43" s="43" t="n">
+        <x:f>SUM(F22:F42)</x:f>
+        <x:v>232000</x:v>
+      </x:c>
+      <x:c r="G43" s="43" t="n">
+        <x:f>SUM(G22:G42)</x:f>
+        <x:v>209000</x:v>
+      </x:c>
+      <x:c r="H43" s="43" t="n">
+        <x:f>SUM(H22:H42)</x:f>
+        <x:v>197000</x:v>
+      </x:c>
+      <x:c r="I43" s="43" t="n">
+        <x:f>SUM(I22:I42)</x:f>
+        <x:v>192000</x:v>
+      </x:c>
+      <x:c r="J43" s="43" t="n">
+        <x:f>SUM(J22:J42)</x:f>
+        <x:v>307000</x:v>
+      </x:c>
+      <x:c r="K43" s="43" t="n">
+        <x:f>SUM(K22:K42)</x:f>
+        <x:v>229000</x:v>
+      </x:c>
+      <x:c r="L43" s="43" t="n">
+        <x:f>SUM(L22:L42)</x:f>
+        <x:v>192000</x:v>
+      </x:c>
+      <x:c r="M43" s="43" t="n">
+        <x:f>SUM(M22:M42)</x:f>
+        <x:v>179000</x:v>
+      </x:c>
+      <x:c r="N43" s="43" t="n">
+        <x:f>SUM(N22:N42)</x:f>
+        <x:v>219000</x:v>
+      </x:c>
+      <x:c r="O43" s="40" t="n">
+        <x:f>SUM(B43:N43)</x:f>
+        <x:v>2707000</x:v>
+      </x:c>
     </x:row>
     <x:row r="44">
-      <x:c r="B44" s="38"/>
-      <x:c r="C44" s="38"/>
-      <x:c r="D44" s="38"/>
-      <x:c r="E44" s="38"/>
-      <x:c r="F44" s="38"/>
-      <x:c r="G44" s="38"/>
-      <x:c r="H44" s="38"/>
-      <x:c r="I44" s="38"/>
-      <x:c r="J44" s="38"/>
-      <x:c r="K44" s="38"/>
-      <x:c r="L44" s="38"/>
-      <x:c r="M44" s="38"/>
-      <x:c r="N44" s="38"/>
-      <x:c r="O44" s="38"/>
+      <x:c r="B44" s="39"/>
+      <x:c r="C44" s="39"/>
+      <x:c r="D44" s="39"/>
+      <x:c r="E44" s="39"/>
+      <x:c r="F44" s="39"/>
+      <x:c r="G44" s="39"/>
+      <x:c r="H44" s="39"/>
+      <x:c r="I44" s="39"/>
+      <x:c r="J44" s="39"/>
+      <x:c r="K44" s="39"/>
+      <x:c r="L44" s="39"/>
+      <x:c r="M44" s="39"/>
+      <x:c r="N44" s="39"/>
+      <x:c r="O44" s="39"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="14" t="str">
         <x:v>CASH POSITION</x:v>
       </x:c>
-      <x:c r="B45" s="40"/>
-      <x:c r="C45" s="40"/>
-      <x:c r="D45" s="40"/>
-      <x:c r="E45" s="40"/>
-      <x:c r="F45" s="40"/>
-      <x:c r="G45" s="40"/>
-      <x:c r="H45" s="40"/>
-      <x:c r="I45" s="40"/>
-      <x:c r="J45" s="40"/>
-      <x:c r="K45" s="40"/>
-      <x:c r="L45" s="40"/>
-      <x:c r="M45" s="40"/>
-      <x:c r="N45" s="40"/>
-      <x:c r="O45" s="40"/>
+      <x:c r="B45" s="41"/>
+      <x:c r="C45" s="41"/>
+      <x:c r="D45" s="41"/>
+      <x:c r="E45" s="41"/>
+      <x:c r="F45" s="41"/>
+      <x:c r="G45" s="41"/>
+      <x:c r="H45" s="41"/>
+      <x:c r="I45" s="41"/>
+      <x:c r="J45" s="41"/>
+      <x:c r="K45" s="41"/>
+      <x:c r="L45" s="41"/>
+      <x:c r="M45" s="41"/>
+      <x:c r="N45" s="41"/>
+      <x:c r="O45" s="41"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" t="str">
         <x:v>Opening cash balance</x:v>
       </x:c>
-      <x:c r="B46" s="38"/>
-      <x:c r="C46" s="38"/>
-      <x:c r="D46" s="38"/>
-      <x:c r="E46" s="38"/>
-      <x:c r="F46" s="38"/>
-      <x:c r="G46" s="38"/>
-      <x:c r="H46" s="38"/>
-      <x:c r="I46" s="38"/>
-      <x:c r="J46" s="38"/>
-      <x:c r="K46" s="38"/>
-      <x:c r="L46" s="38"/>
-      <x:c r="M46" s="38"/>
-      <x:c r="N46" s="38"/>
-      <x:c r="O46" s="38"/>
+      <x:c r="B46" s="44" t="n">
+        <x:f>'Assumptions'!$B$10</x:f>
+        <x:v>400000</x:v>
+      </x:c>
+      <x:c r="C46" s="44" t="n">
+        <x:f>B48</x:f>
+        <x:v>358000</x:v>
+      </x:c>
+      <x:c r="D46" s="44" t="n">
+        <x:f>C48</x:f>
+        <x:v>349000</x:v>
+      </x:c>
+      <x:c r="E46" s="44" t="n">
+        <x:f>D48</x:f>
+        <x:v>325000</x:v>
+      </x:c>
+      <x:c r="F46" s="44" t="n">
+        <x:f>E48</x:f>
+        <x:v>293000</x:v>
+      </x:c>
+      <x:c r="G46" s="44" t="n">
+        <x:f>F48</x:f>
+        <x:v>201000</x:v>
+      </x:c>
+      <x:c r="H46" s="44" t="n">
+        <x:f>G48</x:f>
+        <x:v>133000</x:v>
+      </x:c>
+      <x:c r="I46" s="44" t="n">
+        <x:f>H48</x:f>
+        <x:v>217000</x:v>
+      </x:c>
+      <x:c r="J46" s="44" t="n">
+        <x:f>I48</x:f>
+        <x:v>160000</x:v>
+      </x:c>
+      <x:c r="K46" s="44" t="n">
+        <x:f>J48</x:f>
+        <x:v>117000</x:v>
+      </x:c>
+      <x:c r="L46" s="44" t="n">
+        <x:f>K48</x:f>
+        <x:v>137000</x:v>
+      </x:c>
+      <x:c r="M46" s="44" t="n">
+        <x:f>L48</x:f>
+        <x:v>99000</x:v>
+      </x:c>
+      <x:c r="N46" s="44" t="n">
+        <x:f>M48</x:f>
+        <x:v>82000</x:v>
+      </x:c>
+      <x:c r="O46" s="39" t="n">
+        <x:f>N46</x:f>
+        <x:v>82000</x:v>
+      </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" t="str">
         <x:v>Net cash movement</x:v>
       </x:c>
-      <x:c r="B47" s="38"/>
-      <x:c r="C47" s="38"/>
-      <x:c r="D47" s="38"/>
-      <x:c r="E47" s="38"/>
-      <x:c r="F47" s="38"/>
-      <x:c r="G47" s="38"/>
-      <x:c r="H47" s="38"/>
-      <x:c r="I47" s="38"/>
-      <x:c r="J47" s="38"/>
-      <x:c r="K47" s="38"/>
-      <x:c r="L47" s="38"/>
-      <x:c r="M47" s="38"/>
-      <x:c r="N47" s="38"/>
-      <x:c r="O47" s="38"/>
+      <x:c r="B47" s="42" t="n">
+        <x:f>B19-B43</x:f>
+        <x:v>-42000</x:v>
+      </x:c>
+      <x:c r="C47" s="42" t="n">
+        <x:f>C19-C43</x:f>
+        <x:v>-9000</x:v>
+      </x:c>
+      <x:c r="D47" s="42" t="n">
+        <x:f>D19-D43</x:f>
+        <x:v>-24000</x:v>
+      </x:c>
+      <x:c r="E47" s="42" t="n">
+        <x:f>E19-E43</x:f>
+        <x:v>-32000</x:v>
+      </x:c>
+      <x:c r="F47" s="42" t="n">
+        <x:f>F19-F43</x:f>
+        <x:v>-92000</x:v>
+      </x:c>
+      <x:c r="G47" s="42" t="n">
+        <x:f>G19-G43</x:f>
+        <x:v>-68000</x:v>
+      </x:c>
+      <x:c r="H47" s="42" t="n">
+        <x:f>H19-H43</x:f>
+        <x:v>84000</x:v>
+      </x:c>
+      <x:c r="I47" s="42" t="n">
+        <x:f>I19-I43</x:f>
+        <x:v>-57000</x:v>
+      </x:c>
+      <x:c r="J47" s="42" t="n">
+        <x:f>J19-J43</x:f>
+        <x:v>-43000</x:v>
+      </x:c>
+      <x:c r="K47" s="42" t="n">
+        <x:f>K19-K43</x:f>
+        <x:v>20000</x:v>
+      </x:c>
+      <x:c r="L47" s="42" t="n">
+        <x:f>L19-L43</x:f>
+        <x:v>-38000</x:v>
+      </x:c>
+      <x:c r="M47" s="42" t="n">
+        <x:f>M19-M43</x:f>
+        <x:v>-17000</x:v>
+      </x:c>
+      <x:c r="N47" s="42" t="n">
+        <x:f>N19-N43</x:f>
+        <x:v>-51000</x:v>
+      </x:c>
+      <x:c r="O47" s="39" t="n">
+        <x:f>N47</x:f>
+        <x:v>-51000</x:v>
+      </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="37" t="str">
         <x:v>Closing cash balance</x:v>
       </x:c>
-      <x:c r="B48" s="39"/>
-      <x:c r="C48" s="39"/>
-      <x:c r="D48" s="39"/>
-      <x:c r="E48" s="39"/>
-      <x:c r="F48" s="39"/>
-      <x:c r="G48" s="39"/>
-      <x:c r="H48" s="39"/>
-      <x:c r="I48" s="39"/>
-      <x:c r="J48" s="39"/>
-      <x:c r="K48" s="39"/>
-      <x:c r="L48" s="39"/>
-      <x:c r="M48" s="39"/>
-      <x:c r="N48" s="39"/>
-      <x:c r="O48" s="39"/>
+      <x:c r="B48" s="43" t="n">
+        <x:f>B46+B47</x:f>
+        <x:v>358000</x:v>
+      </x:c>
+      <x:c r="C48" s="43" t="n">
+        <x:f>C46+C47</x:f>
+        <x:v>349000</x:v>
+      </x:c>
+      <x:c r="D48" s="43" t="n">
+        <x:f>D46+D47</x:f>
+        <x:v>325000</x:v>
+      </x:c>
+      <x:c r="E48" s="43" t="n">
+        <x:f>E46+E47</x:f>
+        <x:v>293000</x:v>
+      </x:c>
+      <x:c r="F48" s="43" t="n">
+        <x:f>F46+F47</x:f>
+        <x:v>201000</x:v>
+      </x:c>
+      <x:c r="G48" s="43" t="n">
+        <x:f>G46+G47</x:f>
+        <x:v>133000</x:v>
+      </x:c>
+      <x:c r="H48" s="43" t="n">
+        <x:f>H46+H47</x:f>
+        <x:v>217000</x:v>
+      </x:c>
+      <x:c r="I48" s="43" t="n">
+        <x:f>I46+I47</x:f>
+        <x:v>160000</x:v>
+      </x:c>
+      <x:c r="J48" s="43" t="n">
+        <x:f>J46+J47</x:f>
+        <x:v>117000</x:v>
+      </x:c>
+      <x:c r="K48" s="43" t="n">
+        <x:f>K46+K47</x:f>
+        <x:v>137000</x:v>
+      </x:c>
+      <x:c r="L48" s="43" t="n">
+        <x:f>L46+L47</x:f>
+        <x:v>99000</x:v>
+      </x:c>
+      <x:c r="M48" s="43" t="n">
+        <x:f>M46+M47</x:f>
+        <x:v>82000</x:v>
+      </x:c>
+      <x:c r="N48" s="43" t="n">
+        <x:f>N46+N47</x:f>
+        <x:v>31000</x:v>
+      </x:c>
+      <x:c r="O48" s="40" t="n">
+        <x:f>N48</x:f>
+        <x:v>31000</x:v>
+      </x:c>
     </x:row>
     <x:row r="49">
       <x:c r="A49" t="str">
         <x:v>Minimum cash buffer</x:v>
       </x:c>
-      <x:c r="B49" s="38"/>
-      <x:c r="C49" s="38"/>
-      <x:c r="D49" s="38"/>
-      <x:c r="E49" s="38"/>
-      <x:c r="F49" s="38"/>
-      <x:c r="G49" s="38"/>
-      <x:c r="H49" s="38"/>
-      <x:c r="I49" s="38"/>
-      <x:c r="J49" s="38"/>
-      <x:c r="K49" s="38"/>
-      <x:c r="L49" s="38"/>
-      <x:c r="M49" s="38"/>
-      <x:c r="N49" s="38"/>
-      <x:c r="O49" s="38"/>
+      <x:c r="B49" s="44" t="n">
+        <x:f>'Assumptions'!$B$11</x:f>
+        <x:v>100000</x:v>
+      </x:c>
+      <x:c r="C49" s="44" t="n">
+        <x:f>'Assumptions'!$B$11</x:f>
+        <x:v>100000</x:v>
+      </x:c>
+      <x:c r="D49" s="44" t="n">
+        <x:f>'Assumptions'!$B$11</x:f>
+        <x:v>100000</x:v>
+      </x:c>
+      <x:c r="E49" s="44" t="n">
+        <x:f>'Assumptions'!$B$11</x:f>
+        <x:v>100000</x:v>
+      </x:c>
+      <x:c r="F49" s="44" t="n">
+        <x:f>'Assumptions'!$B$11</x:f>
+        <x:v>100000</x:v>
+      </x:c>
+      <x:c r="G49" s="44" t="n">
+        <x:f>'Assumptions'!$B$11</x:f>
+        <x:v>100000</x:v>
+      </x:c>
+      <x:c r="H49" s="44" t="n">
+        <x:f>'Assumptions'!$B$11</x:f>
+        <x:v>100000</x:v>
+      </x:c>
+      <x:c r="I49" s="44" t="n">
+        <x:f>'Assumptions'!$B$11</x:f>
+        <x:v>100000</x:v>
+      </x:c>
+      <x:c r="J49" s="44" t="n">
+        <x:f>'Assumptions'!$B$11</x:f>
+        <x:v>100000</x:v>
+      </x:c>
+      <x:c r="K49" s="44" t="n">
+        <x:f>'Assumptions'!$B$11</x:f>
+        <x:v>100000</x:v>
+      </x:c>
+      <x:c r="L49" s="44" t="n">
+        <x:f>'Assumptions'!$B$11</x:f>
+        <x:v>100000</x:v>
+      </x:c>
+      <x:c r="M49" s="44" t="n">
+        <x:f>'Assumptions'!$B$11</x:f>
+        <x:v>100000</x:v>
+      </x:c>
+      <x:c r="N49" s="44" t="n">
+        <x:f>'Assumptions'!$B$11</x:f>
+        <x:v>100000</x:v>
+      </x:c>
+      <x:c r="O49" s="39" t="n">
+        <x:f>N49</x:f>
+        <x:v>100000</x:v>
+      </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="37" t="str">
         <x:v>Headroom / (gap)</x:v>
       </x:c>
-      <x:c r="B50" s="39"/>
-      <x:c r="C50" s="39"/>
-      <x:c r="D50" s="39"/>
-      <x:c r="E50" s="39"/>
-      <x:c r="F50" s="39"/>
-      <x:c r="G50" s="39"/>
-      <x:c r="H50" s="39"/>
-      <x:c r="I50" s="39"/>
-      <x:c r="J50" s="39"/>
-      <x:c r="K50" s="39"/>
-      <x:c r="L50" s="39"/>
-      <x:c r="M50" s="39"/>
-      <x:c r="N50" s="39"/>
-      <x:c r="O50" s="39"/>
+      <x:c r="B50" s="43" t="n">
+        <x:f>B48-B49</x:f>
+        <x:v>258000</x:v>
+      </x:c>
+      <x:c r="C50" s="43" t="n">
+        <x:f>C48-C49</x:f>
+        <x:v>249000</x:v>
+      </x:c>
+      <x:c r="D50" s="43" t="n">
+        <x:f>D48-D49</x:f>
+        <x:v>225000</x:v>
+      </x:c>
+      <x:c r="E50" s="43" t="n">
+        <x:f>E48-E49</x:f>
+        <x:v>193000</x:v>
+      </x:c>
+      <x:c r="F50" s="43" t="n">
+        <x:f>F48-F49</x:f>
+        <x:v>101000</x:v>
+      </x:c>
+      <x:c r="G50" s="43" t="n">
+        <x:f>G48-G49</x:f>
+        <x:v>33000</x:v>
+      </x:c>
+      <x:c r="H50" s="43" t="n">
+        <x:f>H48-H49</x:f>
+        <x:v>117000</x:v>
+      </x:c>
+      <x:c r="I50" s="43" t="n">
+        <x:f>I48-I49</x:f>
+        <x:v>60000</x:v>
+      </x:c>
+      <x:c r="J50" s="43" t="n">
+        <x:f>J48-J49</x:f>
+        <x:v>17000</x:v>
+      </x:c>
+      <x:c r="K50" s="43" t="n">
+        <x:f>K48-K49</x:f>
+        <x:v>37000</x:v>
+      </x:c>
+      <x:c r="L50" s="43" t="n">
+        <x:f>L48-L49</x:f>
+        <x:v>-1000</x:v>
+      </x:c>
+      <x:c r="M50" s="43" t="n">
+        <x:f>M48-M49</x:f>
+        <x:v>-18000</x:v>
+      </x:c>
+      <x:c r="N50" s="43" t="n">
+        <x:f>N48-N49</x:f>
+        <x:v>-69000</x:v>
+      </x:c>
+      <x:c r="O50" s="40" t="n">
+        <x:f>N50</x:f>
+        <x:v>-69000</x:v>
+      </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" t="str">
         <x:v>Liquidity status</x:v>
+      </x:c>
+      <x:c r="B51" s="17" t="str">
+        <x:f>IF(B48&lt;B49,"BELOW BUFFER",IF(B48&lt;=B49*1.25,"WATCH","OK"))</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="C51" s="17" t="str">
+        <x:f>IF(C48&lt;C49,"BELOW BUFFER",IF(C48&lt;=C49*1.25,"WATCH","OK"))</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="D51" s="17" t="str">
+        <x:f>IF(D48&lt;D49,"BELOW BUFFER",IF(D48&lt;=D49*1.25,"WATCH","OK"))</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="E51" s="17" t="str">
+        <x:f>IF(E48&lt;E49,"BELOW BUFFER",IF(E48&lt;=E49*1.25,"WATCH","OK"))</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="F51" s="17" t="str">
+        <x:f>IF(F48&lt;F49,"BELOW BUFFER",IF(F48&lt;=F49*1.25,"WATCH","OK"))</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G51" s="17" t="str">
+        <x:f>IF(G48&lt;G49,"BELOW BUFFER",IF(G48&lt;=G49*1.25,"WATCH","OK"))</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="H51" s="17" t="str">
+        <x:f>IF(H48&lt;H49,"BELOW BUFFER",IF(H48&lt;=H49*1.25,"WATCH","OK"))</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I51" s="17" t="str">
+        <x:f>IF(I48&lt;I49,"BELOW BUFFER",IF(I48&lt;=I49*1.25,"WATCH","OK"))</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="J51" s="17" t="str">
+        <x:f>IF(J48&lt;J49,"BELOW BUFFER",IF(J48&lt;=J49*1.25,"WATCH","OK"))</x:f>
+        <x:v>WATCH</x:v>
+      </x:c>
+      <x:c r="K51" s="17" t="str">
+        <x:f>IF(K48&lt;K49,"BELOW BUFFER",IF(K48&lt;=K49*1.25,"WATCH","OK"))</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="L51" s="17" t="str">
+        <x:f>IF(L48&lt;L49,"BELOW BUFFER",IF(L48&lt;=L49*1.25,"WATCH","OK"))</x:f>
+        <x:v>BELOW BUFFER</x:v>
+      </x:c>
+      <x:c r="M51" s="17" t="str">
+        <x:f>IF(M48&lt;M49,"BELOW BUFFER",IF(M48&lt;=M49*1.25,"WATCH","OK"))</x:f>
+        <x:v>BELOW BUFFER</x:v>
+      </x:c>
+      <x:c r="N51" s="17" t="str">
+        <x:f>IF(N48&lt;N49,"BELOW BUFFER",IF(N48&lt;=N49*1.25,"WATCH","OK"))</x:f>
+        <x:v>BELOW BUFFER</x:v>
+      </x:c>
+      <x:c r="O51" t="str">
+        <x:f>N51</x:f>
+        <x:v>BELOW BUFFER</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2038,7 +3446,19 @@
     <x:mergeCell ref="A1:O1"/>
     <x:mergeCell ref="A2:O2"/>
   </x:mergeCells>
+  <x:conditionalFormatting sqref="B51:N51">
+    <x:cfRule type="expression" dxfId="0" priority="1">
+      <x:formula>B51="BELOW BUFFER"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="expression" dxfId="1" priority="2">
+      <x:formula>B51="WATCH"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="expression" dxfId="2" priority="3">
+      <x:formula>B51="OK"</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4c825058279492f"/>
 </x:worksheet>
 </file>
 
@@ -2048,18 +3468,13 @@
   <x:cols>
     <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="17" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="17" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="17" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="17" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="17" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="17" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="17" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="17" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="17" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="16" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="42" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="19" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="19" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="19" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="32" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="28" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -2074,15 +3489,10 @@
       <x:c r="G1" s="4"/>
       <x:c r="H1" s="4"/>
       <x:c r="I1" s="4"/>
-      <x:c r="J1" s="4"/>
-      <x:c r="K1" s="4"/>
-      <x:c r="L1" s="4"/>
-      <x:c r="M1" s="4"/>
-      <x:c r="N1" s="4"/>
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>Forecast accuracy review. Actuals, commentary, owners and actions are added with the forecast engine.</x:v>
+        <x:v>Record actual closing cash, actions and ownership each week. Variance remains blank until an actual is entered.</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -2092,126 +3502,319 @@
       <x:c r="G2" s="8"/>
       <x:c r="H2" s="8"/>
       <x:c r="I2" s="8"/>
-      <x:c r="J2" s="8"/>
-      <x:c r="K2" s="8"/>
-      <x:c r="L2" s="8"/>
-      <x:c r="M2" s="8"/>
-      <x:c r="N2" s="8"/>
     </x:row>
     <x:row r="5" ht="32" customHeight="1">
       <x:c r="A5" s="28" t="str">
         <x:v>Week</x:v>
       </x:c>
       <x:c r="B5" s="28" t="str">
-        <x:v>Week commencing</x:v>
+        <x:v>Week ending</x:v>
       </x:c>
       <x:c r="C5" s="28" t="str">
-        <x:v>Week ending</x:v>
+        <x:v>Forecast closing cash</x:v>
       </x:c>
       <x:c r="D5" s="28" t="str">
-        <x:v>Forecast receipts</x:v>
+        <x:v>Actual closing cash</x:v>
       </x:c>
       <x:c r="E5" s="28" t="str">
-        <x:v>Actual receipts</x:v>
+        <x:v>Variance</x:v>
       </x:c>
       <x:c r="F5" s="28" t="str">
-        <x:v>Receipt variance</x:v>
+        <x:v>Rolling forecast note</x:v>
       </x:c>
       <x:c r="G5" s="28" t="str">
-        <x:v>Forecast payments</x:v>
+        <x:v>Owner</x:v>
       </x:c>
       <x:c r="H5" s="28" t="str">
-        <x:v>Actual payments</x:v>
+        <x:v>Action</x:v>
       </x:c>
       <x:c r="I5" s="28" t="str">
-        <x:v>Payment variance</x:v>
-      </x:c>
-      <x:c r="J5" s="28" t="str">
-        <x:v>Forecast closing cash</x:v>
-      </x:c>
-      <x:c r="K5" s="28" t="str">
-        <x:v>Actual closing cash</x:v>
-      </x:c>
-      <x:c r="L5" s="28" t="str">
-        <x:v>Cash variance</x:v>
-      </x:c>
-      <x:c r="M5" s="28" t="str">
-        <x:v>Owner</x:v>
-      </x:c>
-      <x:c r="N5" s="28" t="str">
-        <x:v>Commentary / action</x:v>
+        <x:v>Status</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="n">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="B6" s="45" t="n">
+        <x:f>'13-Week Forecast'!B$6</x:f>
+        <x:v>46271</x:v>
+      </x:c>
+      <x:c r="C6" s="44" t="n">
+        <x:f>'13-Week Forecast'!B$48</x:f>
+        <x:v>358000</x:v>
+      </x:c>
+      <x:c r="D6" s="38"/>
+      <x:c r="E6" s="42" t="str">
+        <x:f>IF(D6="","",D6-C6)</x:f>
+      </x:c>
+      <x:c r="F6" s="16"/>
+      <x:c r="G6" s="16"/>
+      <x:c r="H6" s="16"/>
+      <x:c r="I6" s="16"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="B7" s="45" t="n">
+        <x:f>'13-Week Forecast'!C$6</x:f>
+        <x:v>46278</x:v>
+      </x:c>
+      <x:c r="C7" s="44" t="n">
+        <x:f>'13-Week Forecast'!C$48</x:f>
+        <x:v>349000</x:v>
+      </x:c>
+      <x:c r="D7" s="38"/>
+      <x:c r="E7" s="42" t="str">
+        <x:f>IF(D7="","",D7-C7)</x:f>
+      </x:c>
+      <x:c r="F7" s="16"/>
+      <x:c r="G7" s="16"/>
+      <x:c r="H7" s="16"/>
+      <x:c r="I7" s="16"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="n">
         <x:v>3</x:v>
       </x:c>
+      <x:c r="B8" s="45" t="n">
+        <x:f>'13-Week Forecast'!D$6</x:f>
+        <x:v>46285</x:v>
+      </x:c>
+      <x:c r="C8" s="44" t="n">
+        <x:f>'13-Week Forecast'!D$48</x:f>
+        <x:v>325000</x:v>
+      </x:c>
+      <x:c r="D8" s="38"/>
+      <x:c r="E8" s="42" t="str">
+        <x:f>IF(D8="","",D8-C8)</x:f>
+      </x:c>
+      <x:c r="F8" s="16"/>
+      <x:c r="G8" s="16"/>
+      <x:c r="H8" s="16"/>
+      <x:c r="I8" s="16"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="n">
         <x:v>4</x:v>
       </x:c>
+      <x:c r="B9" s="45" t="n">
+        <x:f>'13-Week Forecast'!E$6</x:f>
+        <x:v>46292</x:v>
+      </x:c>
+      <x:c r="C9" s="44" t="n">
+        <x:f>'13-Week Forecast'!E$48</x:f>
+        <x:v>293000</x:v>
+      </x:c>
+      <x:c r="D9" s="38"/>
+      <x:c r="E9" s="42" t="str">
+        <x:f>IF(D9="","",D9-C9)</x:f>
+      </x:c>
+      <x:c r="F9" s="16"/>
+      <x:c r="G9" s="16"/>
+      <x:c r="H9" s="16"/>
+      <x:c r="I9" s="16"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="n">
         <x:v>5</x:v>
       </x:c>
+      <x:c r="B10" s="45" t="n">
+        <x:f>'13-Week Forecast'!F$6</x:f>
+        <x:v>46299</x:v>
+      </x:c>
+      <x:c r="C10" s="44" t="n">
+        <x:f>'13-Week Forecast'!F$48</x:f>
+        <x:v>201000</x:v>
+      </x:c>
+      <x:c r="D10" s="38"/>
+      <x:c r="E10" s="42" t="str">
+        <x:f>IF(D10="","",D10-C10)</x:f>
+      </x:c>
+      <x:c r="F10" s="16"/>
+      <x:c r="G10" s="16"/>
+      <x:c r="H10" s="16"/>
+      <x:c r="I10" s="16"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="n">
         <x:v>6</x:v>
       </x:c>
+      <x:c r="B11" s="45" t="n">
+        <x:f>'13-Week Forecast'!G$6</x:f>
+        <x:v>46306</x:v>
+      </x:c>
+      <x:c r="C11" s="44" t="n">
+        <x:f>'13-Week Forecast'!G$48</x:f>
+        <x:v>133000</x:v>
+      </x:c>
+      <x:c r="D11" s="38"/>
+      <x:c r="E11" s="42" t="str">
+        <x:f>IF(D11="","",D11-C11)</x:f>
+      </x:c>
+      <x:c r="F11" s="16"/>
+      <x:c r="G11" s="16"/>
+      <x:c r="H11" s="16"/>
+      <x:c r="I11" s="16"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="n">
         <x:v>7</x:v>
       </x:c>
+      <x:c r="B12" s="45" t="n">
+        <x:f>'13-Week Forecast'!H$6</x:f>
+        <x:v>46313</x:v>
+      </x:c>
+      <x:c r="C12" s="44" t="n">
+        <x:f>'13-Week Forecast'!H$48</x:f>
+        <x:v>217000</x:v>
+      </x:c>
+      <x:c r="D12" s="38"/>
+      <x:c r="E12" s="42" t="str">
+        <x:f>IF(D12="","",D12-C12)</x:f>
+      </x:c>
+      <x:c r="F12" s="16"/>
+      <x:c r="G12" s="16"/>
+      <x:c r="H12" s="16"/>
+      <x:c r="I12" s="16"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="n">
         <x:v>8</x:v>
       </x:c>
+      <x:c r="B13" s="45" t="n">
+        <x:f>'13-Week Forecast'!I$6</x:f>
+        <x:v>46320</x:v>
+      </x:c>
+      <x:c r="C13" s="44" t="n">
+        <x:f>'13-Week Forecast'!I$48</x:f>
+        <x:v>160000</x:v>
+      </x:c>
+      <x:c r="D13" s="38"/>
+      <x:c r="E13" s="42" t="str">
+        <x:f>IF(D13="","",D13-C13)</x:f>
+      </x:c>
+      <x:c r="F13" s="16"/>
+      <x:c r="G13" s="16"/>
+      <x:c r="H13" s="16"/>
+      <x:c r="I13" s="16"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="n">
         <x:v>9</x:v>
       </x:c>
+      <x:c r="B14" s="45" t="n">
+        <x:f>'13-Week Forecast'!J$6</x:f>
+        <x:v>46327</x:v>
+      </x:c>
+      <x:c r="C14" s="44" t="n">
+        <x:f>'13-Week Forecast'!J$48</x:f>
+        <x:v>117000</x:v>
+      </x:c>
+      <x:c r="D14" s="38"/>
+      <x:c r="E14" s="42" t="str">
+        <x:f>IF(D14="","",D14-C14)</x:f>
+      </x:c>
+      <x:c r="F14" s="16"/>
+      <x:c r="G14" s="16"/>
+      <x:c r="H14" s="16"/>
+      <x:c r="I14" s="16"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" t="n">
         <x:v>10</x:v>
       </x:c>
+      <x:c r="B15" s="45" t="n">
+        <x:f>'13-Week Forecast'!K$6</x:f>
+        <x:v>46334</x:v>
+      </x:c>
+      <x:c r="C15" s="44" t="n">
+        <x:f>'13-Week Forecast'!K$48</x:f>
+        <x:v>137000</x:v>
+      </x:c>
+      <x:c r="D15" s="38"/>
+      <x:c r="E15" s="42" t="str">
+        <x:f>IF(D15="","",D15-C15)</x:f>
+      </x:c>
+      <x:c r="F15" s="16"/>
+      <x:c r="G15" s="16"/>
+      <x:c r="H15" s="16"/>
+      <x:c r="I15" s="16"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" t="n">
         <x:v>11</x:v>
       </x:c>
+      <x:c r="B16" s="45" t="n">
+        <x:f>'13-Week Forecast'!L$6</x:f>
+        <x:v>46341</x:v>
+      </x:c>
+      <x:c r="C16" s="44" t="n">
+        <x:f>'13-Week Forecast'!L$48</x:f>
+        <x:v>99000</x:v>
+      </x:c>
+      <x:c r="D16" s="38"/>
+      <x:c r="E16" s="42" t="str">
+        <x:f>IF(D16="","",D16-C16)</x:f>
+      </x:c>
+      <x:c r="F16" s="16"/>
+      <x:c r="G16" s="16"/>
+      <x:c r="H16" s="16"/>
+      <x:c r="I16" s="16"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" t="n">
         <x:v>12</x:v>
       </x:c>
+      <x:c r="B17" s="45" t="n">
+        <x:f>'13-Week Forecast'!M$6</x:f>
+        <x:v>46348</x:v>
+      </x:c>
+      <x:c r="C17" s="44" t="n">
+        <x:f>'13-Week Forecast'!M$48</x:f>
+        <x:v>82000</x:v>
+      </x:c>
+      <x:c r="D17" s="38"/>
+      <x:c r="E17" s="42" t="str">
+        <x:f>IF(D17="","",D17-C17)</x:f>
+      </x:c>
+      <x:c r="F17" s="16"/>
+      <x:c r="G17" s="16"/>
+      <x:c r="H17" s="16"/>
+      <x:c r="I17" s="16"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" t="n">
         <x:v>13</x:v>
       </x:c>
+      <x:c r="B18" s="45" t="n">
+        <x:f>'13-Week Forecast'!N$6</x:f>
+        <x:v>46355</x:v>
+      </x:c>
+      <x:c r="C18" s="44" t="n">
+        <x:f>'13-Week Forecast'!N$48</x:f>
+        <x:v>31000</x:v>
+      </x:c>
+      <x:c r="D18" s="38"/>
+      <x:c r="E18" s="42" t="str">
+        <x:f>IF(D18="","",D18-C18)</x:f>
+      </x:c>
+      <x:c r="F18" s="16"/>
+      <x:c r="G18" s="16"/>
+      <x:c r="H18" s="16"/>
+      <x:c r="I18" s="16"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:N1"/>
-    <x:mergeCell ref="A2:N2"/>
+    <x:mergeCell ref="A1:I1"/>
+    <x:mergeCell ref="A2:I2"/>
   </x:mergeCells>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="I6:I18">
+      <x:formula1>"Open,In progress,Complete"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -2281,16 +3884,16 @@
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="41" t="str">
+      <x:c r="A6" s="47" t="str">
         <x:v>MODEL STATUS: prepared for formula-driven integrity checks</x:v>
       </x:c>
-      <x:c r="B6" s="41"/>
-      <x:c r="C6" s="41"/>
-      <x:c r="D6" s="41"/>
-      <x:c r="E6" s="41"/>
-      <x:c r="F6" s="41"/>
-      <x:c r="G6" s="41"/>
-      <x:c r="H6" s="41"/>
+      <x:c r="B6" s="47"/>
+      <x:c r="C6" s="47"/>
+      <x:c r="D6" s="47"/>
+      <x:c r="E6" s="47"/>
+      <x:c r="F6" s="47"/>
+      <x:c r="G6" s="47"/>
+      <x:c r="H6" s="47"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="14" t="str">
@@ -2313,22 +3916,22 @@
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="43" t="str">
+      <x:c r="A11" s="49" t="str">
         <x:v>Statutory dates and classifications require confirmation for your entity, reporting cycle and agent arrangements.</x:v>
       </x:c>
-      <x:c r="B11" s="43"/>
-      <x:c r="C11" s="43"/>
-      <x:c r="D11" s="43"/>
-      <x:c r="E11" s="43"/>
-      <x:c r="F11" s="43"/>
+      <x:c r="B11" s="49"/>
+      <x:c r="C11" s="49"/>
+      <x:c r="D11" s="49"/>
+      <x:c r="E11" s="49"/>
+      <x:c r="F11" s="49"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="43"/>
-      <x:c r="B12" s="43"/>
-      <x:c r="C12" s="43"/>
-      <x:c r="D12" s="43"/>
-      <x:c r="E12" s="43"/>
-      <x:c r="F12" s="43"/>
+      <x:c r="A12" s="49"/>
+      <x:c r="B12" s="49"/>
+      <x:c r="C12" s="49"/>
+      <x:c r="D12" s="49"/>
+      <x:c r="E12" s="49"/>
+      <x:c r="F12" s="49"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
fix: strengthen cash flow forecast contract
</commit_message>
<xml_diff>
--- a/templates/13-week-cash-flow-forecast.xlsx
+++ b/templates/13-week-cash-flow-forecast.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R163eef40803243ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R36a323b4bd524392"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R55e1d91aef2144cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13-Week Forecast" sheetId="4" r:id="R3a5216492bc244a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Review" sheetId="5" r:id="R6e15a48bc1404b42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks &amp; Sources" sheetId="6" r:id="R40686c5f31a64d21"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R3e53cff34fb3404f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Ra5d9b34592c44d08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R02020629f966456b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13-Week Forecast" sheetId="4" r:id="R9a98a45bf36543f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Review" sheetId="5" r:id="R4948e13d0d524a0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks &amp; Sources" sheetId="6" r:id="R758b2f2e63254719"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="CashFlowScenario">'Assumptions'!$B$12</x:definedName>
@@ -20,10 +20,10 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={E28899D8-E974-D419-CBA0-A3EAED613B76}</x:author>
-    <x:author>tc={17D25D66-7DB0-58F0-CE5E-E2EB2DCDA11F}</x:author>
-    <x:author>tc={6D6F189E-71DD-5AB0-A5B5-8089484B0A68}</x:author>
-    <x:author>tc={E870F557-83E1-4DD3-E5B6-7E48039B894E}</x:author>
+    <x:author>tc={75DE23CE-A935-BFA0-98B0-716B59A88F03}</x:author>
+    <x:author>tc={2E978C1C-A140-5B1A-8A5A-5E0CB2034512}</x:author>
+    <x:author>tc={AB4F57D7-7C83-4B35-BCE8-54405C1832F3}</x:author>
+    <x:author>tc={F00DFA9B-E108-DC3D-4302-EF7DC2B4B9ED}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="B18" authorId="0">
@@ -32,7 +32,7 @@
           <x:t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Scenario receipt adjustment applies the selected scenario only to customer receipts and cash / EFTPOS sales. Week 1 is Actual, so the adjustment is zero.</x:t>
+    Scenario receipt adjustment applies the selected scenario only to current customer receipts, overdue receipts and cash / EFTPOS sales. Week 1 is Actual, so the adjustment is zero.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -335,7 +335,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="User" id="{D4E71844-CD76-4BEE-BAA9-387BBDF1B51C}"/>
+  <xltc:person displayName="User" id="{D45FE37B-BE5A-40E8-9106-C3ABA403F384}"/>
 </xltc:personList>
 </file>
 
@@ -532,16 +532,16 @@
 
 <file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="B18" dT="2026-08-26T13:22:07.159" personId="{D4E71844-CD76-4BEE-BAA9-387BBDF1B51C}" id="{E28899D8-E974-D419-CBA0-A3EAED613B76}">
-    <xltc:text>Scenario receipt adjustment applies the selected scenario only to customer receipts and cash / EFTPOS sales. Week 1 is Actual, so the adjustment is zero.</xltc:text>
+  <xltc:threadedComment ref="B18" dT="2026-08-26T13:28:35.39" personId="{D45FE37B-BE5A-40E8-9106-C3ABA403F384}" id="{75DE23CE-A935-BFA0-98B0-716B59A88F03}">
+    <xltc:text>Scenario receipt adjustment applies the selected scenario only to current customer receipts, overdue receipts and cash / EFTPOS sales. Week 1 is Actual, so the adjustment is zero.</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="B42" dT="2026-08-26T13:22:07.159" personId="{D4E71844-CD76-4BEE-BAA9-387BBDF1B51C}" id="{17D25D66-7DB0-58F0-CE5E-E2EB2DCDA11F}">
+  <xltc:threadedComment ref="B42" dT="2026-08-26T13:28:35.391" personId="{D45FE37B-BE5A-40E8-9106-C3ABA403F384}" id="{2E978C1C-A140-5B1A-8A5A-5E0CB2034512}">
     <xltc:text>Scenario payment adjustment applies the selected scenario only to suppliers, marketing, freight / vehicles / travel and other operating payments. Week 1 is Actual, so the adjustment is zero.</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="B34" dT="2026-08-26T13:22:07.159" personId="{D4E71844-CD76-4BEE-BAA9-387BBDF1B51C}" id="{6D6F189E-71DD-5AB0-A5B5-8089484B0A68}">
+  <xltc:threadedComment ref="B34" dT="2026-08-26T13:28:35.391" personId="{D45FE37B-BE5A-40E8-9106-C3ABA403F384}" id="{AB4F57D7-7C83-4B35-BCE8-54405C1832F3}">
     <xltc:text>GST / BAS cash timing is illustrative. Confirm your entity's reporting cycle, due date and payment arrangement before relying on this forecast.</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="B35" dT="2026-08-26T13:22:07.159" personId="{D4E71844-CD76-4BEE-BAA9-387BBDF1B51C}" id="{E870F557-83E1-4DD3-E5B6-7E48039B894E}">
+  <xltc:threadedComment ref="B35" dT="2026-08-26T13:28:35.391" personId="{D45FE37B-BE5A-40E8-9106-C3ABA403F384}" id="{F00DFA9B-E108-DC3D-4302-EF7DC2B4B9ED}">
     <xltc:text>PAYG income-tax instalment timing and amount are illustrative. Confirm the applicable ATO notice and adviser instructions.</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
@@ -3458,7 +3458,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4c825058279492f"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re5578828a6574f7e"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
fix: strengthen cash flow dashboard contract
</commit_message>
<xml_diff>
--- a/templates/13-week-cash-flow-forecast.xlsx
+++ b/templates/13-week-cash-flow-forecast.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R6365591222b34de4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R63a198b070c74297"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R3c5e1c3bfbe94158"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13-Week Forecast" sheetId="4" r:id="Rbc435d3534754d31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Review" sheetId="5" r:id="Raf7ca443aec049a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks &amp; Sources" sheetId="6" r:id="R6513339d280742ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R5f02dd2468644489"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Ra885b4ee6f8f4aba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R3af6af053bd54b31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13-Week Forecast" sheetId="4" r:id="Rfab8b815b5ca4192"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Review" sheetId="5" r:id="R872022763bea412f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks &amp; Sources" sheetId="6" r:id="R7e8e625aeb7a449f"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="CashFlowScenario">'Assumptions'!$B$12</x:definedName>
@@ -20,10 +20,10 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={98FAA047-B01D-5348-2BF1-D894601FC806}</x:author>
-    <x:author>tc={BE1B932E-612F-4047-F56F-9CDCA82CBB32}</x:author>
-    <x:author>tc={B3C5A793-7724-FDA4-8C59-D102B1FE2C65}</x:author>
-    <x:author>tc={736F7184-3EC3-9C52-7FDB-69574353E070}</x:author>
+    <x:author>tc={9630C31D-6C15-3DCD-6FEC-FFF0920387C0}</x:author>
+    <x:author>tc={78DC6C45-5048-5652-71C1-FFC94265B0A0}</x:author>
+    <x:author>tc={CC57C4BB-274F-5D5B-93F2-2C6F5FC0530F}</x:author>
+    <x:author>tc={B28E83DE-AB9D-F6A0-5F2B-175B1910D78A}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="B18" authorId="0">
@@ -746,6 +746,7 @@
     <c:plotArea>
       <c:barChart>
         <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
         <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="0"/>
@@ -906,7 +907,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ref5028a0a2fe4326"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2c40855584474044"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -936,7 +937,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8ac1622332704bbf"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R41b1b7debcf1437a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -947,7 +948,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="User" id="{40D6A7C4-057F-4C0F-94B0-D08E14A712BD}"/>
+  <xltc:person displayName="User" id="{951688C4-7DF6-4493-9F59-4D169F48BCE3}"/>
 </xltc:personList>
 </file>
 
@@ -1144,16 +1145,16 @@
 
 <file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="B18" dT="2026-08-26T13:42:51.005" personId="{40D6A7C4-057F-4C0F-94B0-D08E14A712BD}" id="{98FAA047-B01D-5348-2BF1-D894601FC806}">
+  <xltc:threadedComment ref="B18" dT="2026-08-26T13:49:48.939" personId="{951688C4-7DF6-4493-9F59-4D169F48BCE3}" id="{9630C31D-6C15-3DCD-6FEC-FFF0920387C0}">
     <xltc:text>Scenario receipt adjustment applies the selected scenario only to current customer receipts, overdue receipts and cash / EFTPOS sales. Week 1 is Actual, so the adjustment is zero.</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="B42" dT="2026-08-26T13:42:51.005" personId="{40D6A7C4-057F-4C0F-94B0-D08E14A712BD}" id="{BE1B932E-612F-4047-F56F-9CDCA82CBB32}">
+  <xltc:threadedComment ref="B42" dT="2026-08-26T13:49:48.939" personId="{951688C4-7DF6-4493-9F59-4D169F48BCE3}" id="{78DC6C45-5048-5652-71C1-FFC94265B0A0}">
     <xltc:text>Scenario payment adjustment applies the selected scenario only to suppliers, marketing, freight / vehicles / travel and other operating payments. Week 1 is Actual, so the adjustment is zero.</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="B34" dT="2026-08-26T13:42:51.005" personId="{40D6A7C4-057F-4C0F-94B0-D08E14A712BD}" id="{B3C5A793-7724-FDA4-8C59-D102B1FE2C65}">
+  <xltc:threadedComment ref="B34" dT="2026-08-26T13:49:48.939" personId="{951688C4-7DF6-4493-9F59-4D169F48BCE3}" id="{CC57C4BB-274F-5D5B-93F2-2C6F5FC0530F}">
     <xltc:text>GST / BAS cash timing is illustrative. Confirm your entity's reporting cycle, due date and payment arrangement before relying on this forecast.</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="B35" dT="2026-08-26T13:42:51.005" personId="{40D6A7C4-057F-4C0F-94B0-D08E14A712BD}" id="{736F7184-3EC3-9C52-7FDB-69574353E070}">
+  <xltc:threadedComment ref="B35" dT="2026-08-26T13:49:48.939" personId="{951688C4-7DF6-4493-9F59-4D169F48BCE3}" id="{B28E83DE-AB9D-F6A0-5F2B-175B1910D78A}">
     <xltc:text>PAYG income-tax instalment timing and amount are illustrative. Confirm the applicable ATO notice and adviser instructions.</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
@@ -2261,7 +2262,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fce3a2c5625401a"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R242e8ccac0354ed6"/>
 </x:worksheet>
 </file>
 
@@ -4777,7 +4778,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3cebc129644548f1"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc4c8ec6ea244832"/>
 </x:worksheet>
 </file>
 
@@ -5543,7 +5544,7 @@
         <x:v>26 August 2026</x:v>
       </x:c>
       <x:c r="E23" s="59" t="str">
-        <x:v>The issued BAS controls. Online lodgement, registered-agent arrangements, holidays and entity circumstances can change the date.</x:v>
+        <x:v>The issued or entity-specific BAS due date controls. Online lodgement, registered-agent arrangements, holidays and entity circumstances can change the date.</x:v>
       </x:c>
       <x:c r="F23" s="59" t="str">
         <x:v>Use issued BAS and user-entered dates.</x:v>

</xml_diff>

<commit_message>
fix: prevent assumptions header clipping
</commit_message>
<xml_diff>
--- a/templates/13-week-cash-flow-forecast.xlsx
+++ b/templates/13-week-cash-flow-forecast.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R5f02dd2468644489"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Ra885b4ee6f8f4aba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R3af6af053bd54b31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13-Week Forecast" sheetId="4" r:id="Rfab8b815b5ca4192"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Review" sheetId="5" r:id="R872022763bea412f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks &amp; Sources" sheetId="6" r:id="R7e8e625aeb7a449f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Rc6463e792faf46f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Ra5bf1840a7a849d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R569615fbea9c4417"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13-Week Forecast" sheetId="4" r:id="R8549e76a58c646a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Review" sheetId="5" r:id="R4b268d1345624768"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks &amp; Sources" sheetId="6" r:id="R7ad570235965495b"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="CashFlowScenario">'Assumptions'!$B$12</x:definedName>
@@ -20,10 +20,10 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={9630C31D-6C15-3DCD-6FEC-FFF0920387C0}</x:author>
-    <x:author>tc={78DC6C45-5048-5652-71C1-FFC94265B0A0}</x:author>
-    <x:author>tc={CC57C4BB-274F-5D5B-93F2-2C6F5FC0530F}</x:author>
-    <x:author>tc={B28E83DE-AB9D-F6A0-5F2B-175B1910D78A}</x:author>
+    <x:author>tc={6150C06D-0457-5C86-C3C0-AE0049FE548F}</x:author>
+    <x:author>tc={10FFFD00-D8ED-6C1E-A4F9-A29DB51051D7}</x:author>
+    <x:author>tc={BDF069F6-163C-548D-0C24-D5CD3190C6B0}</x:author>
+    <x:author>tc={31BA30AE-D302-55C2-C616-5D8A9C3C43C7}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="B18" authorId="0">
@@ -907,7 +907,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2c40855584474044"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0f4d8477e6a94356"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -937,7 +937,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R41b1b7debcf1437a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R496d2c41286a4acb"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -948,7 +948,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="User" id="{951688C4-7DF6-4493-9F59-4D169F48BCE3}"/>
+  <xltc:person displayName="User" id="{1DA5EA16-2278-4414-9D93-50966BD9A7B8}"/>
 </xltc:personList>
 </file>
 
@@ -1145,16 +1145,16 @@
 
 <file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="B18" dT="2026-08-26T13:49:48.939" personId="{951688C4-7DF6-4493-9F59-4D169F48BCE3}" id="{9630C31D-6C15-3DCD-6FEC-FFF0920387C0}">
+  <xltc:threadedComment ref="B18" dT="2026-08-26T14:16:10.492" personId="{1DA5EA16-2278-4414-9D93-50966BD9A7B8}" id="{6150C06D-0457-5C86-C3C0-AE0049FE548F}">
     <xltc:text>Scenario receipt adjustment applies the selected scenario only to current customer receipts, overdue receipts and cash / EFTPOS sales. Week 1 is Actual, so the adjustment is zero.</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="B42" dT="2026-08-26T13:49:48.939" personId="{951688C4-7DF6-4493-9F59-4D169F48BCE3}" id="{78DC6C45-5048-5652-71C1-FFC94265B0A0}">
+  <xltc:threadedComment ref="B42" dT="2026-08-26T14:16:10.492" personId="{1DA5EA16-2278-4414-9D93-50966BD9A7B8}" id="{10FFFD00-D8ED-6C1E-A4F9-A29DB51051D7}">
     <xltc:text>Scenario payment adjustment applies the selected scenario only to suppliers, marketing, freight / vehicles / travel and other operating payments. Week 1 is Actual, so the adjustment is zero.</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="B34" dT="2026-08-26T13:49:48.939" personId="{951688C4-7DF6-4493-9F59-4D169F48BCE3}" id="{CC57C4BB-274F-5D5B-93F2-2C6F5FC0530F}">
+  <xltc:threadedComment ref="B34" dT="2026-08-26T14:16:10.492" personId="{1DA5EA16-2278-4414-9D93-50966BD9A7B8}" id="{BDF069F6-163C-548D-0C24-D5CD3190C6B0}">
     <xltc:text>GST / BAS cash timing is illustrative. Confirm your entity's reporting cycle, due date and payment arrangement before relying on this forecast.</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="B35" dT="2026-08-26T13:49:48.939" personId="{951688C4-7DF6-4493-9F59-4D169F48BCE3}" id="{B28E83DE-AB9D-F6A0-5F2B-175B1910D78A}">
+  <xltc:threadedComment ref="B35" dT="2026-08-26T14:16:10.492" personId="{1DA5EA16-2278-4414-9D93-50966BD9A7B8}" id="{31BA30AE-D302-55C2-C616-5D8A9C3C43C7}">
     <xltc:text>PAYG income-tax instalment timing and amount are illustrative. Confirm the applicable ATO notice and adviser instructions.</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
@@ -2262,7 +2262,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R242e8ccac0354ed6"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64b1483b845a4cf9"/>
 </x:worksheet>
 </file>
 
@@ -2273,7 +2273,7 @@
     <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="48" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
   </x:cols>
@@ -4778,7 +4778,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc4c8ec6ea244832"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03cec6b27bdd4e44"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
fix: close cash flow verification gaps
</commit_message>
<xml_diff>
--- a/templates/13-week-cash-flow-forecast.xlsx
+++ b/templates/13-week-cash-flow-forecast.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Re205b0f6e9714c7a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R626c134bb200410d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="Rbf718284d1eb44d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13-Week Forecast" sheetId="4" r:id="Rd31ed432d30342c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Review" sheetId="5" r:id="R3eeb8bd2f859490e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks &amp; Sources" sheetId="6" r:id="Rb45787a5c4bf4fa8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R0aced715edfa470c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R6bce5e00559047c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="Ree0ec750fe2a4a35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13-Week Forecast" sheetId="4" r:id="R4367c1a2476249bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Review" sheetId="5" r:id="Rcc34dbc9481e43f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks &amp; Sources" sheetId="6" r:id="Rcd66832414704385"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="CashFlowScenario">'Assumptions'!$B$12</x:definedName>
@@ -20,10 +20,10 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={69516E80-B86B-5485-9815-F1D6B4F4A1A6}</x:author>
-    <x:author>tc={218FD7FC-83FB-9E7C-4BEE-9EA002F59077}</x:author>
-    <x:author>tc={8121AE60-30EE-0278-CF63-EC455EEFB906}</x:author>
-    <x:author>tc={E5346B2C-4D96-0537-D519-CF76582AE940}</x:author>
+    <x:author>tc={7258B81E-8D3B-6CE0-FD35-E742545C19CE}</x:author>
+    <x:author>tc={4B221FE6-B027-FA2F-C6F9-1EE0264D0247}</x:author>
+    <x:author>tc={93A359DE-A609-AD0C-0920-C48C5D95F28D}</x:author>
+    <x:author>tc={57C27267-3D72-7DA2-C807-8DC3D2110E18}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="B18" authorId="0">
@@ -1009,7 +1009,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4cb8a91667d04fd2"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra179688aa6fa4295"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1039,7 +1039,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6e1022fa26714d0b"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5cdac9e588944447"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1050,7 +1050,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="User" id="{347AE2E5-ED2C-41D2-9AA6-47721B3B961B}"/>
+  <xltc:person displayName="User" id="{1F1C2A46-2A2C-47F8-83D6-8D7E7B6B5F2A}"/>
 </xltc:personList>
 </file>
 
@@ -1247,16 +1247,16 @@
 
 <file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="B18" dT="2026-08-26T14:43:45.786" personId="{347AE2E5-ED2C-41D2-9AA6-47721B3B961B}" id="{69516E80-B86B-5485-9815-F1D6B4F4A1A6}">
+  <xltc:threadedComment ref="B18" dT="2026-08-26T14:58:01.498" personId="{1F1C2A46-2A2C-47F8-83D6-8D7E7B6B5F2A}" id="{7258B81E-8D3B-6CE0-FD35-E742545C19CE}">
     <xltc:text>Scenario receipt adjustment applies the selected scenario only to current customer receipts, overdue receipts and cash / EFTPOS sales. Week 1 is Actual, so the adjustment is zero.</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="B42" dT="2026-08-26T14:43:45.786" personId="{347AE2E5-ED2C-41D2-9AA6-47721B3B961B}" id="{218FD7FC-83FB-9E7C-4BEE-9EA002F59077}">
+  <xltc:threadedComment ref="B42" dT="2026-08-26T14:58:01.498" personId="{1F1C2A46-2A2C-47F8-83D6-8D7E7B6B5F2A}" id="{4B221FE6-B027-FA2F-C6F9-1EE0264D0247}">
     <xltc:text>Scenario payment adjustment applies the selected scenario only to suppliers, marketing, freight / vehicles / travel and other operating payments. Week 1 is Actual, so the adjustment is zero.</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="B34" dT="2026-08-26T14:43:45.786" personId="{347AE2E5-ED2C-41D2-9AA6-47721B3B961B}" id="{8121AE60-30EE-0278-CF63-EC455EEFB906}">
+  <xltc:threadedComment ref="B34" dT="2026-08-26T14:58:01.498" personId="{1F1C2A46-2A2C-47F8-83D6-8D7E7B6B5F2A}" id="{93A359DE-A609-AD0C-0920-C48C5D95F28D}">
     <xltc:text>GST / BAS cash timing is illustrative. Confirm your entity's reporting cycle, due date and payment arrangement before relying on this forecast.</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="B35" dT="2026-08-26T14:43:45.786" personId="{347AE2E5-ED2C-41D2-9AA6-47721B3B961B}" id="{E5346B2C-4D96-0537-D519-CF76582AE940}">
+  <xltc:threadedComment ref="B35" dT="2026-08-26T14:58:01.498" personId="{1F1C2A46-2A2C-47F8-83D6-8D7E7B6B5F2A}" id="{57C27267-3D72-7DA2-C807-8DC3D2110E18}">
     <xltc:text>PAYG income-tax instalment timing and amount are illustrative. Confirm the applicable ATO notice and adviser instructions.</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
@@ -2373,7 +2373,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d7a0950c2c04bb1"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd417ac4cdfee42a8"/>
 </x:worksheet>
 </file>
 
@@ -4889,7 +4889,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39f6cd30e8d746ad"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R993fc6886ca7468d"/>
 </x:worksheet>
 </file>
 
@@ -5901,7 +5901,7 @@
         <x:v>Formula-error count</x:v>
       </x:c>
       <x:c r="B16" s="50" t="n">
-        <x:f>SUMPRODUCT(--ISERROR('Assumptions'!$B$5:$D$17))+SUMPRODUCT(--ISERROR('13-Week Forecast'!$B$5:$O$51))+SUMPRODUCT(--ISERROR('Weekly Review'!$A$5:$N$18))+SUMPRODUCT(--ISERROR('Dashboard'!$A$6:$J$24))</x:f>
+        <x:f>SUMPRODUCT(--ISERROR('Assumptions'!$B$5:$D$17))+SUMPRODUCT(--ISERROR('13-Week Forecast'!$B$5:$O$51))+SUMPRODUCT(--ISERROR('Weekly Review'!$A$5:$N$18))+SUMPRODUCT(--ISERROR('Dashboard'!$A$6:$J$24))+SUMPRODUCT(--ISERROR('Dashboard'!$P$4:$R$34))</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C16" s="50" t="n">

</xml_diff>

<commit_message>
Use Aptos throughout cash-flow template
</commit_message>
<xml_diff>
--- a/templates/13-week-cash-flow-forecast.xlsx
+++ b/templates/13-week-cash-flow-forecast.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R4d44442af84142eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R6fecb1a629ca4327"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R91bf2385bb964313"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13-Week Forecast" sheetId="4" r:id="Rd2cfaf2133b94566"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Review" sheetId="5" r:id="R906f3a99a7484e34"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks &amp; Sources" sheetId="6" r:id="Ra98aead422a1451b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Rb46856e0cd274e1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Rf51f7fc7c7ac4703"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R09e2d2a5fbda4d95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13-Week Forecast" sheetId="4" r:id="Rdff7daedb25c448a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Review" sheetId="5" r:id="Rda7868aea9f24915"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks &amp; Sources" sheetId="6" r:id="R3349cf15cb6b4e86"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="CashFlowScenario">'Assumptions'!$B$12</x:definedName>
@@ -20,10 +20,10 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={911808D7-7490-7273-81DF-52B18E6A0026}</x:author>
-    <x:author>tc={3CE89642-A655-41DD-1FA6-DE53C860A290}</x:author>
-    <x:author>tc={39CDC10E-89CD-355E-05E8-C2A4AA6F0BB9}</x:author>
-    <x:author>tc={1C0A15C3-71DD-065B-05EE-065A18D44E19}</x:author>
+    <x:author>tc={84D266F6-19BA-B47D-5D1E-5574E3244C5E}</x:author>
+    <x:author>tc={EB8A6292-8349-BCED-0B6A-820E09C1CE7C}</x:author>
+    <x:author>tc={F2C7C3A4-FBBA-3A12-EE58-6838DD9AE503}</x:author>
+    <x:author>tc={72F653C9-5555-6279-61F6-5B5AB1783FF8}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="B18" authorId="0">
@@ -83,7 +83,7 @@
     <x:numFmt numFmtId="203" formatCode="0"/>
     <x:numFmt numFmtId="204" formatCode="#,##0;[Red](#,##0);-"/>
   </x:numFmts>
-  <x:fonts count="14">
+  <x:fonts count="15">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -97,7 +97,7 @@
       <x:b/>
       <x:sz val="18"/>
       <x:color rgb="FFFFFFFF"/>
-      <x:name val="Aptos Display"/>
+      <x:name val="Aptos"/>
     </x:font>
     <x:font>
       <x:sz val="10"/>
@@ -157,6 +157,10 @@
       <x:b/>
       <x:sz val="12"/>
       <x:color rgb="FF04001F"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
@@ -229,7 +233,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="71">
+  <x:cellXfs count="77">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -347,6 +351,18 @@
       <x:alignment horizontal="center"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1022,7 +1038,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rdb280384cd224945"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8d359760a76540fd"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1052,7 +1068,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R67d1bcb11ae843fc"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R85f1f962974a472b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1063,7 +1079,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="User" id="{4E5C786D-4D85-4AFA-B2CD-21FAF79CB976}"/>
+  <xltc:person displayName="User" id="{602EEDB7-EB17-4906-A8BC-ABFEC588047C}"/>
 </xltc:personList>
 </file>
 
@@ -1260,16 +1276,16 @@
 
 <file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="B18" dT="2026-08-26T16:49:11.841" personId="{4E5C786D-4D85-4AFA-B2CD-21FAF79CB976}" id="{911808D7-7490-7273-81DF-52B18E6A0026}">
+  <xltc:threadedComment ref="B18" dT="2026-08-26T17:04:38.821" personId="{602EEDB7-EB17-4906-A8BC-ABFEC588047C}" id="{84D266F6-19BA-B47D-5D1E-5574E3244C5E}">
     <xltc:text>Scenario receipt adjustment applies the selected scenario only to current customer receipts, overdue receipts and cash / EFTPOS sales. Week 1 is Actual, so the adjustment is zero.</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="B42" dT="2026-08-26T16:49:11.842" personId="{4E5C786D-4D85-4AFA-B2CD-21FAF79CB976}" id="{3CE89642-A655-41DD-1FA6-DE53C860A290}">
+  <xltc:threadedComment ref="B42" dT="2026-08-26T17:04:38.821" personId="{602EEDB7-EB17-4906-A8BC-ABFEC588047C}" id="{EB8A6292-8349-BCED-0B6A-820E09C1CE7C}">
     <xltc:text>Scenario payment adjustment applies the selected scenario only to suppliers, marketing, freight / vehicles / travel and other operating payments. Week 1 is Actual, so the adjustment is zero.</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="B34" dT="2026-08-26T16:49:11.842" personId="{4E5C786D-4D85-4AFA-B2CD-21FAF79CB976}" id="{39CDC10E-89CD-355E-05E8-C2A4AA6F0BB9}">
+  <xltc:threadedComment ref="B34" dT="2026-08-26T17:04:38.821" personId="{602EEDB7-EB17-4906-A8BC-ABFEC588047C}" id="{F2C7C3A4-FBBA-3A12-EE58-6838DD9AE503}">
     <xltc:text>GST / BAS cash timing is illustrative. Confirm your entity's reporting cycle, due date and payment arrangement before relying on this forecast.</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="B35" dT="2026-08-26T16:49:11.842" personId="{4E5C786D-4D85-4AFA-B2CD-21FAF79CB976}" id="{1C0A15C3-71DD-065B-05EE-065A18D44E19}">
+  <xltc:threadedComment ref="B35" dT="2026-08-26T17:04:38.821" personId="{602EEDB7-EB17-4906-A8BC-ABFEC588047C}" id="{72F653C9-5555-6279-61F6-5B5AB1783FF8}">
     <xltc:text>PAYG income-tax instalment timing and amount are illustrative. Confirm the applicable ATO notice and adviser instructions.</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
@@ -1313,6 +1329,16 @@
       <x:c r="G2" s="8"/>
       <x:c r="H2" s="8"/>
     </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="71"/>
+      <x:c r="B3" s="71"/>
+      <x:c r="C3" s="71"/>
+      <x:c r="D3" s="71"/>
+      <x:c r="E3" s="71"/>
+      <x:c r="F3" s="71"/>
+      <x:c r="G3" s="71"/>
+      <x:c r="H3" s="71"/>
+    </x:row>
     <x:row r="4">
       <x:c r="A4" s="10" t="str">
         <x:v>ILLUSTRATIVE DATA | Replace every blue input with your organisation's current cash-flow assumptions.</x:v>
@@ -1325,13 +1351,24 @@
       <x:c r="G4" s="10"/>
       <x:c r="H4" s="10"/>
     </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="71"/>
+      <x:c r="B5" s="71"/>
+      <x:c r="C5" s="71"/>
+      <x:c r="D5" s="71"/>
+      <x:c r="E5" s="71"/>
+      <x:c r="F5" s="71"/>
+      <x:c r="G5" s="71"/>
+      <x:c r="H5" s="71"/>
+    </x:row>
     <x:row r="6">
-      <x:c r="A6" t="str">
+      <x:c r="A6" s="71" t="str">
         <x:v>Version</x:v>
       </x:c>
-      <x:c r="B6" t="str">
+      <x:c r="B6" s="71" t="str">
         <x:v>Release 1.1</x:v>
       </x:c>
+      <x:c r="C6" s="71"/>
       <x:c r="D6" s="23" t="str">
         <x:v>Workbook sheets</x:v>
       </x:c>
@@ -1341,54 +1378,81 @@
       <x:c r="H6" s="23"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" t="str">
+      <x:c r="A7" s="71" t="str">
         <x:v>Prepared date</x:v>
       </x:c>
-      <x:c r="B7" s="11" t="n">
+      <x:c r="B7" s="72" t="n">
         <x:v>46260</x:v>
       </x:c>
+      <x:c r="C7" s="71"/>
       <x:c r="D7" s="1" t="str">
         <x:v>Dashboard</x:v>
       </x:c>
+      <x:c r="E7" s="71"/>
+      <x:c r="F7" s="71"/>
+      <x:c r="G7" s="71"/>
+      <x:c r="H7" s="71"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" t="str">
+      <x:c r="A8" s="71" t="str">
         <x:v>Currency</x:v>
       </x:c>
-      <x:c r="B8" t="str">
+      <x:c r="B8" s="71" t="str">
         <x:v>AUD</x:v>
       </x:c>
+      <x:c r="C8" s="71"/>
       <x:c r="D8" s="1" t="str">
         <x:v>Assumptions</x:v>
       </x:c>
+      <x:c r="E8" s="71"/>
+      <x:c r="F8" s="71"/>
+      <x:c r="G8" s="71"/>
+      <x:c r="H8" s="71"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" t="str">
+      <x:c r="A9" s="71" t="str">
         <x:v>Units</x:v>
       </x:c>
-      <x:c r="B9" t="str">
+      <x:c r="B9" s="71" t="str">
         <x:v>Whole dollars</x:v>
       </x:c>
+      <x:c r="C9" s="71"/>
       <x:c r="D9" s="1" t="str">
         <x:v>13-Week Forecast</x:v>
       </x:c>
+      <x:c r="E9" s="71"/>
+      <x:c r="F9" s="71"/>
+      <x:c r="G9" s="71"/>
+      <x:c r="H9" s="71"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" t="str">
+      <x:c r="A10" s="71" t="str">
         <x:v>Selected scenario</x:v>
       </x:c>
       <x:c r="B10" s="12" t="str">
         <x:f>'Assumptions'!$B$12</x:f>
         <x:v>Base</x:v>
       </x:c>
+      <x:c r="C10" s="71"/>
       <x:c r="D10" s="1" t="str">
         <x:v>Weekly Review</x:v>
       </x:c>
+      <x:c r="E10" s="71"/>
+      <x:c r="F10" s="71"/>
+      <x:c r="G10" s="71"/>
+      <x:c r="H10" s="71"/>
     </x:row>
     <x:row r="11">
+      <x:c r="A11" s="71"/>
+      <x:c r="B11" s="71"/>
+      <x:c r="C11" s="71"/>
       <x:c r="D11" s="1" t="str">
         <x:v>Checks &amp; Sources</x:v>
       </x:c>
+      <x:c r="E11" s="71"/>
+      <x:c r="F11" s="71"/>
+      <x:c r="G11" s="71"/>
+      <x:c r="H11" s="71"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="14" t="str">
@@ -1403,44 +1467,84 @@
       <x:c r="H12" s="14"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" t="str">
+      <x:c r="A13" s="71" t="str">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B13" s="15" t="str">
+      <x:c r="B13" s="73" t="str">
         <x:v>Update the Assumptions control panel and selected scenario.</x:v>
       </x:c>
+      <x:c r="C13" s="71"/>
+      <x:c r="D13" s="71"/>
+      <x:c r="E13" s="71"/>
+      <x:c r="F13" s="71"/>
+      <x:c r="G13" s="71"/>
+      <x:c r="H13" s="71"/>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" t="str">
+      <x:c r="A14" s="71" t="str">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B14" s="15" t="str">
+      <x:c r="B14" s="73" t="str">
         <x:v>Replace blue cash-receipt and cash-payment inputs with the latest weekly view.</x:v>
       </x:c>
+      <x:c r="C14" s="71"/>
+      <x:c r="D14" s="71"/>
+      <x:c r="E14" s="71"/>
+      <x:c r="F14" s="71"/>
+      <x:c r="G14" s="71"/>
+      <x:c r="H14" s="71"/>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" t="str">
+      <x:c r="A15" s="71" t="str">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B15" s="15" t="str">
+      <x:c r="B15" s="73" t="str">
         <x:v>Review closing cash, headroom and liquidity status in the 13-Week Forecast.</x:v>
       </x:c>
+      <x:c r="C15" s="71"/>
+      <x:c r="D15" s="71"/>
+      <x:c r="E15" s="71"/>
+      <x:c r="F15" s="71"/>
+      <x:c r="G15" s="71"/>
+      <x:c r="H15" s="71"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" t="str">
+      <x:c r="A16" s="71" t="str">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B16" s="15" t="str">
+      <x:c r="B16" s="73" t="str">
         <x:v>Snapshot the original forecast as values, then record actuals and owner commentary in Weekly Review.</x:v>
       </x:c>
+      <x:c r="C16" s="71"/>
+      <x:c r="D16" s="71"/>
+      <x:c r="E16" s="71"/>
+      <x:c r="F16" s="71"/>
+      <x:c r="G16" s="71"/>
+      <x:c r="H16" s="71"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" t="str">
+      <x:c r="A17" s="71" t="str">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B17" s="15" t="str">
+      <x:c r="B17" s="73" t="str">
         <x:v>Resolve any control failure in Checks &amp; Sources before management review.</x:v>
       </x:c>
+      <x:c r="C17" s="71"/>
+      <x:c r="D17" s="71"/>
+      <x:c r="E17" s="71"/>
+      <x:c r="F17" s="71"/>
+      <x:c r="G17" s="71"/>
+      <x:c r="H17" s="71"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="71"/>
+      <x:c r="B18" s="71"/>
+      <x:c r="C18" s="71"/>
+      <x:c r="D18" s="71"/>
+      <x:c r="E18" s="71"/>
+      <x:c r="F18" s="71"/>
+      <x:c r="G18" s="71"/>
+      <x:c r="H18" s="71"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="14" t="str">
@@ -1458,41 +1562,91 @@
       <x:c r="A20" s="16" t="str">
         <x:v>Blue text / lavender fill</x:v>
       </x:c>
-      <x:c r="B20" t="str">
+      <x:c r="B20" s="71" t="str">
         <x:v>Editable user input</x:v>
       </x:c>
+      <x:c r="C20" s="71"/>
+      <x:c r="D20" s="71"/>
+      <x:c r="E20" s="71"/>
+      <x:c r="F20" s="71"/>
+      <x:c r="G20" s="71"/>
+      <x:c r="H20" s="71"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="17" t="str">
         <x:v>Black text</x:v>
       </x:c>
-      <x:c r="B21" t="str">
+      <x:c r="B21" s="71" t="str">
         <x:v>Formula or calculation</x:v>
       </x:c>
+      <x:c r="C21" s="71"/>
+      <x:c r="D21" s="71"/>
+      <x:c r="E21" s="71"/>
+      <x:c r="F21" s="71"/>
+      <x:c r="G21" s="71"/>
+      <x:c r="H21" s="71"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="12" t="str">
         <x:v>Green text</x:v>
       </x:c>
-      <x:c r="B22" t="str">
+      <x:c r="B22" s="71" t="str">
         <x:v>Cross-sheet link</x:v>
       </x:c>
+      <x:c r="C22" s="71"/>
+      <x:c r="D22" s="71"/>
+      <x:c r="E22" s="71"/>
+      <x:c r="F22" s="71"/>
+      <x:c r="G22" s="71"/>
+      <x:c r="H22" s="71"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="19" t="str">
         <x:v>Red text / pale-red fill</x:v>
       </x:c>
-      <x:c r="B23" t="str">
+      <x:c r="B23" s="71" t="str">
         <x:v>Warning or exception</x:v>
       </x:c>
+      <x:c r="C23" s="71"/>
+      <x:c r="D23" s="71"/>
+      <x:c r="E23" s="71"/>
+      <x:c r="F23" s="71"/>
+      <x:c r="G23" s="71"/>
+      <x:c r="H23" s="71"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="21" t="str">
         <x:v>Dark green / pale-green fill</x:v>
       </x:c>
-      <x:c r="B24" t="str">
+      <x:c r="B24" s="71" t="str">
         <x:v>Passing check</x:v>
       </x:c>
+      <x:c r="C24" s="71"/>
+      <x:c r="D24" s="71"/>
+      <x:c r="E24" s="71"/>
+      <x:c r="F24" s="71"/>
+      <x:c r="G24" s="71"/>
+      <x:c r="H24" s="71"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="71"/>
+      <x:c r="B25" s="71"/>
+      <x:c r="C25" s="71"/>
+      <x:c r="D25" s="71"/>
+      <x:c r="E25" s="71"/>
+      <x:c r="F25" s="71"/>
+      <x:c r="G25" s="71"/>
+      <x:c r="H25" s="71"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="71"/>
+      <x:c r="B26" s="71"/>
+      <x:c r="C26" s="71"/>
+      <x:c r="D26" s="71"/>
+      <x:c r="E26" s="71"/>
+      <x:c r="F26" s="71"/>
+      <x:c r="G26" s="71"/>
+      <x:c r="H26" s="71"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="27" t="str">
@@ -1598,6 +1752,27 @@
       <x:c r="R2" s="8"/>
       <x:c r="S2" s="8"/>
     </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="71"/>
+      <x:c r="B3" s="71"/>
+      <x:c r="C3" s="71"/>
+      <x:c r="D3" s="71"/>
+      <x:c r="E3" s="71"/>
+      <x:c r="F3" s="71"/>
+      <x:c r="G3" s="71"/>
+      <x:c r="H3" s="71"/>
+      <x:c r="I3" s="71"/>
+      <x:c r="J3" s="71"/>
+      <x:c r="K3" s="71"/>
+      <x:c r="L3" s="71"/>
+      <x:c r="M3" s="71"/>
+      <x:c r="N3" s="71"/>
+      <x:c r="O3" s="71"/>
+      <x:c r="P3" s="71"/>
+      <x:c r="Q3" s="71"/>
+      <x:c r="R3" s="71"/>
+      <x:c r="S3" s="71"/>
+    </x:row>
     <x:row r="4">
       <x:c r="A4" s="25" t="str">
         <x:v>No cash-flow inputs belong on this sheet. Update Assumptions and the 13-Week Forecast instead.</x:v>
@@ -1625,20 +1800,37 @@
       <x:c r="R4" s="14" t="str">
         <x:v>Minimum buffer</x:v>
       </x:c>
+      <x:c r="S4" s="71"/>
     </x:row>
     <x:row r="5">
-      <x:c r="P5" s="11" t="str">
+      <x:c r="A5" s="71"/>
+      <x:c r="B5" s="71"/>
+      <x:c r="C5" s="71"/>
+      <x:c r="D5" s="71"/>
+      <x:c r="E5" s="71"/>
+      <x:c r="F5" s="71"/>
+      <x:c r="G5" s="71"/>
+      <x:c r="H5" s="71"/>
+      <x:c r="I5" s="71"/>
+      <x:c r="J5" s="71"/>
+      <x:c r="K5" s="71"/>
+      <x:c r="L5" s="71"/>
+      <x:c r="M5" s="71"/>
+      <x:c r="N5" s="71"/>
+      <x:c r="O5" s="71"/>
+      <x:c r="P5" s="72" t="str">
         <x:f>TEXT('13-Week Forecast'!B$6,"dd mmm")</x:f>
         <x:v>06 Sep</x:v>
       </x:c>
-      <x:c r="Q5" s="39" t="n">
+      <x:c r="Q5" s="74" t="n">
         <x:f>'13-Week Forecast'!B$48</x:f>
         <x:v>358000</x:v>
       </x:c>
-      <x:c r="R5" s="39" t="n">
+      <x:c r="R5" s="74" t="n">
         <x:f>'13-Week Forecast'!B$49</x:f>
         <x:v>100000</x:v>
       </x:c>
+      <x:c r="S5" s="71"/>
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
       <x:c r="A6" s="60" t="str">
@@ -1671,18 +1863,24 @@
       <x:c r="J6" s="60" t="str">
         <x:v>LIQUIDITY STATUS</x:v>
       </x:c>
-      <x:c r="P6" s="11" t="str">
+      <x:c r="K6" s="71"/>
+      <x:c r="L6" s="71"/>
+      <x:c r="M6" s="71"/>
+      <x:c r="N6" s="71"/>
+      <x:c r="O6" s="71"/>
+      <x:c r="P6" s="72" t="str">
         <x:f>TEXT('13-Week Forecast'!C$6,"dd mmm")</x:f>
         <x:v>13 Sep</x:v>
       </x:c>
-      <x:c r="Q6" s="39" t="n">
+      <x:c r="Q6" s="74" t="n">
         <x:f>'13-Week Forecast'!C$48</x:f>
         <x:v>349000</x:v>
       </x:c>
-      <x:c r="R6" s="39" t="n">
+      <x:c r="R6" s="74" t="n">
         <x:f>'13-Week Forecast'!C$49</x:f>
         <x:v>100000</x:v>
       </x:c>
+      <x:c r="S6" s="71"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="63" t="str">
@@ -1725,32 +1923,54 @@
         <x:f>'Checks &amp; Sources'!$E$4</x:f>
         <x:v>ACTION REQUIRED</x:v>
       </x:c>
-      <x:c r="P7" s="11" t="str">
+      <x:c r="K7" s="71"/>
+      <x:c r="L7" s="71"/>
+      <x:c r="M7" s="71"/>
+      <x:c r="N7" s="71"/>
+      <x:c r="O7" s="71"/>
+      <x:c r="P7" s="72" t="str">
         <x:f>TEXT('13-Week Forecast'!D$6,"dd mmm")</x:f>
         <x:v>20 Sep</x:v>
       </x:c>
-      <x:c r="Q7" s="39" t="n">
+      <x:c r="Q7" s="74" t="n">
         <x:f>'13-Week Forecast'!D$48</x:f>
         <x:v>325000</x:v>
       </x:c>
-      <x:c r="R7" s="39" t="n">
+      <x:c r="R7" s="74" t="n">
         <x:f>'13-Week Forecast'!D$49</x:f>
         <x:v>100000</x:v>
       </x:c>
+      <x:c r="S7" s="71"/>
     </x:row>
     <x:row r="8">
-      <x:c r="P8" s="11" t="str">
+      <x:c r="A8" s="71"/>
+      <x:c r="B8" s="71"/>
+      <x:c r="C8" s="71"/>
+      <x:c r="D8" s="71"/>
+      <x:c r="E8" s="71"/>
+      <x:c r="F8" s="71"/>
+      <x:c r="G8" s="71"/>
+      <x:c r="H8" s="71"/>
+      <x:c r="I8" s="71"/>
+      <x:c r="J8" s="71"/>
+      <x:c r="K8" s="71"/>
+      <x:c r="L8" s="71"/>
+      <x:c r="M8" s="71"/>
+      <x:c r="N8" s="71"/>
+      <x:c r="O8" s="71"/>
+      <x:c r="P8" s="72" t="str">
         <x:f>TEXT('13-Week Forecast'!E$6,"dd mmm")</x:f>
         <x:v>27 Sep</x:v>
       </x:c>
-      <x:c r="Q8" s="39" t="n">
+      <x:c r="Q8" s="74" t="n">
         <x:f>'13-Week Forecast'!E$48</x:f>
         <x:v>293000</x:v>
       </x:c>
-      <x:c r="R8" s="39" t="n">
+      <x:c r="R8" s="74" t="n">
         <x:f>'13-Week Forecast'!E$49</x:f>
         <x:v>100000</x:v>
       </x:c>
+      <x:c r="S8" s="71"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="59" t="str">
@@ -1765,18 +1985,30 @@
       <x:c r="D9" s="59" t="str">
         <x:v>Action deadline</x:v>
       </x:c>
-      <x:c r="P9" s="11" t="str">
+      <x:c r="E9" s="71"/>
+      <x:c r="F9" s="71"/>
+      <x:c r="G9" s="71"/>
+      <x:c r="H9" s="71"/>
+      <x:c r="I9" s="71"/>
+      <x:c r="J9" s="71"/>
+      <x:c r="K9" s="71"/>
+      <x:c r="L9" s="71"/>
+      <x:c r="M9" s="71"/>
+      <x:c r="N9" s="71"/>
+      <x:c r="O9" s="71"/>
+      <x:c r="P9" s="72" t="str">
         <x:f>TEXT('13-Week Forecast'!F$6,"dd mmm")</x:f>
         <x:v>04 Oct</x:v>
       </x:c>
-      <x:c r="Q9" s="39" t="n">
+      <x:c r="Q9" s="74" t="n">
         <x:f>'13-Week Forecast'!F$48</x:f>
         <x:v>201000</x:v>
       </x:c>
-      <x:c r="R9" s="39" t="n">
+      <x:c r="R9" s="74" t="n">
         <x:f>'13-Week Forecast'!F$49</x:f>
         <x:v>100000</x:v>
       </x:c>
+      <x:c r="S9" s="71"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="68" t="n">
@@ -1795,18 +2027,30 @@
         <x:f>IF(A10="None","None",A10-7*'Assumptions'!$B$19)</x:f>
         <x:v>46327</x:v>
       </x:c>
-      <x:c r="P10" s="11" t="str">
+      <x:c r="E10" s="71"/>
+      <x:c r="F10" s="71"/>
+      <x:c r="G10" s="71"/>
+      <x:c r="H10" s="71"/>
+      <x:c r="I10" s="71"/>
+      <x:c r="J10" s="71"/>
+      <x:c r="K10" s="71"/>
+      <x:c r="L10" s="71"/>
+      <x:c r="M10" s="71"/>
+      <x:c r="N10" s="71"/>
+      <x:c r="O10" s="71"/>
+      <x:c r="P10" s="72" t="str">
         <x:f>TEXT('13-Week Forecast'!G$6,"dd mmm")</x:f>
         <x:v>11 Oct</x:v>
       </x:c>
-      <x:c r="Q10" s="39" t="n">
+      <x:c r="Q10" s="74" t="n">
         <x:f>'13-Week Forecast'!G$48</x:f>
         <x:v>133000</x:v>
       </x:c>
-      <x:c r="R10" s="39" t="n">
+      <x:c r="R10" s="74" t="n">
         <x:f>'13-Week Forecast'!G$49</x:f>
         <x:v>100000</x:v>
       </x:c>
+      <x:c r="S10" s="71"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="14" t="str">
@@ -1824,21 +2068,32 @@
       <x:c r="E11" s="14" t="str">
         <x:v>Liquidity status</x:v>
       </x:c>
-      <x:c r="P11" s="11" t="str">
+      <x:c r="F11" s="71"/>
+      <x:c r="G11" s="71"/>
+      <x:c r="H11" s="71"/>
+      <x:c r="I11" s="71"/>
+      <x:c r="J11" s="71"/>
+      <x:c r="K11" s="71"/>
+      <x:c r="L11" s="71"/>
+      <x:c r="M11" s="71"/>
+      <x:c r="N11" s="71"/>
+      <x:c r="O11" s="71"/>
+      <x:c r="P11" s="72" t="str">
         <x:f>TEXT('13-Week Forecast'!H$6,"dd mmm")</x:f>
         <x:v>18 Oct</x:v>
       </x:c>
-      <x:c r="Q11" s="39" t="n">
+      <x:c r="Q11" s="74" t="n">
         <x:f>'13-Week Forecast'!H$48</x:f>
         <x:v>217000</x:v>
       </x:c>
-      <x:c r="R11" s="39" t="n">
+      <x:c r="R11" s="74" t="n">
         <x:f>'13-Week Forecast'!H$49</x:f>
         <x:v>100000</x:v>
       </x:c>
+      <x:c r="S11" s="71"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" t="n">
+      <x:c r="A12" s="71" t="n">
         <x:f>ROW()-11</x:f>
         <x:v>1</x:v>
       </x:c>
@@ -1858,21 +2113,32 @@
         <x:f>'13-Week Forecast'!B$51</x:f>
         <x:v>OK</x:v>
       </x:c>
-      <x:c r="P12" s="11" t="str">
+      <x:c r="F12" s="71"/>
+      <x:c r="G12" s="71"/>
+      <x:c r="H12" s="71"/>
+      <x:c r="I12" s="71"/>
+      <x:c r="J12" s="71"/>
+      <x:c r="K12" s="71"/>
+      <x:c r="L12" s="71"/>
+      <x:c r="M12" s="71"/>
+      <x:c r="N12" s="71"/>
+      <x:c r="O12" s="71"/>
+      <x:c r="P12" s="72" t="str">
         <x:f>TEXT('13-Week Forecast'!I$6,"dd mmm")</x:f>
         <x:v>25 Oct</x:v>
       </x:c>
-      <x:c r="Q12" s="39" t="n">
+      <x:c r="Q12" s="74" t="n">
         <x:f>'13-Week Forecast'!I$48</x:f>
         <x:v>160000</x:v>
       </x:c>
-      <x:c r="R12" s="39" t="n">
+      <x:c r="R12" s="74" t="n">
         <x:f>'13-Week Forecast'!I$49</x:f>
         <x:v>100000</x:v>
       </x:c>
+      <x:c r="S12" s="71"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" t="n">
+      <x:c r="A13" s="71" t="n">
         <x:f>ROW()-11</x:f>
         <x:v>2</x:v>
       </x:c>
@@ -1892,21 +2158,32 @@
         <x:f>'13-Week Forecast'!C$51</x:f>
         <x:v>OK</x:v>
       </x:c>
-      <x:c r="P13" s="11" t="str">
+      <x:c r="F13" s="71"/>
+      <x:c r="G13" s="71"/>
+      <x:c r="H13" s="71"/>
+      <x:c r="I13" s="71"/>
+      <x:c r="J13" s="71"/>
+      <x:c r="K13" s="71"/>
+      <x:c r="L13" s="71"/>
+      <x:c r="M13" s="71"/>
+      <x:c r="N13" s="71"/>
+      <x:c r="O13" s="71"/>
+      <x:c r="P13" s="72" t="str">
         <x:f>TEXT('13-Week Forecast'!J$6,"dd mmm")</x:f>
         <x:v>01 Nov</x:v>
       </x:c>
-      <x:c r="Q13" s="39" t="n">
+      <x:c r="Q13" s="74" t="n">
         <x:f>'13-Week Forecast'!J$48</x:f>
         <x:v>117000</x:v>
       </x:c>
-      <x:c r="R13" s="39" t="n">
+      <x:c r="R13" s="74" t="n">
         <x:f>'13-Week Forecast'!J$49</x:f>
         <x:v>100000</x:v>
       </x:c>
+      <x:c r="S13" s="71"/>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" t="n">
+      <x:c r="A14" s="71" t="n">
         <x:f>ROW()-11</x:f>
         <x:v>3</x:v>
       </x:c>
@@ -1926,21 +2203,32 @@
         <x:f>'13-Week Forecast'!D$51</x:f>
         <x:v>OK</x:v>
       </x:c>
-      <x:c r="P14" s="11" t="str">
+      <x:c r="F14" s="71"/>
+      <x:c r="G14" s="71"/>
+      <x:c r="H14" s="71"/>
+      <x:c r="I14" s="71"/>
+      <x:c r="J14" s="71"/>
+      <x:c r="K14" s="71"/>
+      <x:c r="L14" s="71"/>
+      <x:c r="M14" s="71"/>
+      <x:c r="N14" s="71"/>
+      <x:c r="O14" s="71"/>
+      <x:c r="P14" s="72" t="str">
         <x:f>TEXT('13-Week Forecast'!K$6,"dd mmm")</x:f>
         <x:v>08 Nov</x:v>
       </x:c>
-      <x:c r="Q14" s="39" t="n">
+      <x:c r="Q14" s="74" t="n">
         <x:f>'13-Week Forecast'!K$48</x:f>
         <x:v>137000</x:v>
       </x:c>
-      <x:c r="R14" s="39" t="n">
+      <x:c r="R14" s="74" t="n">
         <x:f>'13-Week Forecast'!K$49</x:f>
         <x:v>100000</x:v>
       </x:c>
+      <x:c r="S14" s="71"/>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" t="n">
+      <x:c r="A15" s="71" t="n">
         <x:f>ROW()-11</x:f>
         <x:v>4</x:v>
       </x:c>
@@ -1960,21 +2248,32 @@
         <x:f>'13-Week Forecast'!E$51</x:f>
         <x:v>OK</x:v>
       </x:c>
-      <x:c r="P15" s="11" t="str">
+      <x:c r="F15" s="71"/>
+      <x:c r="G15" s="71"/>
+      <x:c r="H15" s="71"/>
+      <x:c r="I15" s="71"/>
+      <x:c r="J15" s="71"/>
+      <x:c r="K15" s="71"/>
+      <x:c r="L15" s="71"/>
+      <x:c r="M15" s="71"/>
+      <x:c r="N15" s="71"/>
+      <x:c r="O15" s="71"/>
+      <x:c r="P15" s="72" t="str">
         <x:f>TEXT('13-Week Forecast'!L$6,"dd mmm")</x:f>
         <x:v>15 Nov</x:v>
       </x:c>
-      <x:c r="Q15" s="39" t="n">
+      <x:c r="Q15" s="74" t="n">
         <x:f>'13-Week Forecast'!L$48</x:f>
         <x:v>99000</x:v>
       </x:c>
-      <x:c r="R15" s="39" t="n">
+      <x:c r="R15" s="74" t="n">
         <x:f>'13-Week Forecast'!L$49</x:f>
         <x:v>100000</x:v>
       </x:c>
+      <x:c r="S15" s="71"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" t="n">
+      <x:c r="A16" s="71" t="n">
         <x:f>ROW()-11</x:f>
         <x:v>5</x:v>
       </x:c>
@@ -1994,21 +2293,32 @@
         <x:f>'13-Week Forecast'!F$51</x:f>
         <x:v>OK</x:v>
       </x:c>
-      <x:c r="P16" s="11" t="str">
+      <x:c r="F16" s="71"/>
+      <x:c r="G16" s="71"/>
+      <x:c r="H16" s="71"/>
+      <x:c r="I16" s="71"/>
+      <x:c r="J16" s="71"/>
+      <x:c r="K16" s="71"/>
+      <x:c r="L16" s="71"/>
+      <x:c r="M16" s="71"/>
+      <x:c r="N16" s="71"/>
+      <x:c r="O16" s="71"/>
+      <x:c r="P16" s="72" t="str">
         <x:f>TEXT('13-Week Forecast'!M$6,"dd mmm")</x:f>
         <x:v>22 Nov</x:v>
       </x:c>
-      <x:c r="Q16" s="39" t="n">
+      <x:c r="Q16" s="74" t="n">
         <x:f>'13-Week Forecast'!M$48</x:f>
         <x:v>82000</x:v>
       </x:c>
-      <x:c r="R16" s="39" t="n">
+      <x:c r="R16" s="74" t="n">
         <x:f>'13-Week Forecast'!M$49</x:f>
         <x:v>100000</x:v>
       </x:c>
+      <x:c r="S16" s="71"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" t="n">
+      <x:c r="A17" s="71" t="n">
         <x:f>ROW()-11</x:f>
         <x:v>6</x:v>
       </x:c>
@@ -2028,21 +2338,32 @@
         <x:f>'13-Week Forecast'!G$51</x:f>
         <x:v>OK</x:v>
       </x:c>
-      <x:c r="P17" s="11" t="str">
+      <x:c r="F17" s="71"/>
+      <x:c r="G17" s="71"/>
+      <x:c r="H17" s="71"/>
+      <x:c r="I17" s="71"/>
+      <x:c r="J17" s="71"/>
+      <x:c r="K17" s="71"/>
+      <x:c r="L17" s="71"/>
+      <x:c r="M17" s="71"/>
+      <x:c r="N17" s="71"/>
+      <x:c r="O17" s="71"/>
+      <x:c r="P17" s="72" t="str">
         <x:f>TEXT('13-Week Forecast'!N$6,"dd mmm")</x:f>
         <x:v>29 Nov</x:v>
       </x:c>
-      <x:c r="Q17" s="39" t="n">
+      <x:c r="Q17" s="74" t="n">
         <x:f>'13-Week Forecast'!N$48</x:f>
         <x:v>31000</x:v>
       </x:c>
-      <x:c r="R17" s="39" t="n">
+      <x:c r="R17" s="74" t="n">
         <x:f>'13-Week Forecast'!N$49</x:f>
         <x:v>100000</x:v>
       </x:c>
+      <x:c r="S17" s="71"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" t="n">
+      <x:c r="A18" s="71" t="n">
         <x:f>ROW()-11</x:f>
         <x:v>7</x:v>
       </x:c>
@@ -2062,9 +2383,23 @@
         <x:f>'13-Week Forecast'!H$51</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="F18" s="71"/>
+      <x:c r="G18" s="71"/>
+      <x:c r="H18" s="71"/>
+      <x:c r="I18" s="71"/>
+      <x:c r="J18" s="71"/>
+      <x:c r="K18" s="71"/>
+      <x:c r="L18" s="71"/>
+      <x:c r="M18" s="71"/>
+      <x:c r="N18" s="71"/>
+      <x:c r="O18" s="71"/>
+      <x:c r="P18" s="71"/>
+      <x:c r="Q18" s="71"/>
+      <x:c r="R18" s="71"/>
+      <x:c r="S18" s="71"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" t="n">
+      <x:c r="A19" s="71" t="n">
         <x:f>ROW()-11</x:f>
         <x:v>8</x:v>
       </x:c>
@@ -2084,9 +2419,23 @@
         <x:f>'13-Week Forecast'!I$51</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="F19" s="71"/>
+      <x:c r="G19" s="71"/>
+      <x:c r="H19" s="71"/>
+      <x:c r="I19" s="71"/>
+      <x:c r="J19" s="71"/>
+      <x:c r="K19" s="71"/>
+      <x:c r="L19" s="71"/>
+      <x:c r="M19" s="71"/>
+      <x:c r="N19" s="71"/>
+      <x:c r="O19" s="71"/>
+      <x:c r="P19" s="71"/>
+      <x:c r="Q19" s="71"/>
+      <x:c r="R19" s="71"/>
+      <x:c r="S19" s="71"/>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" t="n">
+      <x:c r="A20" s="71" t="n">
         <x:f>ROW()-11</x:f>
         <x:v>9</x:v>
       </x:c>
@@ -2106,9 +2455,23 @@
         <x:f>'13-Week Forecast'!J$51</x:f>
         <x:v>WATCH</x:v>
       </x:c>
+      <x:c r="F20" s="71"/>
+      <x:c r="G20" s="71"/>
+      <x:c r="H20" s="71"/>
+      <x:c r="I20" s="71"/>
+      <x:c r="J20" s="71"/>
+      <x:c r="K20" s="71"/>
+      <x:c r="L20" s="71"/>
+      <x:c r="M20" s="71"/>
+      <x:c r="N20" s="71"/>
+      <x:c r="O20" s="71"/>
+      <x:c r="P20" s="71"/>
+      <x:c r="Q20" s="71"/>
+      <x:c r="R20" s="71"/>
+      <x:c r="S20" s="71"/>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" t="n">
+      <x:c r="A21" s="71" t="n">
         <x:f>ROW()-11</x:f>
         <x:v>10</x:v>
       </x:c>
@@ -2128,6 +2491,16 @@
         <x:f>'13-Week Forecast'!K$51</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="F21" s="71"/>
+      <x:c r="G21" s="71"/>
+      <x:c r="H21" s="71"/>
+      <x:c r="I21" s="71"/>
+      <x:c r="J21" s="71"/>
+      <x:c r="K21" s="71"/>
+      <x:c r="L21" s="71"/>
+      <x:c r="M21" s="71"/>
+      <x:c r="N21" s="71"/>
+      <x:c r="O21" s="71"/>
       <x:c r="P21" s="14" t="str">
         <x:v>Week ending</x:v>
       </x:c>
@@ -2137,9 +2510,10 @@
       <x:c r="R21" s="14" t="str">
         <x:v>Total cash payments</x:v>
       </x:c>
+      <x:c r="S21" s="71"/>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" t="n">
+      <x:c r="A22" s="71" t="n">
         <x:f>ROW()-11</x:f>
         <x:v>11</x:v>
       </x:c>
@@ -2159,21 +2533,32 @@
         <x:f>'13-Week Forecast'!L$51</x:f>
         <x:v>BELOW BUFFER</x:v>
       </x:c>
-      <x:c r="P22" s="11" t="str">
+      <x:c r="F22" s="71"/>
+      <x:c r="G22" s="71"/>
+      <x:c r="H22" s="71"/>
+      <x:c r="I22" s="71"/>
+      <x:c r="J22" s="71"/>
+      <x:c r="K22" s="71"/>
+      <x:c r="L22" s="71"/>
+      <x:c r="M22" s="71"/>
+      <x:c r="N22" s="71"/>
+      <x:c r="O22" s="71"/>
+      <x:c r="P22" s="72" t="str">
         <x:f>TEXT('13-Week Forecast'!B$6,"dd mmm")</x:f>
         <x:v>06 Sep</x:v>
       </x:c>
-      <x:c r="Q22" s="39" t="n">
+      <x:c r="Q22" s="74" t="n">
         <x:f>'13-Week Forecast'!B$19</x:f>
         <x:v>170000</x:v>
       </x:c>
-      <x:c r="R22" s="39" t="n">
+      <x:c r="R22" s="74" t="n">
         <x:f>'13-Week Forecast'!B$43</x:f>
         <x:v>212000</x:v>
       </x:c>
+      <x:c r="S22" s="71"/>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" t="n">
+      <x:c r="A23" s="71" t="n">
         <x:f>ROW()-11</x:f>
         <x:v>12</x:v>
       </x:c>
@@ -2193,21 +2578,32 @@
         <x:f>'13-Week Forecast'!M$51</x:f>
         <x:v>BELOW BUFFER</x:v>
       </x:c>
-      <x:c r="P23" s="11" t="str">
+      <x:c r="F23" s="71"/>
+      <x:c r="G23" s="71"/>
+      <x:c r="H23" s="71"/>
+      <x:c r="I23" s="71"/>
+      <x:c r="J23" s="71"/>
+      <x:c r="K23" s="71"/>
+      <x:c r="L23" s="71"/>
+      <x:c r="M23" s="71"/>
+      <x:c r="N23" s="71"/>
+      <x:c r="O23" s="71"/>
+      <x:c r="P23" s="72" t="str">
         <x:f>TEXT('13-Week Forecast'!C$6,"dd mmm")</x:f>
         <x:v>13 Sep</x:v>
       </x:c>
-      <x:c r="Q23" s="39" t="n">
+      <x:c r="Q23" s="74" t="n">
         <x:f>'13-Week Forecast'!C$19</x:f>
         <x:v>169000</x:v>
       </x:c>
-      <x:c r="R23" s="39" t="n">
+      <x:c r="R23" s="74" t="n">
         <x:f>'13-Week Forecast'!C$43</x:f>
         <x:v>178000</x:v>
       </x:c>
+      <x:c r="S23" s="71"/>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" t="n">
+      <x:c r="A24" s="71" t="n">
         <x:f>ROW()-11</x:f>
         <x:v>13</x:v>
       </x:c>
@@ -2227,46 +2623,89 @@
         <x:f>'13-Week Forecast'!N$51</x:f>
         <x:v>BELOW BUFFER</x:v>
       </x:c>
-      <x:c r="P24" s="11" t="str">
+      <x:c r="F24" s="71"/>
+      <x:c r="G24" s="71"/>
+      <x:c r="H24" s="71"/>
+      <x:c r="I24" s="71"/>
+      <x:c r="J24" s="71"/>
+      <x:c r="K24" s="71"/>
+      <x:c r="L24" s="71"/>
+      <x:c r="M24" s="71"/>
+      <x:c r="N24" s="71"/>
+      <x:c r="O24" s="71"/>
+      <x:c r="P24" s="72" t="str">
         <x:f>TEXT('13-Week Forecast'!D$6,"dd mmm")</x:f>
         <x:v>20 Sep</x:v>
       </x:c>
-      <x:c r="Q24" s="39" t="n">
+      <x:c r="Q24" s="74" t="n">
         <x:f>'13-Week Forecast'!D$19</x:f>
         <x:v>158000</x:v>
       </x:c>
-      <x:c r="R24" s="39" t="n">
+      <x:c r="R24" s="74" t="n">
         <x:f>'13-Week Forecast'!D$43</x:f>
         <x:v>182000</x:v>
       </x:c>
+      <x:c r="S24" s="71"/>
     </x:row>
     <x:row r="25">
-      <x:c r="P25" s="11" t="str">
+      <x:c r="A25" s="71"/>
+      <x:c r="B25" s="71"/>
+      <x:c r="C25" s="71"/>
+      <x:c r="D25" s="71"/>
+      <x:c r="E25" s="71"/>
+      <x:c r="F25" s="71"/>
+      <x:c r="G25" s="71"/>
+      <x:c r="H25" s="71"/>
+      <x:c r="I25" s="71"/>
+      <x:c r="J25" s="71"/>
+      <x:c r="K25" s="71"/>
+      <x:c r="L25" s="71"/>
+      <x:c r="M25" s="71"/>
+      <x:c r="N25" s="71"/>
+      <x:c r="O25" s="71"/>
+      <x:c r="P25" s="72" t="str">
         <x:f>TEXT('13-Week Forecast'!E$6,"dd mmm")</x:f>
         <x:v>27 Sep</x:v>
       </x:c>
-      <x:c r="Q25" s="39" t="n">
+      <x:c r="Q25" s="74" t="n">
         <x:f>'13-Week Forecast'!E$19</x:f>
         <x:v>147000</x:v>
       </x:c>
-      <x:c r="R25" s="39" t="n">
+      <x:c r="R25" s="74" t="n">
         <x:f>'13-Week Forecast'!E$43</x:f>
         <x:v>179000</x:v>
       </x:c>
+      <x:c r="S25" s="71"/>
     </x:row>
     <x:row r="26">
-      <x:c r="P26" s="11" t="str">
+      <x:c r="A26" s="71"/>
+      <x:c r="B26" s="71"/>
+      <x:c r="C26" s="71"/>
+      <x:c r="D26" s="71"/>
+      <x:c r="E26" s="71"/>
+      <x:c r="F26" s="71"/>
+      <x:c r="G26" s="71"/>
+      <x:c r="H26" s="71"/>
+      <x:c r="I26" s="71"/>
+      <x:c r="J26" s="71"/>
+      <x:c r="K26" s="71"/>
+      <x:c r="L26" s="71"/>
+      <x:c r="M26" s="71"/>
+      <x:c r="N26" s="71"/>
+      <x:c r="O26" s="71"/>
+      <x:c r="P26" s="72" t="str">
         <x:f>TEXT('13-Week Forecast'!F$6,"dd mmm")</x:f>
         <x:v>04 Oct</x:v>
       </x:c>
-      <x:c r="Q26" s="39" t="n">
+      <x:c r="Q26" s="74" t="n">
         <x:f>'13-Week Forecast'!F$19</x:f>
         <x:v>140000</x:v>
       </x:c>
-      <x:c r="R26" s="39" t="n">
+      <x:c r="R26" s="74" t="n">
         <x:f>'13-Week Forecast'!F$43</x:f>
         <x:v>232000</x:v>
       </x:c>
+      <x:c r="S26" s="71"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="45" t="str">
@@ -2284,178 +2723,322 @@
       <x:c r="E27" s="45" t="str">
         <x:v>Funding required</x:v>
       </x:c>
-      <x:c r="P27" s="11" t="str">
+      <x:c r="F27" s="71"/>
+      <x:c r="G27" s="71"/>
+      <x:c r="H27" s="71"/>
+      <x:c r="I27" s="71"/>
+      <x:c r="J27" s="71"/>
+      <x:c r="K27" s="71"/>
+      <x:c r="L27" s="71"/>
+      <x:c r="M27" s="71"/>
+      <x:c r="N27" s="71"/>
+      <x:c r="O27" s="71"/>
+      <x:c r="P27" s="72" t="str">
         <x:f>TEXT('13-Week Forecast'!G$6,"dd mmm")</x:f>
         <x:v>11 Oct</x:v>
       </x:c>
-      <x:c r="Q27" s="39" t="n">
+      <x:c r="Q27" s="74" t="n">
         <x:f>'13-Week Forecast'!G$19</x:f>
         <x:v>141000</x:v>
       </x:c>
-      <x:c r="R27" s="39" t="n">
+      <x:c r="R27" s="74" t="n">
         <x:f>'13-Week Forecast'!G$43</x:f>
         <x:v>209000</x:v>
       </x:c>
+      <x:c r="S27" s="71"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="12" t="str">
         <x:f>'Assumptions'!$B$15</x:f>
         <x:v>Base</x:v>
       </x:c>
-      <x:c r="B28" s="39" t="n">
+      <x:c r="B28" s="74" t="n">
         <x:f>Q49</x:f>
         <x:v>31000</x:v>
       </x:c>
-      <x:c r="C28" s="39" t="n">
+      <x:c r="C28" s="74" t="n">
         <x:f>MIN(Q37:Q49)</x:f>
         <x:v>31000</x:v>
       </x:c>
-      <x:c r="D28" s="11" t="n">
+      <x:c r="D28" s="72" t="n">
         <x:f>IF(Q37&lt;'Assumptions'!$B$11,P37,IF(Q38&lt;'Assumptions'!$B$11,P38,IF(Q39&lt;'Assumptions'!$B$11,P39,IF(Q40&lt;'Assumptions'!$B$11,P40,IF(Q41&lt;'Assumptions'!$B$11,P41,IF(Q42&lt;'Assumptions'!$B$11,P42,IF(Q43&lt;'Assumptions'!$B$11,P43,IF(Q44&lt;'Assumptions'!$B$11,P44,IF(Q45&lt;'Assumptions'!$B$11,P45,IF(Q46&lt;'Assumptions'!$B$11,P46,IF(Q47&lt;'Assumptions'!$B$11,P47,IF(Q48&lt;'Assumptions'!$B$11,P48,IF(Q49&lt;'Assumptions'!$B$11,P49,"None")))))))))))))</x:f>
         <x:v>46341</x:v>
       </x:c>
-      <x:c r="E28" s="39" t="n">
+      <x:c r="E28" s="74" t="n">
         <x:f>MAX(0,'Assumptions'!$B$11-MIN(Q37:Q49))</x:f>
         <x:v>69000</x:v>
       </x:c>
-      <x:c r="P28" s="11" t="str">
+      <x:c r="F28" s="71"/>
+      <x:c r="G28" s="71"/>
+      <x:c r="H28" s="71"/>
+      <x:c r="I28" s="71"/>
+      <x:c r="J28" s="71"/>
+      <x:c r="K28" s="71"/>
+      <x:c r="L28" s="71"/>
+      <x:c r="M28" s="71"/>
+      <x:c r="N28" s="71"/>
+      <x:c r="O28" s="71"/>
+      <x:c r="P28" s="72" t="str">
         <x:f>TEXT('13-Week Forecast'!H$6,"dd mmm")</x:f>
         <x:v>18 Oct</x:v>
       </x:c>
-      <x:c r="Q28" s="39" t="n">
+      <x:c r="Q28" s="74" t="n">
         <x:f>'13-Week Forecast'!H$19</x:f>
         <x:v>281000</x:v>
       </x:c>
-      <x:c r="R28" s="39" t="n">
+      <x:c r="R28" s="74" t="n">
         <x:f>'13-Week Forecast'!H$43</x:f>
         <x:v>197000</x:v>
       </x:c>
+      <x:c r="S28" s="71"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="12" t="str">
         <x:f>'Assumptions'!$B$16</x:f>
         <x:v>Upside</x:v>
       </x:c>
-      <x:c r="B29" s="39" t="n">
+      <x:c r="B29" s="74" t="n">
         <x:f>R49</x:f>
         <x:v>199320</x:v>
       </x:c>
-      <x:c r="C29" s="39" t="n">
+      <x:c r="C29" s="74" t="n">
         <x:f>MIN(R37:R49)</x:f>
         <x:v>199320</x:v>
       </x:c>
-      <x:c r="D29" s="11" t="str">
+      <x:c r="D29" s="72" t="str">
         <x:f>IF(R37&lt;'Assumptions'!$B$11,P37,IF(R38&lt;'Assumptions'!$B$11,P38,IF(R39&lt;'Assumptions'!$B$11,P39,IF(R40&lt;'Assumptions'!$B$11,P40,IF(R41&lt;'Assumptions'!$B$11,P41,IF(R42&lt;'Assumptions'!$B$11,P42,IF(R43&lt;'Assumptions'!$B$11,P43,IF(R44&lt;'Assumptions'!$B$11,P44,IF(R45&lt;'Assumptions'!$B$11,P45,IF(R46&lt;'Assumptions'!$B$11,P46,IF(R47&lt;'Assumptions'!$B$11,P47,IF(R48&lt;'Assumptions'!$B$11,P48,IF(R49&lt;'Assumptions'!$B$11,P49,"None")))))))))))))</x:f>
         <x:v>None</x:v>
       </x:c>
-      <x:c r="E29" s="39" t="n">
+      <x:c r="E29" s="74" t="n">
         <x:f>MAX(0,'Assumptions'!$B$11-MIN(R37:R49))</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="P29" s="11" t="str">
+      <x:c r="F29" s="71"/>
+      <x:c r="G29" s="71"/>
+      <x:c r="H29" s="71"/>
+      <x:c r="I29" s="71"/>
+      <x:c r="J29" s="71"/>
+      <x:c r="K29" s="71"/>
+      <x:c r="L29" s="71"/>
+      <x:c r="M29" s="71"/>
+      <x:c r="N29" s="71"/>
+      <x:c r="O29" s="71"/>
+      <x:c r="P29" s="72" t="str">
         <x:f>TEXT('13-Week Forecast'!I$6,"dd mmm")</x:f>
         <x:v>25 Oct</x:v>
       </x:c>
-      <x:c r="Q29" s="39" t="n">
+      <x:c r="Q29" s="74" t="n">
         <x:f>'13-Week Forecast'!I$19</x:f>
         <x:v>135000</x:v>
       </x:c>
-      <x:c r="R29" s="39" t="n">
+      <x:c r="R29" s="74" t="n">
         <x:f>'13-Week Forecast'!I$43</x:f>
         <x:v>192000</x:v>
       </x:c>
+      <x:c r="S29" s="71"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="12" t="str">
         <x:f>'Assumptions'!$B$17</x:f>
         <x:v>Downside</x:v>
       </x:c>
-      <x:c r="B30" s="39" t="n">
+      <x:c r="B30" s="74" t="n">
         <x:f>S49</x:f>
         <x:v>-302550</x:v>
       </x:c>
-      <x:c r="C30" s="39" t="n">
+      <x:c r="C30" s="74" t="n">
         <x:f>MIN(S37:S49)</x:f>
         <x:v>-302550</x:v>
       </x:c>
-      <x:c r="D30" s="11" t="n">
+      <x:c r="D30" s="72" t="n">
         <x:f>IF(S37&lt;'Assumptions'!$B$11,P37,IF(S38&lt;'Assumptions'!$B$11,P38,IF(S39&lt;'Assumptions'!$B$11,P39,IF(S40&lt;'Assumptions'!$B$11,P40,IF(S41&lt;'Assumptions'!$B$11,P41,IF(S42&lt;'Assumptions'!$B$11,P42,IF(S43&lt;'Assumptions'!$B$11,P43,IF(S44&lt;'Assumptions'!$B$11,P44,IF(S45&lt;'Assumptions'!$B$11,P45,IF(S46&lt;'Assumptions'!$B$11,P46,IF(S47&lt;'Assumptions'!$B$11,P47,IF(S48&lt;'Assumptions'!$B$11,P48,IF(S49&lt;'Assumptions'!$B$11,P49,"None")))))))))))))</x:f>
         <x:v>46299</x:v>
       </x:c>
-      <x:c r="E30" s="39" t="n">
+      <x:c r="E30" s="74" t="n">
         <x:f>MAX(0,'Assumptions'!$B$11-MIN(S37:S49))</x:f>
         <x:v>402550</x:v>
       </x:c>
-      <x:c r="P30" s="11" t="str">
+      <x:c r="F30" s="71"/>
+      <x:c r="G30" s="71"/>
+      <x:c r="H30" s="71"/>
+      <x:c r="I30" s="71"/>
+      <x:c r="J30" s="71"/>
+      <x:c r="K30" s="71"/>
+      <x:c r="L30" s="71"/>
+      <x:c r="M30" s="71"/>
+      <x:c r="N30" s="71"/>
+      <x:c r="O30" s="71"/>
+      <x:c r="P30" s="72" t="str">
         <x:f>TEXT('13-Week Forecast'!J$6,"dd mmm")</x:f>
         <x:v>01 Nov</x:v>
       </x:c>
-      <x:c r="Q30" s="39" t="n">
+      <x:c r="Q30" s="74" t="n">
         <x:f>'13-Week Forecast'!J$19</x:f>
         <x:v>264000</x:v>
       </x:c>
-      <x:c r="R30" s="39" t="n">
+      <x:c r="R30" s="74" t="n">
         <x:f>'13-Week Forecast'!J$43</x:f>
         <x:v>307000</x:v>
       </x:c>
+      <x:c r="S30" s="71"/>
     </x:row>
     <x:row r="31">
-      <x:c r="P31" s="11" t="str">
+      <x:c r="A31" s="71"/>
+      <x:c r="B31" s="71"/>
+      <x:c r="C31" s="71"/>
+      <x:c r="D31" s="71"/>
+      <x:c r="E31" s="71"/>
+      <x:c r="F31" s="71"/>
+      <x:c r="G31" s="71"/>
+      <x:c r="H31" s="71"/>
+      <x:c r="I31" s="71"/>
+      <x:c r="J31" s="71"/>
+      <x:c r="K31" s="71"/>
+      <x:c r="L31" s="71"/>
+      <x:c r="M31" s="71"/>
+      <x:c r="N31" s="71"/>
+      <x:c r="O31" s="71"/>
+      <x:c r="P31" s="72" t="str">
         <x:f>TEXT('13-Week Forecast'!K$6,"dd mmm")</x:f>
         <x:v>08 Nov</x:v>
       </x:c>
-      <x:c r="Q31" s="39" t="n">
+      <x:c r="Q31" s="74" t="n">
         <x:f>'13-Week Forecast'!K$19</x:f>
         <x:v>249000</x:v>
       </x:c>
-      <x:c r="R31" s="39" t="n">
+      <x:c r="R31" s="74" t="n">
         <x:f>'13-Week Forecast'!K$43</x:f>
         <x:v>229000</x:v>
       </x:c>
+      <x:c r="S31" s="71"/>
     </x:row>
     <x:row r="32">
-      <x:c r="P32" s="11" t="str">
+      <x:c r="A32" s="71"/>
+      <x:c r="B32" s="71"/>
+      <x:c r="C32" s="71"/>
+      <x:c r="D32" s="71"/>
+      <x:c r="E32" s="71"/>
+      <x:c r="F32" s="71"/>
+      <x:c r="G32" s="71"/>
+      <x:c r="H32" s="71"/>
+      <x:c r="I32" s="71"/>
+      <x:c r="J32" s="71"/>
+      <x:c r="K32" s="71"/>
+      <x:c r="L32" s="71"/>
+      <x:c r="M32" s="71"/>
+      <x:c r="N32" s="71"/>
+      <x:c r="O32" s="71"/>
+      <x:c r="P32" s="72" t="str">
         <x:f>TEXT('13-Week Forecast'!L$6,"dd mmm")</x:f>
         <x:v>15 Nov</x:v>
       </x:c>
-      <x:c r="Q32" s="39" t="n">
+      <x:c r="Q32" s="74" t="n">
         <x:f>'13-Week Forecast'!L$19</x:f>
         <x:v>154000</x:v>
       </x:c>
-      <x:c r="R32" s="39" t="n">
+      <x:c r="R32" s="74" t="n">
         <x:f>'13-Week Forecast'!L$43</x:f>
         <x:v>192000</x:v>
       </x:c>
+      <x:c r="S32" s="71"/>
     </x:row>
     <x:row r="33">
-      <x:c r="P33" s="11" t="str">
+      <x:c r="A33" s="71"/>
+      <x:c r="B33" s="71"/>
+      <x:c r="C33" s="71"/>
+      <x:c r="D33" s="71"/>
+      <x:c r="E33" s="71"/>
+      <x:c r="F33" s="71"/>
+      <x:c r="G33" s="71"/>
+      <x:c r="H33" s="71"/>
+      <x:c r="I33" s="71"/>
+      <x:c r="J33" s="71"/>
+      <x:c r="K33" s="71"/>
+      <x:c r="L33" s="71"/>
+      <x:c r="M33" s="71"/>
+      <x:c r="N33" s="71"/>
+      <x:c r="O33" s="71"/>
+      <x:c r="P33" s="72" t="str">
         <x:f>TEXT('13-Week Forecast'!M$6,"dd mmm")</x:f>
         <x:v>22 Nov</x:v>
       </x:c>
-      <x:c r="Q33" s="39" t="n">
+      <x:c r="Q33" s="74" t="n">
         <x:f>'13-Week Forecast'!M$19</x:f>
         <x:v>162000</x:v>
       </x:c>
-      <x:c r="R33" s="39" t="n">
+      <x:c r="R33" s="74" t="n">
         <x:f>'13-Week Forecast'!M$43</x:f>
         <x:v>179000</x:v>
       </x:c>
+      <x:c r="S33" s="71"/>
     </x:row>
     <x:row r="34">
-      <x:c r="P34" s="11" t="str">
+      <x:c r="A34" s="71"/>
+      <x:c r="B34" s="71"/>
+      <x:c r="C34" s="71"/>
+      <x:c r="D34" s="71"/>
+      <x:c r="E34" s="71"/>
+      <x:c r="F34" s="71"/>
+      <x:c r="G34" s="71"/>
+      <x:c r="H34" s="71"/>
+      <x:c r="I34" s="71"/>
+      <x:c r="J34" s="71"/>
+      <x:c r="K34" s="71"/>
+      <x:c r="L34" s="71"/>
+      <x:c r="M34" s="71"/>
+      <x:c r="N34" s="71"/>
+      <x:c r="O34" s="71"/>
+      <x:c r="P34" s="72" t="str">
         <x:f>TEXT('13-Week Forecast'!N$6,"dd mmm")</x:f>
         <x:v>29 Nov</x:v>
       </x:c>
-      <x:c r="Q34" s="39" t="n">
+      <x:c r="Q34" s="74" t="n">
         <x:f>'13-Week Forecast'!N$19</x:f>
         <x:v>168000</x:v>
       </x:c>
-      <x:c r="R34" s="39" t="n">
+      <x:c r="R34" s="74" t="n">
         <x:f>'13-Week Forecast'!N$43</x:f>
         <x:v>219000</x:v>
       </x:c>
+      <x:c r="S34" s="71"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="71"/>
+      <x:c r="B35" s="71"/>
+      <x:c r="C35" s="71"/>
+      <x:c r="D35" s="71"/>
+      <x:c r="E35" s="71"/>
+      <x:c r="F35" s="71"/>
+      <x:c r="G35" s="71"/>
+      <x:c r="H35" s="71"/>
+      <x:c r="I35" s="71"/>
+      <x:c r="J35" s="71"/>
+      <x:c r="K35" s="71"/>
+      <x:c r="L35" s="71"/>
+      <x:c r="M35" s="71"/>
+      <x:c r="N35" s="71"/>
+      <x:c r="O35" s="71"/>
+      <x:c r="P35" s="71"/>
+      <x:c r="Q35" s="71"/>
+      <x:c r="R35" s="71"/>
+      <x:c r="S35" s="71"/>
     </x:row>
     <x:row r="36">
+      <x:c r="A36" s="71"/>
+      <x:c r="B36" s="71"/>
+      <x:c r="C36" s="71"/>
+      <x:c r="D36" s="71"/>
+      <x:c r="E36" s="71"/>
+      <x:c r="F36" s="71"/>
+      <x:c r="G36" s="71"/>
+      <x:c r="H36" s="71"/>
+      <x:c r="I36" s="71"/>
+      <x:c r="J36" s="71"/>
+      <x:c r="K36" s="71"/>
+      <x:c r="L36" s="71"/>
+      <x:c r="M36" s="71"/>
+      <x:c r="N36" s="71"/>
+      <x:c r="O36" s="71"/>
       <x:c r="P36" s="14" t="str">
         <x:v>Week ending</x:v>
       </x:c>
@@ -2470,235 +3053,430 @@
       </x:c>
     </x:row>
     <x:row r="37">
-      <x:c r="P37" s="11" t="n">
+      <x:c r="A37" s="71"/>
+      <x:c r="B37" s="71"/>
+      <x:c r="C37" s="71"/>
+      <x:c r="D37" s="71"/>
+      <x:c r="E37" s="71"/>
+      <x:c r="F37" s="71"/>
+      <x:c r="G37" s="71"/>
+      <x:c r="H37" s="71"/>
+      <x:c r="I37" s="71"/>
+      <x:c r="J37" s="71"/>
+      <x:c r="K37" s="71"/>
+      <x:c r="L37" s="71"/>
+      <x:c r="M37" s="71"/>
+      <x:c r="N37" s="71"/>
+      <x:c r="O37" s="71"/>
+      <x:c r="P37" s="72" t="n">
         <x:f>'13-Week Forecast'!B$6</x:f>
         <x:v>46271</x:v>
       </x:c>
-      <x:c r="Q37" s="39" t="n">
+      <x:c r="Q37" s="74" t="n">
         <x:f>'Assumptions'!$B$10+SUM('13-Week Forecast'!B10:B17)+IF('13-Week Forecast'!B$7="Actual",0,SUM('13-Week Forecast'!B10:B12)*('Assumptions'!$C$15-1))-(SUM('13-Week Forecast'!B22:B41)+IF('13-Week Forecast'!B$7="Actual",0,SUM('13-Week Forecast'!B22,'13-Week Forecast'!B31,'13-Week Forecast'!B33,'13-Week Forecast'!B41)*('Assumptions'!$D$15-1)))</x:f>
         <x:v>358000</x:v>
       </x:c>
-      <x:c r="R37" s="39" t="n">
+      <x:c r="R37" s="74" t="n">
         <x:f>'Assumptions'!$B$10+SUM('13-Week Forecast'!B10:B17)+IF('13-Week Forecast'!B$7="Actual",0,SUM('13-Week Forecast'!B10:B12)*('Assumptions'!$C$16-1))-(SUM('13-Week Forecast'!B22:B41)+IF('13-Week Forecast'!B$7="Actual",0,SUM('13-Week Forecast'!B22,'13-Week Forecast'!B31,'13-Week Forecast'!B33,'13-Week Forecast'!B41)*('Assumptions'!$D$16-1)))</x:f>
         <x:v>358000</x:v>
       </x:c>
-      <x:c r="S37" s="39" t="n">
+      <x:c r="S37" s="74" t="n">
         <x:f>'Assumptions'!$B$10+SUM('13-Week Forecast'!B10:B17)+IF('13-Week Forecast'!B$7="Actual",0,SUM('13-Week Forecast'!B10:B12)*('Assumptions'!$C$17-1))-(SUM('13-Week Forecast'!B22:B41)+IF('13-Week Forecast'!B$7="Actual",0,SUM('13-Week Forecast'!B22,'13-Week Forecast'!B31,'13-Week Forecast'!B33,'13-Week Forecast'!B41)*('Assumptions'!$D$17-1)))</x:f>
         <x:v>358000</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
-      <x:c r="P38" s="11" t="n">
+      <x:c r="A38" s="71"/>
+      <x:c r="B38" s="71"/>
+      <x:c r="C38" s="71"/>
+      <x:c r="D38" s="71"/>
+      <x:c r="E38" s="71"/>
+      <x:c r="F38" s="71"/>
+      <x:c r="G38" s="71"/>
+      <x:c r="H38" s="71"/>
+      <x:c r="I38" s="71"/>
+      <x:c r="J38" s="71"/>
+      <x:c r="K38" s="71"/>
+      <x:c r="L38" s="71"/>
+      <x:c r="M38" s="71"/>
+      <x:c r="N38" s="71"/>
+      <x:c r="O38" s="71"/>
+      <x:c r="P38" s="72" t="n">
         <x:f>'13-Week Forecast'!C$6</x:f>
         <x:v>46278</x:v>
       </x:c>
-      <x:c r="Q38" s="39" t="n">
+      <x:c r="Q38" s="74" t="n">
         <x:f>Q37+SUM('13-Week Forecast'!C10:C17)+IF('13-Week Forecast'!C$7="Actual",0,SUM('13-Week Forecast'!C10:C12)*('Assumptions'!$C$15-1))-(SUM('13-Week Forecast'!C22:C41)+IF('13-Week Forecast'!C$7="Actual",0,SUM('13-Week Forecast'!C22,'13-Week Forecast'!C31,'13-Week Forecast'!C33,'13-Week Forecast'!C41)*('Assumptions'!$D$15-1)))</x:f>
         <x:v>349000</x:v>
       </x:c>
-      <x:c r="R38" s="39" t="n">
+      <x:c r="R38" s="74" t="n">
         <x:f>R37+SUM('13-Week Forecast'!C10:C17)+IF('13-Week Forecast'!C$7="Actual",0,SUM('13-Week Forecast'!C10:C12)*('Assumptions'!$C$16-1))-(SUM('13-Week Forecast'!C22:C41)+IF('13-Week Forecast'!C$7="Actual",0,SUM('13-Week Forecast'!C22,'13-Week Forecast'!C31,'13-Week Forecast'!C33,'13-Week Forecast'!C41)*('Assumptions'!$D$16-1)))</x:f>
         <x:v>364380</x:v>
       </x:c>
-      <x:c r="S38" s="39" t="n">
+      <x:c r="S38" s="74" t="n">
         <x:f>S37+SUM('13-Week Forecast'!C10:C17)+IF('13-Week Forecast'!C$7="Actual",0,SUM('13-Week Forecast'!C10:C12)*('Assumptions'!$C$17-1))-(SUM('13-Week Forecast'!C22:C41)+IF('13-Week Forecast'!C$7="Actual",0,SUM('13-Week Forecast'!C22,'13-Week Forecast'!C31,'13-Week Forecast'!C33,'13-Week Forecast'!C41)*('Assumptions'!$D$17-1)))</x:f>
         <x:v>318800</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
-      <x:c r="P39" s="11" t="n">
+      <x:c r="A39" s="71"/>
+      <x:c r="B39" s="71"/>
+      <x:c r="C39" s="71"/>
+      <x:c r="D39" s="71"/>
+      <x:c r="E39" s="71"/>
+      <x:c r="F39" s="71"/>
+      <x:c r="G39" s="71"/>
+      <x:c r="H39" s="71"/>
+      <x:c r="I39" s="71"/>
+      <x:c r="J39" s="71"/>
+      <x:c r="K39" s="71"/>
+      <x:c r="L39" s="71"/>
+      <x:c r="M39" s="71"/>
+      <x:c r="N39" s="71"/>
+      <x:c r="O39" s="71"/>
+      <x:c r="P39" s="72" t="n">
         <x:f>'13-Week Forecast'!D$6</x:f>
         <x:v>46285</x:v>
       </x:c>
-      <x:c r="Q39" s="39" t="n">
+      <x:c r="Q39" s="74" t="n">
         <x:f>Q38+SUM('13-Week Forecast'!D10:D17)+IF('13-Week Forecast'!D$7="Actual",0,SUM('13-Week Forecast'!D10:D12)*('Assumptions'!$C$15-1))-(SUM('13-Week Forecast'!D22:D41)+IF('13-Week Forecast'!D$7="Actual",0,SUM('13-Week Forecast'!D22,'13-Week Forecast'!D31,'13-Week Forecast'!D33,'13-Week Forecast'!D41)*('Assumptions'!$D$15-1)))</x:f>
         <x:v>325000</x:v>
       </x:c>
-      <x:c r="R39" s="39" t="n">
+      <x:c r="R39" s="74" t="n">
         <x:f>R38+SUM('13-Week Forecast'!D10:D17)+IF('13-Week Forecast'!D$7="Actual",0,SUM('13-Week Forecast'!D10:D12)*('Assumptions'!$C$16-1))-(SUM('13-Week Forecast'!D22:D41)+IF('13-Week Forecast'!D$7="Actual",0,SUM('13-Week Forecast'!D22,'13-Week Forecast'!D31,'13-Week Forecast'!D33,'13-Week Forecast'!D41)*('Assumptions'!$D$16-1)))</x:f>
         <x:v>354920</x:v>
       </x:c>
-      <x:c r="S39" s="39" t="n">
+      <x:c r="S39" s="74" t="n">
         <x:f>S38+SUM('13-Week Forecast'!D10:D17)+IF('13-Week Forecast'!D$7="Actual",0,SUM('13-Week Forecast'!D10:D12)*('Assumptions'!$C$17-1))-(SUM('13-Week Forecast'!D22:D41)+IF('13-Week Forecast'!D$7="Actual",0,SUM('13-Week Forecast'!D22,'13-Week Forecast'!D31,'13-Week Forecast'!D33,'13-Week Forecast'!D41)*('Assumptions'!$D$17-1)))</x:f>
         <x:v>266150</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
-      <x:c r="P40" s="11" t="n">
+      <x:c r="A40" s="71"/>
+      <x:c r="B40" s="71"/>
+      <x:c r="C40" s="71"/>
+      <x:c r="D40" s="71"/>
+      <x:c r="E40" s="71"/>
+      <x:c r="F40" s="71"/>
+      <x:c r="G40" s="71"/>
+      <x:c r="H40" s="71"/>
+      <x:c r="I40" s="71"/>
+      <x:c r="J40" s="71"/>
+      <x:c r="K40" s="71"/>
+      <x:c r="L40" s="71"/>
+      <x:c r="M40" s="71"/>
+      <x:c r="N40" s="71"/>
+      <x:c r="O40" s="71"/>
+      <x:c r="P40" s="72" t="n">
         <x:f>'13-Week Forecast'!E$6</x:f>
         <x:v>46292</x:v>
       </x:c>
-      <x:c r="Q40" s="39" t="n">
+      <x:c r="Q40" s="74" t="n">
         <x:f>Q39+SUM('13-Week Forecast'!E10:E17)+IF('13-Week Forecast'!E$7="Actual",0,SUM('13-Week Forecast'!E10:E12)*('Assumptions'!$C$15-1))-(SUM('13-Week Forecast'!E22:E41)+IF('13-Week Forecast'!E$7="Actual",0,SUM('13-Week Forecast'!E22,'13-Week Forecast'!E31,'13-Week Forecast'!E33,'13-Week Forecast'!E41)*('Assumptions'!$D$15-1)))</x:f>
         <x:v>293000</x:v>
       </x:c>
-      <x:c r="R40" s="39" t="n">
+      <x:c r="R40" s="74" t="n">
         <x:f>R39+SUM('13-Week Forecast'!E10:E17)+IF('13-Week Forecast'!E$7="Actual",0,SUM('13-Week Forecast'!E10:E12)*('Assumptions'!$C$16-1))-(SUM('13-Week Forecast'!E22:E41)+IF('13-Week Forecast'!E$7="Actual",0,SUM('13-Week Forecast'!E22,'13-Week Forecast'!E31,'13-Week Forecast'!E33,'13-Week Forecast'!E41)*('Assumptions'!$D$16-1)))</x:f>
         <x:v>336680</x:v>
       </x:c>
-      <x:c r="S40" s="39" t="n">
+      <x:c r="S40" s="74" t="n">
         <x:f>S39+SUM('13-Week Forecast'!E10:E17)+IF('13-Week Forecast'!E$7="Actual",0,SUM('13-Week Forecast'!E10:E12)*('Assumptions'!$C$17-1))-(SUM('13-Week Forecast'!E22:E41)+IF('13-Week Forecast'!E$7="Actual",0,SUM('13-Week Forecast'!E22,'13-Week Forecast'!E31,'13-Week Forecast'!E33,'13-Week Forecast'!E41)*('Assumptions'!$D$17-1)))</x:f>
         <x:v>206900</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
-      <x:c r="P41" s="11" t="n">
+      <x:c r="A41" s="71"/>
+      <x:c r="B41" s="71"/>
+      <x:c r="C41" s="71"/>
+      <x:c r="D41" s="71"/>
+      <x:c r="E41" s="71"/>
+      <x:c r="F41" s="71"/>
+      <x:c r="G41" s="71"/>
+      <x:c r="H41" s="71"/>
+      <x:c r="I41" s="71"/>
+      <x:c r="J41" s="71"/>
+      <x:c r="K41" s="71"/>
+      <x:c r="L41" s="71"/>
+      <x:c r="M41" s="71"/>
+      <x:c r="N41" s="71"/>
+      <x:c r="O41" s="71"/>
+      <x:c r="P41" s="72" t="n">
         <x:f>'13-Week Forecast'!F$6</x:f>
         <x:v>46299</x:v>
       </x:c>
-      <x:c r="Q41" s="39" t="n">
+      <x:c r="Q41" s="74" t="n">
         <x:f>Q40+SUM('13-Week Forecast'!F10:F17)+IF('13-Week Forecast'!F$7="Actual",0,SUM('13-Week Forecast'!F10:F12)*('Assumptions'!$C$15-1))-(SUM('13-Week Forecast'!F22:F41)+IF('13-Week Forecast'!F$7="Actual",0,SUM('13-Week Forecast'!F22,'13-Week Forecast'!F31,'13-Week Forecast'!F33,'13-Week Forecast'!F41)*('Assumptions'!$D$15-1)))</x:f>
         <x:v>201000</x:v>
       </x:c>
-      <x:c r="R41" s="39" t="n">
+      <x:c r="R41" s="74" t="n">
         <x:f>R40+SUM('13-Week Forecast'!F10:F17)+IF('13-Week Forecast'!F$7="Actual",0,SUM('13-Week Forecast'!F10:F12)*('Assumptions'!$C$16-1))-(SUM('13-Week Forecast'!F22:F41)+IF('13-Week Forecast'!F$7="Actual",0,SUM('13-Week Forecast'!F22,'13-Week Forecast'!F31,'13-Week Forecast'!F33,'13-Week Forecast'!F41)*('Assumptions'!$D$16-1)))</x:f>
         <x:v>257940</x:v>
       </x:c>
-      <x:c r="S41" s="39" t="n">
+      <x:c r="S41" s="74" t="n">
         <x:f>S40+SUM('13-Week Forecast'!F10:F17)+IF('13-Week Forecast'!F$7="Actual",0,SUM('13-Week Forecast'!F10:F12)*('Assumptions'!$C$17-1))-(SUM('13-Week Forecast'!F22:F41)+IF('13-Week Forecast'!F$7="Actual",0,SUM('13-Week Forecast'!F22,'13-Week Forecast'!F31,'13-Week Forecast'!F33,'13-Week Forecast'!F41)*('Assumptions'!$D$17-1)))</x:f>
         <x:v>88550</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
-      <x:c r="P42" s="11" t="n">
+      <x:c r="A42" s="71"/>
+      <x:c r="B42" s="71"/>
+      <x:c r="C42" s="71"/>
+      <x:c r="D42" s="71"/>
+      <x:c r="E42" s="71"/>
+      <x:c r="F42" s="71"/>
+      <x:c r="G42" s="71"/>
+      <x:c r="H42" s="71"/>
+      <x:c r="I42" s="71"/>
+      <x:c r="J42" s="71"/>
+      <x:c r="K42" s="71"/>
+      <x:c r="L42" s="71"/>
+      <x:c r="M42" s="71"/>
+      <x:c r="N42" s="71"/>
+      <x:c r="O42" s="71"/>
+      <x:c r="P42" s="72" t="n">
         <x:f>'13-Week Forecast'!G$6</x:f>
         <x:v>46306</x:v>
       </x:c>
-      <x:c r="Q42" s="39" t="n">
+      <x:c r="Q42" s="74" t="n">
         <x:f>Q41+SUM('13-Week Forecast'!G10:G17)+IF('13-Week Forecast'!G$7="Actual",0,SUM('13-Week Forecast'!G10:G12)*('Assumptions'!$C$15-1))-(SUM('13-Week Forecast'!G22:G41)+IF('13-Week Forecast'!G$7="Actual",0,SUM('13-Week Forecast'!G22,'13-Week Forecast'!G31,'13-Week Forecast'!G33,'13-Week Forecast'!G41)*('Assumptions'!$D$15-1)))</x:f>
         <x:v>133000</x:v>
       </x:c>
-      <x:c r="R42" s="39" t="n">
+      <x:c r="R42" s="74" t="n">
         <x:f>R41+SUM('13-Week Forecast'!G10:G17)+IF('13-Week Forecast'!G$7="Actual",0,SUM('13-Week Forecast'!G10:G12)*('Assumptions'!$C$16-1))-(SUM('13-Week Forecast'!G22:G41)+IF('13-Week Forecast'!G$7="Actual",0,SUM('13-Week Forecast'!G22,'13-Week Forecast'!G31,'13-Week Forecast'!G33,'13-Week Forecast'!G41)*('Assumptions'!$D$16-1)))</x:f>
         <x:v>203320</x:v>
       </x:c>
-      <x:c r="S42" s="39" t="n">
+      <x:c r="S42" s="74" t="n">
         <x:f>S41+SUM('13-Week Forecast'!G10:G17)+IF('13-Week Forecast'!G$7="Actual",0,SUM('13-Week Forecast'!G10:G12)*('Assumptions'!$C$17-1))-(SUM('13-Week Forecast'!G22:G41)+IF('13-Week Forecast'!G$7="Actual",0,SUM('13-Week Forecast'!G22,'13-Week Forecast'!G31,'13-Week Forecast'!G33,'13-Week Forecast'!G41)*('Assumptions'!$D$17-1)))</x:f>
         <x:v>-6050</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
-      <x:c r="P43" s="11" t="n">
+      <x:c r="A43" s="71"/>
+      <x:c r="B43" s="71"/>
+      <x:c r="C43" s="71"/>
+      <x:c r="D43" s="71"/>
+      <x:c r="E43" s="71"/>
+      <x:c r="F43" s="71"/>
+      <x:c r="G43" s="71"/>
+      <x:c r="H43" s="71"/>
+      <x:c r="I43" s="71"/>
+      <x:c r="J43" s="71"/>
+      <x:c r="K43" s="71"/>
+      <x:c r="L43" s="71"/>
+      <x:c r="M43" s="71"/>
+      <x:c r="N43" s="71"/>
+      <x:c r="O43" s="71"/>
+      <x:c r="P43" s="72" t="n">
         <x:f>'13-Week Forecast'!H$6</x:f>
         <x:v>46313</x:v>
       </x:c>
-      <x:c r="Q43" s="39" t="n">
+      <x:c r="Q43" s="74" t="n">
         <x:f>Q42+SUM('13-Week Forecast'!H10:H17)+IF('13-Week Forecast'!H$7="Actual",0,SUM('13-Week Forecast'!H10:H12)*('Assumptions'!$C$15-1))-(SUM('13-Week Forecast'!H22:H41)+IF('13-Week Forecast'!H$7="Actual",0,SUM('13-Week Forecast'!H22,'13-Week Forecast'!H31,'13-Week Forecast'!H33,'13-Week Forecast'!H41)*('Assumptions'!$D$15-1)))</x:f>
         <x:v>217000</x:v>
       </x:c>
-      <x:c r="R43" s="39" t="n">
+      <x:c r="R43" s="74" t="n">
         <x:f>R42+SUM('13-Week Forecast'!H10:H17)+IF('13-Week Forecast'!H$7="Actual",0,SUM('13-Week Forecast'!H10:H12)*('Assumptions'!$C$16-1))-(SUM('13-Week Forecast'!H22:H41)+IF('13-Week Forecast'!H$7="Actual",0,SUM('13-Week Forecast'!H22,'13-Week Forecast'!H31,'13-Week Forecast'!H33,'13-Week Forecast'!H41)*('Assumptions'!$D$16-1)))</x:f>
         <x:v>300000</x:v>
       </x:c>
-      <x:c r="S43" s="39" t="n">
+      <x:c r="S43" s="74" t="n">
         <x:f>S42+SUM('13-Week Forecast'!H10:H17)+IF('13-Week Forecast'!H$7="Actual",0,SUM('13-Week Forecast'!H10:H12)*('Assumptions'!$C$17-1))-(SUM('13-Week Forecast'!H22:H41)+IF('13-Week Forecast'!H$7="Actual",0,SUM('13-Week Forecast'!H22,'13-Week Forecast'!H31,'13-Week Forecast'!H33,'13-Week Forecast'!H41)*('Assumptions'!$D$17-1)))</x:f>
         <x:v>52600</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
-      <x:c r="P44" s="11" t="n">
+      <x:c r="A44" s="71"/>
+      <x:c r="B44" s="71"/>
+      <x:c r="C44" s="71"/>
+      <x:c r="D44" s="71"/>
+      <x:c r="E44" s="71"/>
+      <x:c r="F44" s="71"/>
+      <x:c r="G44" s="71"/>
+      <x:c r="H44" s="71"/>
+      <x:c r="I44" s="71"/>
+      <x:c r="J44" s="71"/>
+      <x:c r="K44" s="71"/>
+      <x:c r="L44" s="71"/>
+      <x:c r="M44" s="71"/>
+      <x:c r="N44" s="71"/>
+      <x:c r="O44" s="71"/>
+      <x:c r="P44" s="72" t="n">
         <x:f>'13-Week Forecast'!I$6</x:f>
         <x:v>46320</x:v>
       </x:c>
-      <x:c r="Q44" s="39" t="n">
+      <x:c r="Q44" s="74" t="n">
         <x:f>Q43+SUM('13-Week Forecast'!I10:I17)+IF('13-Week Forecast'!I$7="Actual",0,SUM('13-Week Forecast'!I10:I12)*('Assumptions'!$C$15-1))-(SUM('13-Week Forecast'!I22:I41)+IF('13-Week Forecast'!I$7="Actual",0,SUM('13-Week Forecast'!I22,'13-Week Forecast'!I31,'13-Week Forecast'!I33,'13-Week Forecast'!I41)*('Assumptions'!$D$15-1)))</x:f>
         <x:v>160000</x:v>
       </x:c>
-      <x:c r="R44" s="39" t="n">
+      <x:c r="R44" s="74" t="n">
         <x:f>R43+SUM('13-Week Forecast'!I10:I17)+IF('13-Week Forecast'!I$7="Actual",0,SUM('13-Week Forecast'!I10:I12)*('Assumptions'!$C$16-1))-(SUM('13-Week Forecast'!I22:I41)+IF('13-Week Forecast'!I$7="Actual",0,SUM('13-Week Forecast'!I22,'13-Week Forecast'!I31,'13-Week Forecast'!I33,'13-Week Forecast'!I41)*('Assumptions'!$D$16-1)))</x:f>
         <x:v>256060</x:v>
       </x:c>
-      <x:c r="S44" s="39" t="n">
+      <x:c r="S44" s="74" t="n">
         <x:f>S43+SUM('13-Week Forecast'!I10:I17)+IF('13-Week Forecast'!I$7="Actual",0,SUM('13-Week Forecast'!I10:I12)*('Assumptions'!$C$17-1))-(SUM('13-Week Forecast'!I22:I41)+IF('13-Week Forecast'!I$7="Actual",0,SUM('13-Week Forecast'!I22,'13-Week Forecast'!I31,'13-Week Forecast'!I33,'13-Week Forecast'!I41)*('Assumptions'!$D$17-1)))</x:f>
         <x:v>-30500</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
-      <x:c r="P45" s="11" t="n">
+      <x:c r="A45" s="71"/>
+      <x:c r="B45" s="71"/>
+      <x:c r="C45" s="71"/>
+      <x:c r="D45" s="71"/>
+      <x:c r="E45" s="71"/>
+      <x:c r="F45" s="71"/>
+      <x:c r="G45" s="71"/>
+      <x:c r="H45" s="71"/>
+      <x:c r="I45" s="71"/>
+      <x:c r="J45" s="71"/>
+      <x:c r="K45" s="71"/>
+      <x:c r="L45" s="71"/>
+      <x:c r="M45" s="71"/>
+      <x:c r="N45" s="71"/>
+      <x:c r="O45" s="71"/>
+      <x:c r="P45" s="72" t="n">
         <x:f>'13-Week Forecast'!J$6</x:f>
         <x:v>46327</x:v>
       </x:c>
-      <x:c r="Q45" s="39" t="n">
+      <x:c r="Q45" s="74" t="n">
         <x:f>Q44+SUM('13-Week Forecast'!J10:J17)+IF('13-Week Forecast'!J$7="Actual",0,SUM('13-Week Forecast'!J10:J12)*('Assumptions'!$C$15-1))-(SUM('13-Week Forecast'!J22:J41)+IF('13-Week Forecast'!J$7="Actual",0,SUM('13-Week Forecast'!J22,'13-Week Forecast'!J31,'13-Week Forecast'!J33,'13-Week Forecast'!J41)*('Assumptions'!$D$15-1)))</x:f>
         <x:v>117000</x:v>
       </x:c>
-      <x:c r="R45" s="39" t="n">
+      <x:c r="R45" s="74" t="n">
         <x:f>R44+SUM('13-Week Forecast'!J10:J17)+IF('13-Week Forecast'!J$7="Actual",0,SUM('13-Week Forecast'!J10:J12)*('Assumptions'!$C$16-1))-(SUM('13-Week Forecast'!J22:J41)+IF('13-Week Forecast'!J$7="Actual",0,SUM('13-Week Forecast'!J22,'13-Week Forecast'!J31,'13-Week Forecast'!J33,'13-Week Forecast'!J41)*('Assumptions'!$D$16-1)))</x:f>
         <x:v>226480</x:v>
       </x:c>
-      <x:c r="S45" s="39" t="n">
+      <x:c r="S45" s="74" t="n">
         <x:f>S44+SUM('13-Week Forecast'!J10:J17)+IF('13-Week Forecast'!J$7="Actual",0,SUM('13-Week Forecast'!J10:J12)*('Assumptions'!$C$17-1))-(SUM('13-Week Forecast'!J22:J41)+IF('13-Week Forecast'!J$7="Actual",0,SUM('13-Week Forecast'!J22,'13-Week Forecast'!J31,'13-Week Forecast'!J33,'13-Week Forecast'!J41)*('Assumptions'!$D$17-1)))</x:f>
         <x:v>-100300</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
-      <x:c r="P46" s="11" t="n">
+      <x:c r="A46" s="71"/>
+      <x:c r="B46" s="71"/>
+      <x:c r="C46" s="71"/>
+      <x:c r="D46" s="71"/>
+      <x:c r="E46" s="71"/>
+      <x:c r="F46" s="71"/>
+      <x:c r="G46" s="71"/>
+      <x:c r="H46" s="71"/>
+      <x:c r="I46" s="71"/>
+      <x:c r="J46" s="71"/>
+      <x:c r="K46" s="71"/>
+      <x:c r="L46" s="71"/>
+      <x:c r="M46" s="71"/>
+      <x:c r="N46" s="71"/>
+      <x:c r="O46" s="71"/>
+      <x:c r="P46" s="72" t="n">
         <x:f>'13-Week Forecast'!K$6</x:f>
         <x:v>46334</x:v>
       </x:c>
-      <x:c r="Q46" s="39" t="n">
+      <x:c r="Q46" s="74" t="n">
         <x:f>Q45+SUM('13-Week Forecast'!K10:K17)+IF('13-Week Forecast'!K$7="Actual",0,SUM('13-Week Forecast'!K10:K12)*('Assumptions'!$C$15-1))-(SUM('13-Week Forecast'!K22:K41)+IF('13-Week Forecast'!K$7="Actual",0,SUM('13-Week Forecast'!K22,'13-Week Forecast'!K31,'13-Week Forecast'!K33,'13-Week Forecast'!K41)*('Assumptions'!$D$15-1)))</x:f>
         <x:v>137000</x:v>
       </x:c>
-      <x:c r="R46" s="39" t="n">
+      <x:c r="R46" s="74" t="n">
         <x:f>R45+SUM('13-Week Forecast'!K10:K17)+IF('13-Week Forecast'!K$7="Actual",0,SUM('13-Week Forecast'!K10:K12)*('Assumptions'!$C$16-1))-(SUM('13-Week Forecast'!K22:K41)+IF('13-Week Forecast'!K$7="Actual",0,SUM('13-Week Forecast'!K22,'13-Week Forecast'!K31,'13-Week Forecast'!K33,'13-Week Forecast'!K41)*('Assumptions'!$D$16-1)))</x:f>
         <x:v>260600</x:v>
       </x:c>
-      <x:c r="S46" s="39" t="n">
+      <x:c r="S46" s="74" t="n">
         <x:f>S45+SUM('13-Week Forecast'!K10:K17)+IF('13-Week Forecast'!K$7="Actual",0,SUM('13-Week Forecast'!K10:K12)*('Assumptions'!$C$17-1))-(SUM('13-Week Forecast'!K22:K41)+IF('13-Week Forecast'!K$7="Actual",0,SUM('13-Week Forecast'!K22,'13-Week Forecast'!K31,'13-Week Forecast'!K33,'13-Week Forecast'!K41)*('Assumptions'!$D$17-1)))</x:f>
         <x:v>-108350</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
-      <x:c r="P47" s="11" t="n">
+      <x:c r="A47" s="71"/>
+      <x:c r="B47" s="71"/>
+      <x:c r="C47" s="71"/>
+      <x:c r="D47" s="71"/>
+      <x:c r="E47" s="71"/>
+      <x:c r="F47" s="71"/>
+      <x:c r="G47" s="71"/>
+      <x:c r="H47" s="71"/>
+      <x:c r="I47" s="71"/>
+      <x:c r="J47" s="71"/>
+      <x:c r="K47" s="71"/>
+      <x:c r="L47" s="71"/>
+      <x:c r="M47" s="71"/>
+      <x:c r="N47" s="71"/>
+      <x:c r="O47" s="71"/>
+      <x:c r="P47" s="72" t="n">
         <x:f>'13-Week Forecast'!L$6</x:f>
         <x:v>46341</x:v>
       </x:c>
-      <x:c r="Q47" s="39" t="n">
+      <x:c r="Q47" s="74" t="n">
         <x:f>Q46+SUM('13-Week Forecast'!L10:L17)+IF('13-Week Forecast'!L$7="Actual",0,SUM('13-Week Forecast'!L10:L12)*('Assumptions'!$C$15-1))-(SUM('13-Week Forecast'!L22:L41)+IF('13-Week Forecast'!L$7="Actual",0,SUM('13-Week Forecast'!L22,'13-Week Forecast'!L31,'13-Week Forecast'!L33,'13-Week Forecast'!L41)*('Assumptions'!$D$15-1)))</x:f>
         <x:v>99000</x:v>
       </x:c>
-      <x:c r="R47" s="39" t="n">
+      <x:c r="R47" s="74" t="n">
         <x:f>R46+SUM('13-Week Forecast'!L10:L17)+IF('13-Week Forecast'!L$7="Actual",0,SUM('13-Week Forecast'!L10:L12)*('Assumptions'!$C$16-1))-(SUM('13-Week Forecast'!L22:L41)+IF('13-Week Forecast'!L$7="Actual",0,SUM('13-Week Forecast'!L22,'13-Week Forecast'!L31,'13-Week Forecast'!L33,'13-Week Forecast'!L41)*('Assumptions'!$D$16-1)))</x:f>
         <x:v>237020</x:v>
       </x:c>
-      <x:c r="S47" s="39" t="n">
+      <x:c r="S47" s="74" t="n">
         <x:f>S46+SUM('13-Week Forecast'!L10:L17)+IF('13-Week Forecast'!L$7="Actual",0,SUM('13-Week Forecast'!L10:L12)*('Assumptions'!$C$17-1))-(SUM('13-Week Forecast'!L22:L41)+IF('13-Week Forecast'!L$7="Actual",0,SUM('13-Week Forecast'!L22,'13-Week Forecast'!L31,'13-Week Forecast'!L33,'13-Week Forecast'!L41)*('Assumptions'!$D$17-1)))</x:f>
         <x:v>-174900</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
-      <x:c r="P48" s="11" t="n">
+      <x:c r="A48" s="71"/>
+      <x:c r="B48" s="71"/>
+      <x:c r="C48" s="71"/>
+      <x:c r="D48" s="71"/>
+      <x:c r="E48" s="71"/>
+      <x:c r="F48" s="71"/>
+      <x:c r="G48" s="71"/>
+      <x:c r="H48" s="71"/>
+      <x:c r="I48" s="71"/>
+      <x:c r="J48" s="71"/>
+      <x:c r="K48" s="71"/>
+      <x:c r="L48" s="71"/>
+      <x:c r="M48" s="71"/>
+      <x:c r="N48" s="71"/>
+      <x:c r="O48" s="71"/>
+      <x:c r="P48" s="72" t="n">
         <x:f>'13-Week Forecast'!M$6</x:f>
         <x:v>46348</x:v>
       </x:c>
-      <x:c r="Q48" s="39" t="n">
+      <x:c r="Q48" s="74" t="n">
         <x:f>Q47+SUM('13-Week Forecast'!M10:M17)+IF('13-Week Forecast'!M$7="Actual",0,SUM('13-Week Forecast'!M10:M12)*('Assumptions'!$C$15-1))-(SUM('13-Week Forecast'!M22:M41)+IF('13-Week Forecast'!M$7="Actual",0,SUM('13-Week Forecast'!M22,'13-Week Forecast'!M31,'13-Week Forecast'!M33,'13-Week Forecast'!M41)*('Assumptions'!$D$15-1)))</x:f>
         <x:v>82000</x:v>
       </x:c>
-      <x:c r="R48" s="39" t="n">
+      <x:c r="R48" s="74" t="n">
         <x:f>R47+SUM('13-Week Forecast'!M10:M17)+IF('13-Week Forecast'!M$7="Actual",0,SUM('13-Week Forecast'!M10:M12)*('Assumptions'!$C$16-1))-(SUM('13-Week Forecast'!M22:M41)+IF('13-Week Forecast'!M$7="Actual",0,SUM('13-Week Forecast'!M22,'13-Week Forecast'!M31,'13-Week Forecast'!M33,'13-Week Forecast'!M41)*('Assumptions'!$D$16-1)))</x:f>
         <x:v>234980</x:v>
       </x:c>
-      <x:c r="S48" s="39" t="n">
+      <x:c r="S48" s="74" t="n">
         <x:f>S47+SUM('13-Week Forecast'!M10:M17)+IF('13-Week Forecast'!M$7="Actual",0,SUM('13-Week Forecast'!M10:M12)*('Assumptions'!$C$17-1))-(SUM('13-Week Forecast'!M22:M41)+IF('13-Week Forecast'!M$7="Actual",0,SUM('13-Week Forecast'!M22,'13-Week Forecast'!M31,'13-Week Forecast'!M33,'13-Week Forecast'!M41)*('Assumptions'!$D$17-1)))</x:f>
         <x:v>-221400</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
-      <x:c r="P49" s="11" t="n">
+      <x:c r="A49" s="71"/>
+      <x:c r="B49" s="71"/>
+      <x:c r="C49" s="71"/>
+      <x:c r="D49" s="71"/>
+      <x:c r="E49" s="71"/>
+      <x:c r="F49" s="71"/>
+      <x:c r="G49" s="71"/>
+      <x:c r="H49" s="71"/>
+      <x:c r="I49" s="71"/>
+      <x:c r="J49" s="71"/>
+      <x:c r="K49" s="71"/>
+      <x:c r="L49" s="71"/>
+      <x:c r="M49" s="71"/>
+      <x:c r="N49" s="71"/>
+      <x:c r="O49" s="71"/>
+      <x:c r="P49" s="72" t="n">
         <x:f>'13-Week Forecast'!N$6</x:f>
         <x:v>46355</x:v>
       </x:c>
-      <x:c r="Q49" s="39" t="n">
+      <x:c r="Q49" s="74" t="n">
         <x:f>Q48+SUM('13-Week Forecast'!N10:N17)+IF('13-Week Forecast'!N$7="Actual",0,SUM('13-Week Forecast'!N10:N12)*('Assumptions'!$C$15-1))-(SUM('13-Week Forecast'!N22:N41)+IF('13-Week Forecast'!N$7="Actual",0,SUM('13-Week Forecast'!N22,'13-Week Forecast'!N31,'13-Week Forecast'!N33,'13-Week Forecast'!N41)*('Assumptions'!$D$15-1)))</x:f>
         <x:v>31000</x:v>
       </x:c>
-      <x:c r="R49" s="39" t="n">
+      <x:c r="R49" s="74" t="n">
         <x:f>R48+SUM('13-Week Forecast'!N10:N17)+IF('13-Week Forecast'!N$7="Actual",0,SUM('13-Week Forecast'!N10:N12)*('Assumptions'!$C$16-1))-(SUM('13-Week Forecast'!N22:N41)+IF('13-Week Forecast'!N$7="Actual",0,SUM('13-Week Forecast'!N22,'13-Week Forecast'!N31,'13-Week Forecast'!N33,'13-Week Forecast'!N41)*('Assumptions'!$D$16-1)))</x:f>
         <x:v>199320</x:v>
       </x:c>
-      <x:c r="S49" s="39" t="n">
+      <x:c r="S49" s="74" t="n">
         <x:f>S48+SUM('13-Week Forecast'!N10:N17)+IF('13-Week Forecast'!N$7="Actual",0,SUM('13-Week Forecast'!N10:N12)*('Assumptions'!$C$17-1))-(SUM('13-Week Forecast'!N22:N41)+IF('13-Week Forecast'!N$7="Actual",0,SUM('13-Week Forecast'!N22,'13-Week Forecast'!N31,'13-Week Forecast'!N33,'13-Week Forecast'!N41)*('Assumptions'!$D$17-1)))</x:f>
         <x:v>-302550</x:v>
       </x:c>
@@ -2740,7 +3518,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfed8bbef86874f97"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rca6d148ad5dd4b41"/>
 </x:worksheet>
 </file>
 
@@ -2776,6 +3554,14 @@
       <x:c r="E2" s="8"/>
       <x:c r="F2" s="8"/>
     </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="71"/>
+      <x:c r="B3" s="71"/>
+      <x:c r="C3" s="71"/>
+      <x:c r="D3" s="71"/>
+      <x:c r="E3" s="71"/>
+      <x:c r="F3" s="71"/>
+    </x:row>
     <x:row r="4">
       <x:c r="A4" s="14" t="str">
         <x:v>Core controls</x:v>
@@ -2783,70 +3569,114 @@
       <x:c r="B4" s="14" t="str">
         <x:v>Value</x:v>
       </x:c>
+      <x:c r="C4" s="71"/>
+      <x:c r="D4" s="71"/>
+      <x:c r="E4" s="71"/>
+      <x:c r="F4" s="71"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" t="str">
+      <x:c r="A5" s="71" t="str">
         <x:v>Business name</x:v>
       </x:c>
       <x:c r="B5" s="28" t="str">
         <x:v>Illustrative Australian business</x:v>
       </x:c>
+      <x:c r="C5" s="71"/>
+      <x:c r="D5" s="71"/>
+      <x:c r="E5" s="71"/>
+      <x:c r="F5" s="71"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" t="str">
+      <x:c r="A6" s="71" t="str">
         <x:v>Currency</x:v>
       </x:c>
       <x:c r="B6" s="28" t="str">
         <x:v>AUD</x:v>
       </x:c>
+      <x:c r="C6" s="71"/>
+      <x:c r="D6" s="71"/>
+      <x:c r="E6" s="71"/>
+      <x:c r="F6" s="71"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" t="str">
+      <x:c r="A7" s="71" t="str">
         <x:v>Units</x:v>
       </x:c>
       <x:c r="B7" s="28" t="str">
         <x:v>Whole dollars</x:v>
       </x:c>
+      <x:c r="C7" s="71"/>
+      <x:c r="D7" s="71"/>
+      <x:c r="E7" s="71"/>
+      <x:c r="F7" s="71"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" t="str">
+      <x:c r="A8" s="71" t="str">
         <x:v>Forecast start date</x:v>
       </x:c>
       <x:c r="B8" s="29" t="n">
         <x:v>46265</x:v>
       </x:c>
+      <x:c r="C8" s="71"/>
+      <x:c r="D8" s="71"/>
+      <x:c r="E8" s="71"/>
+      <x:c r="F8" s="71"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" t="str">
+      <x:c r="A9" s="71" t="str">
         <x:v>As-at date</x:v>
       </x:c>
       <x:c r="B9" s="29" t="n">
         <x:v>46271</x:v>
       </x:c>
+      <x:c r="C9" s="71"/>
+      <x:c r="D9" s="71"/>
+      <x:c r="E9" s="71"/>
+      <x:c r="F9" s="71"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" t="str">
+      <x:c r="A10" s="71" t="str">
         <x:v>Opening cash</x:v>
       </x:c>
       <x:c r="B10" s="30" t="n">
         <x:v>400000</x:v>
       </x:c>
+      <x:c r="C10" s="71"/>
+      <x:c r="D10" s="71"/>
+      <x:c r="E10" s="71"/>
+      <x:c r="F10" s="71"/>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" t="str">
+      <x:c r="A11" s="71" t="str">
         <x:v>Minimum cash buffer</x:v>
       </x:c>
       <x:c r="B11" s="30" t="n">
         <x:v>100000</x:v>
       </x:c>
+      <x:c r="C11" s="71"/>
+      <x:c r="D11" s="71"/>
+      <x:c r="E11" s="71"/>
+      <x:c r="F11" s="71"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" t="str">
+      <x:c r="A12" s="71" t="str">
         <x:v>Selected scenario</x:v>
       </x:c>
       <x:c r="B12" s="28" t="str">
         <x:v>Base</x:v>
       </x:c>
+      <x:c r="C12" s="71"/>
+      <x:c r="D12" s="71"/>
+      <x:c r="E12" s="71"/>
+      <x:c r="F12" s="71"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="71"/>
+      <x:c r="B13" s="71"/>
+      <x:c r="C13" s="71"/>
+      <x:c r="D13" s="71"/>
+      <x:c r="E13" s="71"/>
+      <x:c r="F13" s="71"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="14" t="str">
@@ -2864,8 +3694,10 @@
       <x:c r="E14" s="14" t="str">
         <x:v>Description</x:v>
       </x:c>
+      <x:c r="F14" s="71"/>
     </x:row>
     <x:row r="15">
+      <x:c r="A15" s="71"/>
       <x:c r="B15" s="16" t="str">
         <x:v>Base</x:v>
       </x:c>
@@ -2878,8 +3710,10 @@
       <x:c r="E15" s="16" t="str">
         <x:v>Current operating expectation</x:v>
       </x:c>
+      <x:c r="F15" s="71"/>
     </x:row>
     <x:row r="16">
+      <x:c r="A16" s="71"/>
       <x:c r="B16" s="16" t="str">
         <x:v>Upside</x:v>
       </x:c>
@@ -2892,8 +3726,10 @@
       <x:c r="E16" s="16" t="str">
         <x:v>Stronger receipts and lower selected variable payments</x:v>
       </x:c>
+      <x:c r="F16" s="71"/>
     </x:row>
     <x:row r="17">
+      <x:c r="A17" s="71"/>
       <x:c r="B17" s="16" t="str">
         <x:v>Downside</x:v>
       </x:c>
@@ -2906,14 +3742,27 @@
       <x:c r="E17" s="16" t="str">
         <x:v>Softer receipts and higher selected variable payments</x:v>
       </x:c>
+      <x:c r="F17" s="71"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="71"/>
+      <x:c r="B18" s="71"/>
+      <x:c r="C18" s="71"/>
+      <x:c r="D18" s="71"/>
+      <x:c r="E18" s="71"/>
+      <x:c r="F18" s="71"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" t="str">
+      <x:c r="A19" s="71" t="str">
         <x:v>Liquidity action lead time (weeks)</x:v>
       </x:c>
       <x:c r="B19" s="32" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="C19" s="71"/>
+      <x:c r="D19" s="71"/>
+      <x:c r="E19" s="71"/>
+      <x:c r="F19" s="71"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="14" t="str">
@@ -3030,8 +3879,42 @@
       <x:c r="N2" s="8"/>
       <x:c r="O2" s="8"/>
     </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="71"/>
+      <x:c r="B3" s="71"/>
+      <x:c r="C3" s="71"/>
+      <x:c r="D3" s="71"/>
+      <x:c r="E3" s="71"/>
+      <x:c r="F3" s="71"/>
+      <x:c r="G3" s="71"/>
+      <x:c r="H3" s="71"/>
+      <x:c r="I3" s="71"/>
+      <x:c r="J3" s="71"/>
+      <x:c r="K3" s="71"/>
+      <x:c r="L3" s="71"/>
+      <x:c r="M3" s="71"/>
+      <x:c r="N3" s="71"/>
+      <x:c r="O3" s="71"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="71"/>
+      <x:c r="B4" s="71"/>
+      <x:c r="C4" s="71"/>
+      <x:c r="D4" s="71"/>
+      <x:c r="E4" s="71"/>
+      <x:c r="F4" s="71"/>
+      <x:c r="G4" s="71"/>
+      <x:c r="H4" s="71"/>
+      <x:c r="I4" s="71"/>
+      <x:c r="J4" s="71"/>
+      <x:c r="K4" s="71"/>
+      <x:c r="L4" s="71"/>
+      <x:c r="M4" s="71"/>
+      <x:c r="N4" s="71"/>
+      <x:c r="O4" s="71"/>
+    </x:row>
     <x:row r="5">
-      <x:c r="A5" t="str">
+      <x:c r="A5" s="71" t="str">
         <x:v>Week commencing</x:v>
       </x:c>
       <x:c r="B5" s="34" t="n">
@@ -3086,12 +3969,12 @@
         <x:f>M5+7</x:f>
         <x:v>46349</x:v>
       </x:c>
-      <x:c r="O5" t="str">
+      <x:c r="O5" s="71" t="str">
         <x:v>13-week total / terminal</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" t="str">
+      <x:c r="A6" s="71" t="str">
         <x:v>Week ending</x:v>
       </x:c>
       <x:c r="B6" s="34" t="n">
@@ -3146,12 +4029,12 @@
         <x:f>N5+6</x:f>
         <x:v>46355</x:v>
       </x:c>
-      <x:c r="O6" t="str">
+      <x:c r="O6" s="71" t="str">
         <x:v>Week 13 value</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" t="str">
+      <x:c r="A7" s="71" t="str">
         <x:v>Actual / Forecast</x:v>
       </x:c>
       <x:c r="B7" s="35" t="str">
@@ -3206,7 +4089,24 @@
         <x:f>IF(N6&lt;='Assumptions'!$B$9,"Actual","Forecast")</x:f>
         <x:v>Forecast</x:v>
       </x:c>
-      <x:c r="O7" t="str"/>
+      <x:c r="O7" s="71" t="str"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="71"/>
+      <x:c r="B8" s="71"/>
+      <x:c r="C8" s="71"/>
+      <x:c r="D8" s="71"/>
+      <x:c r="E8" s="71"/>
+      <x:c r="F8" s="71"/>
+      <x:c r="G8" s="71"/>
+      <x:c r="H8" s="71"/>
+      <x:c r="I8" s="71"/>
+      <x:c r="J8" s="71"/>
+      <x:c r="K8" s="71"/>
+      <x:c r="L8" s="71"/>
+      <x:c r="M8" s="71"/>
+      <x:c r="N8" s="71"/>
+      <x:c r="O8" s="71"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="14" t="str">
@@ -3228,7 +4128,7 @@
       <x:c r="O9" s="14"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" t="str">
+      <x:c r="A10" s="71" t="str">
         <x:v>Customer receipts</x:v>
       </x:c>
       <x:c r="B10" s="38" t="n">
@@ -3270,13 +4170,13 @@
       <x:c r="N10" s="38" t="n">
         <x:v>130000</x:v>
       </x:c>
-      <x:c r="O10" s="39" t="n">
+      <x:c r="O10" s="74" t="n">
         <x:f>SUM(B10:N10)</x:f>
         <x:v>1514000</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" t="str">
+      <x:c r="A11" s="71" t="str">
         <x:v>Overdue receipts</x:v>
       </x:c>
       <x:c r="B11" s="38" t="n">
@@ -3318,13 +4218,13 @@
       <x:c r="N11" s="38" t="n">
         <x:v>12000</x:v>
       </x:c>
-      <x:c r="O11" s="39" t="n">
+      <x:c r="O11" s="74" t="n">
         <x:f>SUM(B11:N11)</x:f>
         <x:v>152000</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" t="str">
+      <x:c r="A12" s="71" t="str">
         <x:v>Cash / EFTPOS sales</x:v>
       </x:c>
       <x:c r="B12" s="38" t="n">
@@ -3366,13 +4266,13 @@
       <x:c r="N12" s="38" t="n">
         <x:v>22000</x:v>
       </x:c>
-      <x:c r="O12" s="39" t="n">
+      <x:c r="O12" s="74" t="n">
         <x:f>SUM(B12:N12)</x:f>
         <x:v>245000</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" t="str">
+      <x:c r="A13" s="71" t="str">
         <x:v>GST refunds / credits</x:v>
       </x:c>
       <x:c r="B13" s="38" t="n">
@@ -3414,13 +4314,13 @@
       <x:c r="N13" s="38" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="O13" s="39" t="n">
+      <x:c r="O13" s="74" t="n">
         <x:f>SUM(B13:N13)</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" t="str">
+      <x:c r="A14" s="71" t="str">
         <x:v>Other operating</x:v>
       </x:c>
       <x:c r="B14" s="38" t="n">
@@ -3462,13 +4362,13 @@
       <x:c r="N14" s="38" t="n">
         <x:v>4000</x:v>
       </x:c>
-      <x:c r="O14" s="39" t="n">
+      <x:c r="O14" s="74" t="n">
         <x:f>SUM(B14:N14)</x:f>
         <x:v>52000</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" t="str">
+      <x:c r="A15" s="71" t="str">
         <x:v>Asset sale proceeds</x:v>
       </x:c>
       <x:c r="B15" s="38" t="n">
@@ -3510,13 +4410,13 @@
       <x:c r="N15" s="38" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="O15" s="39" t="n">
+      <x:c r="O15" s="74" t="n">
         <x:f>SUM(B15:N15)</x:f>
         <x:v>100000</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" t="str">
+      <x:c r="A16" s="71" t="str">
         <x:v>Equity / owner funding</x:v>
       </x:c>
       <x:c r="B16" s="38" t="n">
@@ -3558,13 +4458,13 @@
       <x:c r="N16" s="38" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="O16" s="39" t="n">
+      <x:c r="O16" s="74" t="n">
         <x:f>SUM(B16:N16)</x:f>
         <x:v>150000</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" t="str">
+      <x:c r="A17" s="71" t="str">
         <x:v>Loan proceeds</x:v>
       </x:c>
       <x:c r="B17" s="38" t="n">
@@ -3606,13 +4506,13 @@
       <x:c r="N17" s="38" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="O17" s="39" t="n">
+      <x:c r="O17" s="74" t="n">
         <x:f>SUM(B17:N17)</x:f>
         <x:v>125000</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" t="str">
+      <x:c r="A18" s="71" t="str">
         <x:v>Scenario receipt adjustment</x:v>
       </x:c>
       <x:c r="B18" s="42" t="n">
@@ -3667,7 +4567,7 @@
         <x:f>IF(N$7="Actual",0,SUM(N10:N12)*(INDEX(Assumptions!$C$15:$C$17,MATCH(Assumptions!$B$12,Assumptions!$B$15:$B$17,0))-1))</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="O18" s="39" t="n">
+      <x:c r="O18" s="74" t="n">
         <x:f>SUM(B18:N18)</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -3734,20 +4634,21 @@
       </x:c>
     </x:row>
     <x:row r="20">
-      <x:c r="B20" s="39"/>
-      <x:c r="C20" s="39"/>
-      <x:c r="D20" s="39"/>
-      <x:c r="E20" s="39"/>
-      <x:c r="F20" s="39"/>
-      <x:c r="G20" s="39"/>
-      <x:c r="H20" s="39"/>
-      <x:c r="I20" s="39"/>
-      <x:c r="J20" s="39"/>
-      <x:c r="K20" s="39"/>
-      <x:c r="L20" s="39"/>
-      <x:c r="M20" s="39"/>
-      <x:c r="N20" s="39"/>
-      <x:c r="O20" s="39"/>
+      <x:c r="A20" s="71"/>
+      <x:c r="B20" s="74"/>
+      <x:c r="C20" s="74"/>
+      <x:c r="D20" s="74"/>
+      <x:c r="E20" s="74"/>
+      <x:c r="F20" s="74"/>
+      <x:c r="G20" s="74"/>
+      <x:c r="H20" s="74"/>
+      <x:c r="I20" s="74"/>
+      <x:c r="J20" s="74"/>
+      <x:c r="K20" s="74"/>
+      <x:c r="L20" s="74"/>
+      <x:c r="M20" s="74"/>
+      <x:c r="N20" s="74"/>
+      <x:c r="O20" s="74"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="14" t="str">
@@ -3769,7 +4670,7 @@
       <x:c r="O21" s="41"/>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" t="str">
+      <x:c r="A22" s="71" t="str">
         <x:v>Suppliers and inventory</x:v>
       </x:c>
       <x:c r="B22" s="38" t="n">
@@ -3811,13 +4712,13 @@
       <x:c r="N22" s="38" t="n">
         <x:v>90000</x:v>
       </x:c>
-      <x:c r="O22" s="39" t="n">
+      <x:c r="O22" s="74" t="n">
         <x:f>SUM(B22:N22)</x:f>
         <x:v>1266000</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" t="str">
+      <x:c r="A23" s="71" t="str">
         <x:v>Net wages</x:v>
       </x:c>
       <x:c r="B23" s="38" t="n">
@@ -3859,13 +4760,13 @@
       <x:c r="N23" s="38" t="n">
         <x:v>42000</x:v>
       </x:c>
-      <x:c r="O23" s="39" t="n">
+      <x:c r="O23" s="74" t="n">
         <x:f>SUM(B23:N23)</x:f>
         <x:v>546000</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" t="str">
+      <x:c r="A24" s="71" t="str">
         <x:v>PAYG withholding</x:v>
       </x:c>
       <x:c r="B24" s="38" t="n">
@@ -3907,13 +4808,13 @@
       <x:c r="N24" s="38" t="n">
         <x:v>12000</x:v>
       </x:c>
-      <x:c r="O24" s="39" t="n">
+      <x:c r="O24" s="74" t="n">
         <x:f>SUM(B24:N24)</x:f>
         <x:v>156000</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" t="str">
+      <x:c r="A25" s="71" t="str">
         <x:v>Superannuation</x:v>
       </x:c>
       <x:c r="B25" s="38" t="n">
@@ -3955,13 +4856,13 @@
       <x:c r="N25" s="38" t="n">
         <x:v>6000</x:v>
       </x:c>
-      <x:c r="O25" s="39" t="n">
+      <x:c r="O25" s="74" t="n">
         <x:f>SUM(B25:N25)</x:f>
         <x:v>78000</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" t="str">
+      <x:c r="A26" s="71" t="str">
         <x:v>Payroll tax / workers compensation</x:v>
       </x:c>
       <x:c r="B26" s="38" t="n">
@@ -4003,13 +4904,13 @@
       <x:c r="N26" s="38" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="O26" s="39" t="n">
+      <x:c r="O26" s="74" t="n">
         <x:f>SUM(B26:N26)</x:f>
         <x:v>15000</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" t="str">
+      <x:c r="A27" s="71" t="str">
         <x:v>Rent</x:v>
       </x:c>
       <x:c r="B27" s="38" t="n">
@@ -4051,13 +4952,13 @@
       <x:c r="N27" s="38" t="n">
         <x:v>25000</x:v>
       </x:c>
-      <x:c r="O27" s="39" t="n">
+      <x:c r="O27" s="74" t="n">
         <x:f>SUM(B27:N27)</x:f>
         <x:v>100000</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" t="str">
+      <x:c r="A28" s="71" t="str">
         <x:v>Utilities</x:v>
       </x:c>
       <x:c r="B28" s="38" t="n">
@@ -4099,13 +5000,13 @@
       <x:c r="N28" s="38" t="n">
         <x:v>4000</x:v>
       </x:c>
-      <x:c r="O28" s="39" t="n">
+      <x:c r="O28" s="74" t="n">
         <x:f>SUM(B28:N28)</x:f>
         <x:v>12000</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" t="str">
+      <x:c r="A29" s="71" t="str">
         <x:v>Insurance</x:v>
       </x:c>
       <x:c r="B29" s="38" t="n">
@@ -4147,13 +5048,13 @@
       <x:c r="N29" s="38" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="O29" s="39" t="n">
+      <x:c r="O29" s="74" t="n">
         <x:f>SUM(B29:N29)</x:f>
         <x:v>6000</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" t="str">
+      <x:c r="A30" s="71" t="str">
         <x:v>Software and subscriptions</x:v>
       </x:c>
       <x:c r="B30" s="38" t="n">
@@ -4195,13 +5096,13 @@
       <x:c r="N30" s="38" t="n">
         <x:v>3000</x:v>
       </x:c>
-      <x:c r="O30" s="39" t="n">
+      <x:c r="O30" s="74" t="n">
         <x:f>SUM(B30:N30)</x:f>
         <x:v>39000</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" t="str">
+      <x:c r="A31" s="71" t="str">
         <x:v>Marketing</x:v>
       </x:c>
       <x:c r="B31" s="38" t="n">
@@ -4243,13 +5144,13 @@
       <x:c r="N31" s="38" t="n">
         <x:v>6000</x:v>
       </x:c>
-      <x:c r="O31" s="39" t="n">
+      <x:c r="O31" s="74" t="n">
         <x:f>SUM(B31:N31)</x:f>
         <x:v>78000</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" t="str">
+      <x:c r="A32" s="71" t="str">
         <x:v>Professional services</x:v>
       </x:c>
       <x:c r="B32" s="38" t="n">
@@ -4291,13 +5192,13 @@
       <x:c r="N32" s="38" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="O32" s="39" t="n">
+      <x:c r="O32" s="74" t="n">
         <x:f>SUM(B32:N32)</x:f>
         <x:v>24000</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" t="str">
+      <x:c r="A33" s="71" t="str">
         <x:v>Freight, vehicles and travel</x:v>
       </x:c>
       <x:c r="B33" s="38" t="n">
@@ -4339,13 +5240,13 @@
       <x:c r="N33" s="38" t="n">
         <x:v>10000</x:v>
       </x:c>
-      <x:c r="O33" s="39" t="n">
+      <x:c r="O33" s="74" t="n">
         <x:f>SUM(B33:N33)</x:f>
         <x:v>130000</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
-      <x:c r="A34" t="str">
+      <x:c r="A34" s="71" t="str">
         <x:v>GST / BAS payments</x:v>
       </x:c>
       <x:c r="B34" s="38" t="n">
@@ -4387,13 +5288,13 @@
       <x:c r="N34" s="38" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="O34" s="39" t="n">
+      <x:c r="O34" s="74" t="n">
         <x:f>SUM(B34:N34)</x:f>
         <x:v>45000</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
-      <x:c r="A35" t="str">
+      <x:c r="A35" s="71" t="str">
         <x:v>PAYG income tax instalments</x:v>
       </x:c>
       <x:c r="B35" s="38" t="n">
@@ -4435,13 +5336,13 @@
       <x:c r="N35" s="38" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="O35" s="39" t="n">
+      <x:c r="O35" s="74" t="n">
         <x:f>SUM(B35:N35)</x:f>
         <x:v>18000</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" t="str">
+      <x:c r="A36" s="71" t="str">
         <x:v>FBT / other tax</x:v>
       </x:c>
       <x:c r="B36" s="38" t="n">
@@ -4483,13 +5384,13 @@
       <x:c r="N36" s="38" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="O36" s="39" t="n">
+      <x:c r="O36" s="74" t="n">
         <x:f>SUM(B36:N36)</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
-      <x:c r="A37" t="str">
+      <x:c r="A37" s="71" t="str">
         <x:v>Interest and bank fees</x:v>
       </x:c>
       <x:c r="B37" s="38" t="n">
@@ -4531,13 +5432,13 @@
       <x:c r="N37" s="38" t="n">
         <x:v>4000</x:v>
       </x:c>
-      <x:c r="O37" s="39" t="n">
+      <x:c r="O37" s="74" t="n">
         <x:f>SUM(B37:N37)</x:f>
         <x:v>16000</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
-      <x:c r="A38" t="str">
+      <x:c r="A38" s="71" t="str">
         <x:v>Loan principal</x:v>
       </x:c>
       <x:c r="B38" s="38" t="n">
@@ -4579,13 +5480,13 @@
       <x:c r="N38" s="38" t="n">
         <x:v>12000</x:v>
       </x:c>
-      <x:c r="O38" s="39" t="n">
+      <x:c r="O38" s="74" t="n">
         <x:f>SUM(B38:N38)</x:f>
         <x:v>48000</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
-      <x:c r="A39" t="str">
+      <x:c r="A39" s="71" t="str">
         <x:v>Capital expenditure</x:v>
       </x:c>
       <x:c r="B39" s="38" t="n">
@@ -4627,13 +5528,13 @@
       <x:c r="N39" s="38" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="O39" s="39" t="n">
+      <x:c r="O39" s="74" t="n">
         <x:f>SUM(B39:N39)</x:f>
         <x:v>65000</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
-      <x:c r="A40" t="str">
+      <x:c r="A40" s="71" t="str">
         <x:v>Dividends / distributions</x:v>
       </x:c>
       <x:c r="B40" s="38" t="n">
@@ -4675,13 +5576,13 @@
       <x:c r="N40" s="38" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="O40" s="39" t="n">
+      <x:c r="O40" s="74" t="n">
         <x:f>SUM(B40:N40)</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
-      <x:c r="A41" t="str">
+      <x:c r="A41" s="71" t="str">
         <x:v>Other operating</x:v>
       </x:c>
       <x:c r="B41" s="38" t="n">
@@ -4723,13 +5624,13 @@
       <x:c r="N41" s="38" t="n">
         <x:v>5000</x:v>
       </x:c>
-      <x:c r="O41" s="39" t="n">
+      <x:c r="O41" s="74" t="n">
         <x:f>SUM(B41:N41)</x:f>
         <x:v>65000</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
-      <x:c r="A42" t="str">
+      <x:c r="A42" s="71" t="str">
         <x:v>Scenario payment adjustment</x:v>
       </x:c>
       <x:c r="B42" s="42" t="n">
@@ -4784,7 +5685,7 @@
         <x:f>IF(N$7="Actual",0,SUM(N22,N31,N33,N41)*(INDEX(Assumptions!$D$15:$D$17,MATCH(Assumptions!$B$12,Assumptions!$B$15:$B$17,0))-1))</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="O42" s="39" t="n">
+      <x:c r="O42" s="74" t="n">
         <x:f>SUM(B42:N42)</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -4851,20 +5752,21 @@
       </x:c>
     </x:row>
     <x:row r="44">
-      <x:c r="B44" s="39"/>
-      <x:c r="C44" s="39"/>
-      <x:c r="D44" s="39"/>
-      <x:c r="E44" s="39"/>
-      <x:c r="F44" s="39"/>
-      <x:c r="G44" s="39"/>
-      <x:c r="H44" s="39"/>
-      <x:c r="I44" s="39"/>
-      <x:c r="J44" s="39"/>
-      <x:c r="K44" s="39"/>
-      <x:c r="L44" s="39"/>
-      <x:c r="M44" s="39"/>
-      <x:c r="N44" s="39"/>
-      <x:c r="O44" s="39"/>
+      <x:c r="A44" s="71"/>
+      <x:c r="B44" s="74"/>
+      <x:c r="C44" s="74"/>
+      <x:c r="D44" s="74"/>
+      <x:c r="E44" s="74"/>
+      <x:c r="F44" s="74"/>
+      <x:c r="G44" s="74"/>
+      <x:c r="H44" s="74"/>
+      <x:c r="I44" s="74"/>
+      <x:c r="J44" s="74"/>
+      <x:c r="K44" s="74"/>
+      <x:c r="L44" s="74"/>
+      <x:c r="M44" s="74"/>
+      <x:c r="N44" s="74"/>
+      <x:c r="O44" s="74"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="14" t="str">
@@ -4886,7 +5788,7 @@
       <x:c r="O45" s="41"/>
     </x:row>
     <x:row r="46">
-      <x:c r="A46" t="str">
+      <x:c r="A46" s="71" t="str">
         <x:v>Opening cash balance</x:v>
       </x:c>
       <x:c r="B46" s="44" t="n">
@@ -4941,13 +5843,13 @@
         <x:f>M48</x:f>
         <x:v>82000</x:v>
       </x:c>
-      <x:c r="O46" s="39" t="n">
+      <x:c r="O46" s="74" t="n">
         <x:f>N46</x:f>
         <x:v>82000</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
-      <x:c r="A47" t="str">
+      <x:c r="A47" s="71" t="str">
         <x:v>Net cash movement</x:v>
       </x:c>
       <x:c r="B47" s="42" t="n">
@@ -5002,7 +5904,7 @@
         <x:f>N19-N43</x:f>
         <x:v>-51000</x:v>
       </x:c>
-      <x:c r="O47" s="39" t="n">
+      <x:c r="O47" s="74" t="n">
         <x:f>SUM(B47:N47)</x:f>
         <x:v>-369000</x:v>
       </x:c>
@@ -5069,7 +5971,7 @@
       </x:c>
     </x:row>
     <x:row r="49">
-      <x:c r="A49" t="str">
+      <x:c r="A49" s="71" t="str">
         <x:v>Minimum cash buffer</x:v>
       </x:c>
       <x:c r="B49" s="44" t="n">
@@ -5124,7 +6026,7 @@
         <x:f>'Assumptions'!$B$11</x:f>
         <x:v>100000</x:v>
       </x:c>
-      <x:c r="O49" s="39" t="n">
+      <x:c r="O49" s="74" t="n">
         <x:f>N49</x:f>
         <x:v>100000</x:v>
       </x:c>
@@ -5191,7 +6093,7 @@
       </x:c>
     </x:row>
     <x:row r="51">
-      <x:c r="A51" t="str">
+      <x:c r="A51" s="71" t="str">
         <x:v>Liquidity status</x:v>
       </x:c>
       <x:c r="B51" s="17" t="str">
@@ -5246,7 +6148,7 @@
         <x:f>IF(N48&lt;N49,"BELOW BUFFER",IF(N48&lt;=N49*1.25,"WATCH","OK"))</x:f>
         <x:v>BELOW BUFFER</x:v>
       </x:c>
-      <x:c r="O51" t="str">
+      <x:c r="O51" s="71" t="str">
         <x:f>N51</x:f>
         <x:v>BELOW BUFFER</x:v>
       </x:c>
@@ -5268,7 +6170,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb3415d0a01b41c9"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62ee5fc974354fc5"/>
 </x:worksheet>
 </file>
 
@@ -5327,6 +6229,22 @@
       <x:c r="L2" s="8"/>
       <x:c r="M2" s="8"/>
       <x:c r="N2" s="8"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="71"/>
+      <x:c r="B3" s="71"/>
+      <x:c r="C3" s="71"/>
+      <x:c r="D3" s="71"/>
+      <x:c r="E3" s="71"/>
+      <x:c r="F3" s="71"/>
+      <x:c r="G3" s="71"/>
+      <x:c r="H3" s="71"/>
+      <x:c r="I3" s="71"/>
+      <x:c r="J3" s="71"/>
+      <x:c r="K3" s="71"/>
+      <x:c r="L3" s="71"/>
+      <x:c r="M3" s="71"/>
+      <x:c r="N3" s="71"/>
     </x:row>
     <x:row r="4" ht="34" customHeight="1">
       <x:c r="A4" s="27" t="str">
@@ -5946,6 +6864,16 @@
       <x:c r="G2" s="8"/>
       <x:c r="H2" s="8"/>
     </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="71"/>
+      <x:c r="B3" s="71"/>
+      <x:c r="C3" s="71"/>
+      <x:c r="D3" s="71"/>
+      <x:c r="E3" s="71"/>
+      <x:c r="F3" s="71"/>
+      <x:c r="G3" s="71"/>
+      <x:c r="H3" s="71"/>
+    </x:row>
     <x:row r="4">
       <x:c r="A4" s="51" t="str">
         <x:v>MODEL STATUS</x:v>
@@ -5962,6 +6890,29 @@
         <x:f>IF(COUNTIF('13-Week Forecast'!$B$51:$N$51,"BELOW BUFFER")&gt;0,"ACTION REQUIRED",IF(COUNTIF('13-Week Forecast'!$B$51:$N$51,"WATCH")&gt;0,"WATCH","OK"))</x:f>
         <x:v>ACTION REQUIRED</x:v>
       </x:c>
+      <x:c r="F4" s="71"/>
+      <x:c r="G4" s="71"/>
+      <x:c r="H4" s="71"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="71"/>
+      <x:c r="B5" s="71"/>
+      <x:c r="C5" s="71"/>
+      <x:c r="D5" s="71"/>
+      <x:c r="E5" s="71"/>
+      <x:c r="F5" s="71"/>
+      <x:c r="G5" s="71"/>
+      <x:c r="H5" s="71"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="71"/>
+      <x:c r="B6" s="71"/>
+      <x:c r="C6" s="71"/>
+      <x:c r="D6" s="71"/>
+      <x:c r="E6" s="71"/>
+      <x:c r="F6" s="71"/>
+      <x:c r="G6" s="71"/>
+      <x:c r="H6" s="71"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="14" t="str">
@@ -5990,274 +6941,314 @@
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="15" t="str">
+      <x:c r="A8" s="73" t="str">
         <x:v>Exactly 13 forecast weeks</x:v>
       </x:c>
-      <x:c r="B8" s="52" t="n">
+      <x:c r="B8" s="75" t="n">
         <x:f>COLUMNS('13-Week Forecast'!$B$5:$N$5)</x:f>
         <x:v>13</x:v>
       </x:c>
-      <x:c r="C8" s="52" t="n">
+      <x:c r="C8" s="75" t="n">
         <x:f>13</x:f>
         <x:v>13</x:v>
       </x:c>
-      <x:c r="D8" s="52" t="n">
+      <x:c r="D8" s="75" t="n">
         <x:f>B8-C8</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E8" s="52" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F8" s="15" t="str">
+      <x:c r="E8" s="75" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F8" s="73" t="str">
         <x:f>IF(ABS(D8)&lt;=E8,"PASS","FAIL")</x:f>
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="G8" s="15" t="str">
+      <x:c r="G8" s="73" t="str">
         <x:v>13-Week Forecast!B5:N5</x:v>
       </x:c>
-      <x:c r="H8" s="15" t="str">
+      <x:c r="H8" s="73" t="str">
         <x:v>The weekly horizon must contain exactly 13 columns.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="15" t="str">
+      <x:c r="A9" s="73" t="str">
         <x:v>Forecast starts Monday</x:v>
       </x:c>
-      <x:c r="B9" s="52" t="n">
+      <x:c r="B9" s="75" t="n">
         <x:f>WEEKDAY('Assumptions'!$B$8,2)</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C9" s="52" t="n">
+      <x:c r="C9" s="75" t="n">
         <x:f>1</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D9" s="52" t="n">
+      <x:c r="D9" s="75" t="n">
         <x:f>B9-C9</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E9" s="52" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F9" s="15" t="str">
+      <x:c r="E9" s="75" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F9" s="73" t="str">
         <x:f>IF(ABS(D9)&lt;=E9,"PASS","FAIL")</x:f>
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="G9" s="15" t="str">
+      <x:c r="G9" s="73" t="str">
         <x:v>Assumptions!B8</x:v>
       </x:c>
-      <x:c r="H9" s="15" t="str">
+      <x:c r="H9" s="73" t="str">
         <x:v>Forecast start date must be a Monday.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="15" t="str">
+      <x:c r="A10" s="73" t="str">
         <x:v>Selected scenario recognised</x:v>
       </x:c>
-      <x:c r="B10" s="52" t="n">
+      <x:c r="B10" s="75" t="n">
         <x:f>COUNTIF('Assumptions'!$B$15:$B$17,'Assumptions'!$B$12)</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C10" s="52" t="n">
+      <x:c r="C10" s="75" t="n">
         <x:f>1</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D10" s="52" t="n">
+      <x:c r="D10" s="75" t="n">
         <x:f>B10-C10</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E10" s="52" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F10" s="15" t="str">
+      <x:c r="E10" s="75" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F10" s="73" t="str">
         <x:f>IF(ABS(D10)&lt;=E10,"PASS","FAIL")</x:f>
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="G10" s="15" t="str">
+      <x:c r="G10" s="73" t="str">
         <x:v>Assumptions!B12</x:v>
       </x:c>
-      <x:c r="H10" s="15" t="str">
+      <x:c r="H10" s="73" t="str">
         <x:v>Select Base, Upside or Downside.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="15" t="str">
+      <x:c r="A11" s="73" t="str">
         <x:v>Week 1 opening cash ties</x:v>
       </x:c>
-      <x:c r="B11" s="53" t="n">
+      <x:c r="B11" s="76" t="n">
         <x:f>'13-Week Forecast'!$B$46</x:f>
         <x:v>400000</x:v>
       </x:c>
-      <x:c r="C11" s="53" t="n">
+      <x:c r="C11" s="76" t="n">
         <x:f>'Assumptions'!$B$10</x:f>
         <x:v>400000</x:v>
       </x:c>
-      <x:c r="D11" s="52" t="n">
+      <x:c r="D11" s="75" t="n">
         <x:f>B11-C11</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E11" s="52" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F11" s="15" t="str">
+      <x:c r="E11" s="75" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F11" s="73" t="str">
         <x:f>IF(ABS(D11)&lt;=E11,"PASS","FAIL")</x:f>
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="G11" s="15" t="str">
+      <x:c r="G11" s="73" t="str">
         <x:v>13-Week Forecast!B46</x:v>
       </x:c>
-      <x:c r="H11" s="15" t="str">
+      <x:c r="H11" s="73" t="str">
         <x:v>Week 1 opening cash must link to the control panel.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="15" t="str">
+      <x:c r="A12" s="73" t="str">
         <x:v>Weekly cash roll-forward equations</x:v>
       </x:c>
-      <x:c r="B12" s="52" t="n">
+      <x:c r="B12" s="75" t="n">
         <x:f>MAX(ABS('13-Week Forecast'!$B$48-'13-Week Forecast'!$B$46-'13-Week Forecast'!$B$47),ABS('13-Week Forecast'!$C$48-'13-Week Forecast'!$C$46-'13-Week Forecast'!$C$47),ABS('13-Week Forecast'!$D$48-'13-Week Forecast'!$D$46-'13-Week Forecast'!$D$47),ABS('13-Week Forecast'!$E$48-'13-Week Forecast'!$E$46-'13-Week Forecast'!$E$47),ABS('13-Week Forecast'!$F$48-'13-Week Forecast'!$F$46-'13-Week Forecast'!$F$47),ABS('13-Week Forecast'!$G$48-'13-Week Forecast'!$G$46-'13-Week Forecast'!$G$47),ABS('13-Week Forecast'!$H$48-'13-Week Forecast'!$H$46-'13-Week Forecast'!$H$47),ABS('13-Week Forecast'!$I$48-'13-Week Forecast'!$I$46-'13-Week Forecast'!$I$47),ABS('13-Week Forecast'!$J$48-'13-Week Forecast'!$J$46-'13-Week Forecast'!$J$47),ABS('13-Week Forecast'!$K$48-'13-Week Forecast'!$K$46-'13-Week Forecast'!$K$47),ABS('13-Week Forecast'!$L$48-'13-Week Forecast'!$L$46-'13-Week Forecast'!$L$47),ABS('13-Week Forecast'!$M$48-'13-Week Forecast'!$M$46-'13-Week Forecast'!$M$47),ABS('13-Week Forecast'!$N$48-'13-Week Forecast'!$N$46-'13-Week Forecast'!$N$47),ABS('13-Week Forecast'!$C$46-'13-Week Forecast'!$B$48),ABS('13-Week Forecast'!$D$46-'13-Week Forecast'!$C$48),ABS('13-Week Forecast'!$E$46-'13-Week Forecast'!$D$48),ABS('13-Week Forecast'!$F$46-'13-Week Forecast'!$E$48),ABS('13-Week Forecast'!$G$46-'13-Week Forecast'!$F$48),ABS('13-Week Forecast'!$H$46-'13-Week Forecast'!$G$48),ABS('13-Week Forecast'!$I$46-'13-Week Forecast'!$H$48),ABS('13-Week Forecast'!$J$46-'13-Week Forecast'!$I$48),ABS('13-Week Forecast'!$K$46-'13-Week Forecast'!$J$48),ABS('13-Week Forecast'!$L$46-'13-Week Forecast'!$K$48),ABS('13-Week Forecast'!$M$46-'13-Week Forecast'!$L$48),ABS('13-Week Forecast'!$N$46-'13-Week Forecast'!$M$48))</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C12" s="52" t="n">
+      <x:c r="C12" s="75" t="n">
         <x:f>0</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D12" s="52" t="n">
+      <x:c r="D12" s="75" t="n">
         <x:f>B12-C12</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E12" s="52" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F12" s="15" t="str">
+      <x:c r="E12" s="75" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F12" s="73" t="str">
         <x:f>IF(ABS(D12)&lt;=E12,"PASS","FAIL")</x:f>
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="G12" s="15" t="str">
+      <x:c r="G12" s="73" t="str">
         <x:v>13-Week Forecast!B46:N48</x:v>
       </x:c>
-      <x:c r="H12" s="15" t="str">
+      <x:c r="H12" s="73" t="str">
         <x:v>Each close must equal opening plus net movement; each opening after Week 1 must equal the prior close.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="15" t="str">
+      <x:c r="A13" s="73" t="str">
         <x:v>Cash receipt totals reconcile</x:v>
       </x:c>
-      <x:c r="B13" s="52" t="n">
+      <x:c r="B13" s="75" t="n">
         <x:f>MAX(ABS('13-Week Forecast'!$B$19-SUM('13-Week Forecast'!$B$10:$B$18)),ABS('13-Week Forecast'!$C$19-SUM('13-Week Forecast'!$C$10:$C$18)),ABS('13-Week Forecast'!$D$19-SUM('13-Week Forecast'!$D$10:$D$18)),ABS('13-Week Forecast'!$E$19-SUM('13-Week Forecast'!$E$10:$E$18)),ABS('13-Week Forecast'!$F$19-SUM('13-Week Forecast'!$F$10:$F$18)),ABS('13-Week Forecast'!$G$19-SUM('13-Week Forecast'!$G$10:$G$18)),ABS('13-Week Forecast'!$H$19-SUM('13-Week Forecast'!$H$10:$H$18)),ABS('13-Week Forecast'!$I$19-SUM('13-Week Forecast'!$I$10:$I$18)),ABS('13-Week Forecast'!$J$19-SUM('13-Week Forecast'!$J$10:$J$18)),ABS('13-Week Forecast'!$K$19-SUM('13-Week Forecast'!$K$10:$K$18)),ABS('13-Week Forecast'!$L$19-SUM('13-Week Forecast'!$L$10:$L$18)),ABS('13-Week Forecast'!$M$19-SUM('13-Week Forecast'!$M$10:$M$18)),ABS('13-Week Forecast'!$N$19-SUM('13-Week Forecast'!$N$10:$N$18)))</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C13" s="52" t="n">
+      <x:c r="C13" s="75" t="n">
         <x:f>0</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D13" s="52" t="n">
+      <x:c r="D13" s="75" t="n">
         <x:f>B13-C13</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E13" s="52" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F13" s="15" t="str">
+      <x:c r="E13" s="75" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F13" s="73" t="str">
         <x:f>IF(ABS(D13)&lt;=E13,"PASS","FAIL")</x:f>
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="G13" s="15" t="str">
+      <x:c r="G13" s="73" t="str">
         <x:v>13-Week Forecast!B19:N19</x:v>
       </x:c>
-      <x:c r="H13" s="15" t="str">
+      <x:c r="H13" s="73" t="str">
         <x:v>Maximum weekly difference; includes the selected-scenario receipt adjustment.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="15" t="str">
+      <x:c r="A14" s="73" t="str">
         <x:v>Cash payment totals reconcile</x:v>
       </x:c>
-      <x:c r="B14" s="52" t="n">
+      <x:c r="B14" s="75" t="n">
         <x:f>MAX(ABS('13-Week Forecast'!$B$43-SUM('13-Week Forecast'!$B$22:$B$42)),ABS('13-Week Forecast'!$C$43-SUM('13-Week Forecast'!$C$22:$C$42)),ABS('13-Week Forecast'!$D$43-SUM('13-Week Forecast'!$D$22:$D$42)),ABS('13-Week Forecast'!$E$43-SUM('13-Week Forecast'!$E$22:$E$42)),ABS('13-Week Forecast'!$F$43-SUM('13-Week Forecast'!$F$22:$F$42)),ABS('13-Week Forecast'!$G$43-SUM('13-Week Forecast'!$G$22:$G$42)),ABS('13-Week Forecast'!$H$43-SUM('13-Week Forecast'!$H$22:$H$42)),ABS('13-Week Forecast'!$I$43-SUM('13-Week Forecast'!$I$22:$I$42)),ABS('13-Week Forecast'!$J$43-SUM('13-Week Forecast'!$J$22:$J$42)),ABS('13-Week Forecast'!$K$43-SUM('13-Week Forecast'!$K$22:$K$42)),ABS('13-Week Forecast'!$L$43-SUM('13-Week Forecast'!$L$22:$L$42)),ABS('13-Week Forecast'!$M$43-SUM('13-Week Forecast'!$M$22:$M$42)),ABS('13-Week Forecast'!$N$43-SUM('13-Week Forecast'!$N$22:$N$42)))</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C14" s="52" t="n">
+      <x:c r="C14" s="75" t="n">
         <x:f>0</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D14" s="52" t="n">
+      <x:c r="D14" s="75" t="n">
         <x:f>B14-C14</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E14" s="52" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F14" s="15" t="str">
+      <x:c r="E14" s="75" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F14" s="73" t="str">
         <x:f>IF(ABS(D14)&lt;=E14,"PASS","FAIL")</x:f>
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="G14" s="15" t="str">
+      <x:c r="G14" s="73" t="str">
         <x:v>13-Week Forecast!B43:N43</x:v>
       </x:c>
-      <x:c r="H14" s="15" t="str">
+      <x:c r="H14" s="73" t="str">
         <x:v>Maximum weekly difference; includes the selected-scenario payment adjustment.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="15" t="str">
+      <x:c r="A15" s="73" t="str">
         <x:v>Week 13 closing cash equation</x:v>
       </x:c>
-      <x:c r="B15" s="53" t="n">
+      <x:c r="B15" s="76" t="n">
         <x:f>'13-Week Forecast'!$N$48</x:f>
         <x:v>31000</x:v>
       </x:c>
-      <x:c r="C15" s="53" t="n">
+      <x:c r="C15" s="76" t="n">
         <x:f>'Assumptions'!$B$10+SUM('13-Week Forecast'!$B$47:$N$47)</x:f>
         <x:v>31000</x:v>
       </x:c>
-      <x:c r="D15" s="52" t="n">
+      <x:c r="D15" s="75" t="n">
         <x:f>B15-C15</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E15" s="52" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F15" s="15" t="str">
+      <x:c r="E15" s="75" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F15" s="73" t="str">
         <x:f>IF(ABS(D15)&lt;=E15,"PASS","FAIL")</x:f>
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="G15" s="15" t="str">
+      <x:c r="G15" s="73" t="str">
         <x:v>13-Week Forecast!N48</x:v>
       </x:c>
-      <x:c r="H15" s="15" t="str">
+      <x:c r="H15" s="73" t="str">
         <x:v>Week 13 close must equal opening cash plus cumulative net movement.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="15" t="str">
+      <x:c r="A16" s="73" t="str">
         <x:v>Formula-error count</x:v>
       </x:c>
-      <x:c r="B16" s="52" t="n">
+      <x:c r="B16" s="75" t="n">
         <x:f>SUMPRODUCT(--ISERROR('Assumptions'!$B$5:$E$19))+SUMPRODUCT(--ISERROR('13-Week Forecast'!$B$5:$O$51))+SUMPRODUCT(--ISERROR('Weekly Review'!$A$4:$N$18))+SUMPRODUCT(--ISERROR('Dashboard'!$A$6:$J$30))+SUMPRODUCT(--ISERROR('Dashboard'!$P$4:$S$49))</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C16" s="52" t="n">
+      <x:c r="C16" s="75" t="n">
         <x:f>0</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D16" s="52" t="n">
+      <x:c r="D16" s="75" t="n">
         <x:f>B16-C16</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E16" s="52" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F16" s="15" t="str">
+      <x:c r="E16" s="75" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F16" s="73" t="str">
         <x:f>IF(ABS(D16)&lt;=E16,"PASS","FAIL")</x:f>
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="G16" s="15" t="str">
+      <x:c r="G16" s="73" t="str">
         <x:v>Assumptions, Forecast, Weekly Review and Dashboard</x:v>
       </x:c>
-      <x:c r="H16" s="15" t="str">
+      <x:c r="H16" s="73" t="str">
         <x:v>Any formula error in the model ranges fails this check.</x:v>
       </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="71"/>
+      <x:c r="B17" s="71"/>
+      <x:c r="C17" s="71"/>
+      <x:c r="D17" s="71"/>
+      <x:c r="E17" s="71"/>
+      <x:c r="F17" s="71"/>
+      <x:c r="G17" s="71"/>
+      <x:c r="H17" s="71"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="71"/>
+      <x:c r="B18" s="71"/>
+      <x:c r="C18" s="71"/>
+      <x:c r="D18" s="71"/>
+      <x:c r="E18" s="71"/>
+      <x:c r="F18" s="71"/>
+      <x:c r="G18" s="71"/>
+      <x:c r="H18" s="71"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="71"/>
+      <x:c r="B19" s="71"/>
+      <x:c r="C19" s="71"/>
+      <x:c r="D19" s="71"/>
+      <x:c r="E19" s="71"/>
+      <x:c r="F19" s="71"/>
+      <x:c r="G19" s="71"/>
+      <x:c r="H19" s="71"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="71"/>
+      <x:c r="B20" s="71"/>
+      <x:c r="C20" s="71"/>
+      <x:c r="D20" s="71"/>
+      <x:c r="E20" s="71"/>
+      <x:c r="F20" s="71"/>
+      <x:c r="G20" s="71"/>
+      <x:c r="H20" s="71"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="14" t="str">
@@ -6278,6 +7269,8 @@
       <x:c r="F21" s="14" t="str">
         <x:v>Planning treatment</x:v>
       </x:c>
+      <x:c r="G21" s="71"/>
+      <x:c r="H21" s="71"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="55" t="str">
@@ -6298,6 +7291,8 @@
       <x:c r="F22" s="55" t="str">
         <x:v>Keep tax classifications user-confirmed.</x:v>
       </x:c>
+      <x:c r="G22" s="71"/>
+      <x:c r="H22" s="71"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="55" t="str">
@@ -6318,6 +7313,8 @@
       <x:c r="F23" s="55" t="str">
         <x:v>Use issued BAS and user-entered dates.</x:v>
       </x:c>
+      <x:c r="G23" s="71"/>
+      <x:c r="H23" s="71"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="55" t="str">
@@ -6338,6 +7335,8 @@
       <x:c r="F24" s="55" t="str">
         <x:v>Keep payment dates user-entered and confirmed.</x:v>
       </x:c>
+      <x:c r="G24" s="71"/>
+      <x:c r="H24" s="71"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="55" t="str">
@@ -6358,6 +7357,8 @@
       <x:c r="F25" s="55" t="str">
         <x:v>Weekly super is illustrative FP&amp;A input.</x:v>
       </x:c>
+      <x:c r="G25" s="71"/>
+      <x:c r="H25" s="71"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="55" t="str">
@@ -6378,6 +7379,18 @@
       <x:c r="F26" s="55" t="str">
         <x:v>Illustrative forecast starts after the July 2026 transition.</x:v>
       </x:c>
+      <x:c r="G26" s="71"/>
+      <x:c r="H26" s="71"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="71"/>
+      <x:c r="B27" s="71"/>
+      <x:c r="C27" s="71"/>
+      <x:c r="D27" s="71"/>
+      <x:c r="E27" s="71"/>
+      <x:c r="F27" s="71"/>
+      <x:c r="G27" s="71"/>
+      <x:c r="H27" s="71"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="58" t="str">

</xml_diff>